<commit_message>
Add comprehensive form validation to Internal Audit module
- Add Risk ID auto-generation with new API endpoint /api/internal-audit/risks/next-id
- Add validation with toast messages and required field asterisks to all settings forms
  (categories, audit types, departments, escalation, nature of controls, periodicity, risk assessment, user management, process)
- Process settings: validate Process Name and Process Owner (matching reference website)
- Add validation to Risk Register forms (inherent and residual risk fields)
- Add validation to fieldwork evidence requests and findings
- Add validation to risk identification page
- Keep buttons active and show toast error messages on validation failure
- Update translations for new validation messages

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C775"/>
+  <dimension ref="A1:C797"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -7039,1899 +7039,2141 @@
     </row>
     <row r="604">
       <c r="A604" t="str">
-        <v>Select type</v>
+        <v>Select Sub Category first</v>
       </c>
       <c r="B604" t="str">
-        <v>اختر النوع</v>
+        <v>اختر الفئة الفرعية أولاً</v>
       </c>
       <c r="C604" t="str">
-        <v>Izvēlieties tipu</v>
+        <v>Vispirms izvēlieties apakškategoriju</v>
       </c>
     </row>
     <row r="605">
       <c r="A605" t="str">
-        <v>Enter issue description</v>
+        <v>Select type</v>
       </c>
       <c r="B605" t="str">
-        <v>أدخل وصف القضية</v>
+        <v>اختر النوع</v>
       </c>
       <c r="C605" t="str">
-        <v>Ievadiet problēmas aprakstu</v>
+        <v>Izvēlieties tipu</v>
       </c>
     </row>
     <row r="606">
       <c r="A606" t="str">
-        <v>New Stakeholder</v>
+        <v>Enter issue description</v>
       </c>
       <c r="B606" t="str">
-        <v>صاحب مصلحة جديد</v>
+        <v>أدخل وصف القضية</v>
       </c>
       <c r="C606" t="str">
-        <v>Jauna ieinteresētā puse</v>
+        <v>Ievadiet problēmas aprakstu</v>
       </c>
     </row>
     <row r="607">
       <c r="A607" t="str">
-        <v>Edit Stakeholder</v>
+        <v>New Stakeholder</v>
       </c>
       <c r="B607" t="str">
-        <v>تعديل صاحب المصلحة</v>
+        <v>صاحب مصلحة جديد</v>
       </c>
       <c r="C607" t="str">
-        <v>Rediģēt ieinteresēto pusi</v>
+        <v>Jauna ieinteresētā puse</v>
       </c>
     </row>
     <row r="608">
       <c r="A608" t="str">
-        <v>Search stakeholders...</v>
+        <v>Edit Stakeholder</v>
       </c>
       <c r="B608" t="str">
-        <v>البحث في أصحاب المصلحة...</v>
+        <v>تعديل صاحب المصلحة</v>
       </c>
       <c r="C608" t="str">
-        <v>Meklēt ieinteresētās puses...</v>
+        <v>Rediģēt ieinteresēto pusi</v>
       </c>
     </row>
     <row r="609">
       <c r="A609" t="str">
-        <v>Search issues...</v>
+        <v>Search stakeholders...</v>
       </c>
       <c r="B609" t="str">
-        <v>البحث في القضايا...</v>
+        <v>البحث في أصحاب المصلحة...</v>
       </c>
       <c r="C609" t="str">
-        <v>Meklēt problēmas...</v>
+        <v>Meklēt ieinteresētās puses...</v>
       </c>
     </row>
     <row r="610">
       <c r="A610" t="str">
-        <v>All Types</v>
+        <v>Search issues...</v>
       </c>
       <c r="B610" t="str">
-        <v>جميع الأنواع</v>
+        <v>البحث في القضايا...</v>
       </c>
       <c r="C610" t="str">
-        <v>Visi tipi</v>
+        <v>Meklēt problēmas...</v>
       </c>
     </row>
     <row r="611">
       <c r="A611" t="str">
-        <v>All Status</v>
+        <v>All Types</v>
       </c>
       <c r="B611" t="str">
-        <v>جميع الحالات</v>
+        <v>جميع الأنواع</v>
       </c>
       <c r="C611" t="str">
-        <v>Visi statusi</v>
+        <v>Visi tipi</v>
       </c>
     </row>
     <row r="612">
       <c r="A612" t="str">
-        <v>All Categories</v>
+        <v>All Status</v>
       </c>
       <c r="B612" t="str">
-        <v>جميع الفئات</v>
+        <v>جميع الحالات</v>
       </c>
       <c r="C612" t="str">
-        <v>Visas kategorijas</v>
+        <v>Visi statusi</v>
       </c>
     </row>
     <row r="613">
       <c r="A613" t="str">
-        <v>All Domains</v>
+        <v>All Categories</v>
       </c>
       <c r="B613" t="str">
-        <v>جميع المجالات</v>
+        <v>جميع الفئات</v>
       </c>
       <c r="C613" t="str">
-        <v>Visi domēni</v>
+        <v>Visas kategorijas</v>
       </c>
     </row>
     <row r="614">
       <c r="A614" t="str">
-        <v>No Issues Found</v>
+        <v>All Domains</v>
       </c>
       <c r="B614" t="str">
-        <v>لم يتم العثور على قضايا</v>
+        <v>جميع المجالات</v>
       </c>
       <c r="C614" t="str">
-        <v>Problēmas nav atrastas</v>
+        <v>Visi domēni</v>
       </c>
     </row>
     <row r="615">
       <c r="A615" t="str">
-        <v>Try adjusting your filters to find issues.</v>
+        <v>No Issues Found</v>
       </c>
       <c r="B615" t="str">
-        <v>حاول تعديل الفلاتر للعثور على القضايا.</v>
+        <v>لم يتم العثور على قضايا</v>
       </c>
       <c r="C615" t="str">
-        <v>Mēģiniet pielāgot filtrus, lai atrastu problēmas.</v>
+        <v>Problēmas nav atrastas</v>
       </c>
     </row>
     <row r="616">
       <c r="A616" t="str">
-        <v>Create your first issue to get started.</v>
+        <v>Try adjusting your filters to find issues.</v>
       </c>
       <c r="B616" t="str">
-        <v>أنشئ أول قضية للبدء.</v>
+        <v>حاول تعديل الفلاتر للعثور على القضايا.</v>
       </c>
       <c r="C616" t="str">
-        <v>Izveidojiet savu pirmo problēmu, lai sāktu.</v>
+        <v>Mēģiniet pielāgot filtrus, lai atrastu problēmas.</v>
       </c>
     </row>
     <row r="617">
       <c r="A617" t="str">
-        <v>Create Action</v>
+        <v>Create your first issue to get started.</v>
       </c>
       <c r="B617" t="str">
-        <v>إنشاء إجراء</v>
+        <v>أنشئ أول قضية للبدء.</v>
       </c>
       <c r="C617" t="str">
-        <v>Izveidot darbību</v>
+        <v>Izveidojiet savu pirmo problēmu, lai sāktu.</v>
       </c>
     </row>
     <row r="618">
       <c r="A618" t="str">
-        <v>View Actions</v>
+        <v>Create Action</v>
       </c>
       <c r="B618" t="str">
-        <v>عرض الإجراءات</v>
+        <v>إنشاء إجراء</v>
       </c>
       <c r="C618" t="str">
-        <v>Skatīt darbības</v>
+        <v>Izveidot darbību</v>
       </c>
     </row>
     <row r="619">
       <c r="A619" t="str">
-        <v>Review Actions</v>
+        <v>View Actions</v>
       </c>
       <c r="B619" t="str">
-        <v>مراجعة الإجراءات</v>
+        <v>عرض الإجراءات</v>
       </c>
       <c r="C619" t="str">
-        <v>Pārskatīt darbības</v>
+        <v>Skatīt darbības</v>
       </c>
     </row>
     <row r="620">
       <c r="A620" t="str">
-        <v>Select stakeholder</v>
+        <v>Review Actions</v>
       </c>
       <c r="B620" t="str">
-        <v>اختر صاحب المصلحة</v>
+        <v>مراجعة الإجراءات</v>
       </c>
       <c r="C620" t="str">
-        <v>Izvēlieties ieinteresēto pusi</v>
+        <v>Pārskatīt darbības</v>
       </c>
     </row>
     <row r="621">
       <c r="A621" t="str">
-        <v>Need and Expectation</v>
+        <v>Select stakeholder</v>
       </c>
       <c r="B621" t="str">
-        <v>الاحتياجات والتوقعات</v>
+        <v>اختر صاحب المصلحة</v>
       </c>
       <c r="C621" t="str">
-        <v>Vajadzība un gaidījums</v>
+        <v>Izvēlieties ieinteresēto pusi</v>
       </c>
     </row>
     <row r="622">
       <c r="A622" t="str">
-        <v>Select need/expectation</v>
+        <v>Need and Expectation</v>
       </c>
       <c r="B622" t="str">
-        <v>اختر الاحتياج/التوقع</v>
+        <v>الاحتياجات والتوقعات</v>
       </c>
       <c r="C622" t="str">
-        <v>Izvēlieties vajadzību/gaidījumu</v>
+        <v>Vajadzība un gaidījums</v>
       </c>
     </row>
     <row r="623">
       <c r="A623" t="str">
-        <v>Stakeholder Needs and Expectations</v>
+        <v>Select need/expectation</v>
       </c>
       <c r="B623" t="str">
-        <v>احتياجات وتوقعات أصحاب المصلحة</v>
+        <v>اختر الاحتياج/التوقع</v>
       </c>
       <c r="C623" t="str">
-        <v>Ieinteresēto pušu vajadzības un gaidījumi</v>
+        <v>Izvēlieties vajadzību/gaidījumu</v>
       </c>
     </row>
     <row r="624">
       <c r="A624" t="str">
-        <v>Add New Domain</v>
+        <v>Stakeholder Needs and Expectations</v>
       </c>
       <c r="B624" t="str">
-        <v>إضافة مجال جديد</v>
+        <v>احتياجات وتوقعات أصحاب المصلحة</v>
       </c>
       <c r="C624" t="str">
-        <v>Pievienot jaunu domēnu</v>
+        <v>Ieinteresēto pušu vajadzības un gaidījumi</v>
       </c>
     </row>
     <row r="625">
       <c r="A625" t="str">
-        <v>Enter domain name</v>
+        <v>Add New Domain</v>
       </c>
       <c r="B625" t="str">
-        <v>أدخل اسم المجال</v>
+        <v>إضافة مجال جديد</v>
       </c>
       <c r="C625" t="str">
-        <v>Ievadiet domēna nosaukumu</v>
+        <v>Pievienot jaunu domēnu</v>
       </c>
     </row>
     <row r="626">
       <c r="A626" t="str">
-        <v>Add New Category</v>
+        <v>Enter domain name</v>
       </c>
       <c r="B626" t="str">
-        <v>إضافة فئة جديدة</v>
+        <v>أدخل اسم المجال</v>
       </c>
       <c r="C626" t="str">
-        <v>Pievienot jaunu kategoriju</v>
+        <v>Ievadiet domēna nosaukumu</v>
       </c>
     </row>
     <row r="627">
       <c r="A627" t="str">
-        <v>Add New Issue Type</v>
+        <v>Add New Category</v>
       </c>
       <c r="B627" t="str">
-        <v>إضافة نوع قضية جديد</v>
+        <v>إضافة فئة جديدة</v>
       </c>
       <c r="C627" t="str">
-        <v>Pievienot jaunu problēmas tipu</v>
+        <v>Pievienot jaunu kategoriju</v>
       </c>
     </row>
     <row r="628">
       <c r="A628" t="str">
-        <v>Issue Type Name</v>
+        <v>Add New Issue Type</v>
       </c>
       <c r="B628" t="str">
-        <v>اسم نوع القضية</v>
+        <v>إضافة نوع قضية جديد</v>
       </c>
       <c r="C628" t="str">
-        <v>Problēmas tipa nosaukums</v>
+        <v>Pievienot jaunu problēmas tipu</v>
       </c>
     </row>
     <row r="629">
       <c r="A629" t="str">
-        <v>Enter issue type name</v>
+        <v>Issue Type Name</v>
       </c>
       <c r="B629" t="str">
-        <v>أدخل اسم نوع القضية</v>
+        <v>اسم نوع القضية</v>
       </c>
       <c r="C629" t="str">
-        <v>Ievadiet problēmas tipa nosaukumu</v>
+        <v>Problēmas tipa nosaukums</v>
       </c>
     </row>
     <row r="630">
       <c r="A630" t="str">
-        <v>Link Process</v>
+        <v>Enter issue type name</v>
       </c>
       <c r="B630" t="str">
-        <v>ربط العملية</v>
+        <v>أدخل اسم نوع القضية</v>
       </c>
       <c r="C630" t="str">
-        <v>Saistīt procesu</v>
+        <v>Ievadiet problēmas tipa nosaukumu</v>
       </c>
     </row>
     <row r="631">
       <c r="A631" t="str">
-        <v>No processes found</v>
+        <v>Link Process</v>
       </c>
       <c r="B631" t="str">
-        <v>لم يتم العثور على عمليات</v>
+        <v>ربط العملية</v>
       </c>
       <c r="C631" t="str">
-        <v>Procesi nav atrasti</v>
+        <v>Saistīt procesu</v>
       </c>
     </row>
     <row r="632">
       <c r="A632" t="str">
-        <v>Add New Need/Expectation</v>
+        <v>No processes found</v>
       </c>
       <c r="B632" t="str">
-        <v>إضافة احتياج/توقع جديد</v>
+        <v>لم يتم العثور على عمليات</v>
       </c>
       <c r="C632" t="str">
-        <v>Pievienot jaunu vajadzību/gaidījumu</v>
+        <v>Procesi nav atrasti</v>
       </c>
     </row>
     <row r="633">
       <c r="A633" t="str">
-        <v>Need/Expectation</v>
+        <v>Add New Need/Expectation</v>
       </c>
       <c r="B633" t="str">
-        <v>الاحتياج/التوقع</v>
+        <v>إضافة احتياج/توقع جديد</v>
       </c>
       <c r="C633" t="str">
-        <v>Vajadzība/Gaidījums</v>
+        <v>Pievienot jaunu vajadzību/gaidījumu</v>
       </c>
     </row>
     <row r="634">
       <c r="A634" t="str">
-        <v>Enter need/expectation</v>
+        <v>Need/Expectation</v>
       </c>
       <c r="B634" t="str">
-        <v>أدخل الاحتياج/التوقع</v>
+        <v>الاحتياج/التوقع</v>
       </c>
       <c r="C634" t="str">
-        <v>Ievadiet vajadzību/gaidījumu</v>
+        <v>Vajadzība/Gaidījums</v>
       </c>
     </row>
     <row r="635">
       <c r="A635" t="str">
-        <v>Enter a new need or expectation type.</v>
+        <v>Enter need/expectation</v>
       </c>
       <c r="B635" t="str">
-        <v>أدخل نوع احتياج أو توقع جديد.</v>
+        <v>أدخل الاحتياج/التوقع</v>
       </c>
       <c r="C635" t="str">
-        <v>Ievadiet jaunu vajadzības vai gaidījumu tipu.</v>
+        <v>Ievadiet vajadzību/gaidījumu</v>
       </c>
     </row>
     <row r="636">
       <c r="A636" t="str">
-        <v>Title is required</v>
+        <v>Enter a new need or expectation type.</v>
       </c>
       <c r="B636" t="str">
-        <v>العنوان مطلوب</v>
+        <v>أدخل نوع احتياج أو توقع جديد.</v>
       </c>
       <c r="C636" t="str">
-        <v>Nosaukums ir obligāts</v>
+        <v>Ievadiet jaunu vajadzības vai gaidījumu tipu.</v>
       </c>
     </row>
     <row r="637">
       <c r="A637" t="str">
-        <v>Issue created successfully</v>
+        <v>Title is required</v>
       </c>
       <c r="B637" t="str">
-        <v>تم إنشاء القضية بنجاح</v>
+        <v>العنوان مطلوب</v>
       </c>
       <c r="C637" t="str">
-        <v>Problēma veiksmīgi izveidota</v>
+        <v>Nosaukums ir obligāts</v>
       </c>
     </row>
     <row r="638">
       <c r="A638" t="str">
-        <v>Failed to create issue</v>
+        <v>Issue created successfully</v>
       </c>
       <c r="B638" t="str">
-        <v>فشل في إنشاء القضية</v>
+        <v>تم إنشاء القضية بنجاح</v>
       </c>
       <c r="C638" t="str">
-        <v>Neizdevās izveidot problēmu</v>
+        <v>Problēma veiksmīgi izveidota</v>
       </c>
     </row>
     <row r="639">
       <c r="A639" t="str">
-        <v>Issue updated successfully</v>
+        <v>Failed to create issue</v>
       </c>
       <c r="B639" t="str">
-        <v>تم تحديث القضية بنجاح</v>
+        <v>فشل في إنشاء القضية</v>
       </c>
       <c r="C639" t="str">
-        <v>Problēma veiksmīgi atjaunināta</v>
+        <v>Neizdevās izveidot problēmu</v>
       </c>
     </row>
     <row r="640">
       <c r="A640" t="str">
-        <v>Failed to update issue</v>
+        <v>Issue updated successfully</v>
       </c>
       <c r="B640" t="str">
-        <v>فشل في تحديث القضية</v>
+        <v>تم تحديث القضية بنجاح</v>
       </c>
       <c r="C640" t="str">
-        <v>Neizdevās atjaunināt problēmu</v>
+        <v>Problēma veiksmīgi atjaunināta</v>
       </c>
     </row>
     <row r="641">
       <c r="A641" t="str">
-        <v>Stakeholder updated successfully</v>
+        <v>Failed to update issue</v>
       </c>
       <c r="B641" t="str">
-        <v>تم تحديث صاحب المصلحة بنجاح</v>
+        <v>فشل في تحديث القضية</v>
       </c>
       <c r="C641" t="str">
-        <v>Ieinteresētā puse veiksmīgi atjaunināta</v>
+        <v>Neizdevās atjaunināt problēmu</v>
       </c>
     </row>
     <row r="642">
       <c r="A642" t="str">
-        <v>Failed to update stakeholder</v>
+        <v>Stakeholder updated successfully</v>
       </c>
       <c r="B642" t="str">
-        <v>فشل في تحديث صاحب المصلحة</v>
+        <v>تم تحديث صاحب المصلحة بنجاح</v>
       </c>
       <c r="C642" t="str">
-        <v>Neizdevās atjaunināt ieinteresēto pusi</v>
+        <v>Ieinteresētā puse veiksmīgi atjaunināta</v>
       </c>
     </row>
     <row r="643">
       <c r="A643" t="str">
-        <v>Open</v>
+        <v>Failed to update stakeholder</v>
       </c>
       <c r="B643" t="str">
-        <v>مفتوح</v>
+        <v>فشل في تحديث صاحب المصلحة</v>
       </c>
       <c r="C643" t="str">
-        <v>Atvērts</v>
+        <v>Neizdevās atjaunināt ieinteresēto pusi</v>
       </c>
     </row>
     <row r="644">
       <c r="A644" t="str">
-        <v>In Progress</v>
+        <v>Open</v>
       </c>
       <c r="B644" t="str">
-        <v>قيد التنفيذ</v>
+        <v>مفتوح</v>
       </c>
       <c r="C644" t="str">
-        <v>Procesā</v>
+        <v>Atvērts</v>
       </c>
     </row>
     <row r="645">
       <c r="A645" t="str">
-        <v>Action type and description are required</v>
+        <v>In Progress</v>
       </c>
       <c r="B645" t="str">
-        <v>نوع الإجراء والوصف مطلوبان</v>
+        <v>قيد التنفيذ</v>
       </c>
       <c r="C645" t="str">
-        <v>Darbības tips un apraksts ir obligāti</v>
+        <v>Procesā</v>
       </c>
     </row>
     <row r="646">
       <c r="A646" t="str">
-        <v>Action created successfully</v>
+        <v>Action type and description are required</v>
       </c>
       <c r="B646" t="str">
-        <v>تم إنشاء الإجراء بنجاح</v>
+        <v>نوع الإجراء والوصف مطلوبان</v>
       </c>
       <c r="C646" t="str">
-        <v>Darbība veiksmīgi izveidota</v>
+        <v>Darbības tips un apraksts ir obligāti</v>
       </c>
     </row>
     <row r="647">
       <c r="A647" t="str">
-        <v>Failed to create action</v>
+        <v>Action created successfully</v>
       </c>
       <c r="B647" t="str">
-        <v>فشل في إنشاء الإجراء</v>
+        <v>تم إنشاء الإجراء بنجاح</v>
       </c>
       <c r="C647" t="str">
-        <v>Neizdevās izveidot darbību</v>
+        <v>Darbība veiksmīgi izveidota</v>
       </c>
     </row>
     <row r="648">
       <c r="A648" t="str">
-        <v>Action is resolved</v>
+        <v>Failed to create action</v>
       </c>
       <c r="B648" t="str">
-        <v>تم حل الإجراء</v>
+        <v>فشل في إنشاء الإجراء</v>
       </c>
       <c r="C648" t="str">
-        <v>Darbība ir atrisināta</v>
+        <v>Neizdevās izveidot darbību</v>
       </c>
     </row>
     <row r="649">
       <c r="A649" t="str">
-        <v>Failed to resolve action</v>
+        <v>Action is resolved</v>
       </c>
       <c r="B649" t="str">
-        <v>فشل في حل الإجراء</v>
+        <v>تم حل الإجراء</v>
       </c>
       <c r="C649" t="str">
-        <v>Neizdevās atrisināt darbību</v>
+        <v>Darbība ir atrisināta</v>
       </c>
     </row>
     <row r="650">
       <c r="A650" t="str">
-        <v>Comment is required</v>
+        <v>Failed to resolve action</v>
       </c>
       <c r="B650" t="str">
-        <v>التعليق مطلوب</v>
+        <v>فشل في حل الإجراء</v>
       </c>
       <c r="C650" t="str">
-        <v>Komentārs ir obligāts</v>
+        <v>Neizdevās atrisināt darbību</v>
       </c>
     </row>
     <row r="651">
       <c r="A651" t="str">
-        <v>Action is sent back</v>
+        <v>Comment is required</v>
       </c>
       <c r="B651" t="str">
-        <v>تم إرجاع الإجراء</v>
+        <v>التعليق مطلوب</v>
       </c>
       <c r="C651" t="str">
-        <v>Darbība ir nosūtīta atpakaļ</v>
+        <v>Komentārs ir obligāts</v>
       </c>
     </row>
     <row r="652">
       <c r="A652" t="str">
-        <v>Failed to send back action</v>
+        <v>Action is sent back</v>
       </c>
       <c r="B652" t="str">
-        <v>فشل في إرجاع الإجراء</v>
+        <v>تم إرجاع الإجراء</v>
       </c>
       <c r="C652" t="str">
-        <v>Neizdevās nosūtīt atpakaļ darbību</v>
+        <v>Darbība ir nosūtīta atpakaļ</v>
       </c>
     </row>
     <row r="653">
       <c r="A653" t="str">
-        <v>Action updated and resubmitted</v>
+        <v>Failed to send back action</v>
       </c>
       <c r="B653" t="str">
-        <v>تم تحديث الإجراء وإعادة إرساله</v>
+        <v>فشل في إرجاع الإجراء</v>
       </c>
       <c r="C653" t="str">
-        <v>Darbība atjaunināta un atkārtoti iesniegta</v>
+        <v>Neizdevās nosūtīt atpakaļ darbību</v>
       </c>
     </row>
     <row r="654">
       <c r="A654" t="str">
-        <v>Failed to update action</v>
+        <v>Action updated and resubmitted</v>
       </c>
       <c r="B654" t="str">
-        <v>فشل في تحديث الإجراء</v>
+        <v>تم تحديث الإجراء وإعادة إرساله</v>
       </c>
       <c r="C654" t="str">
-        <v>Neizdevās atjaunināt darbību</v>
+        <v>Darbība atjaunināta un atkārtoti iesniegta</v>
       </c>
     </row>
     <row r="655">
       <c r="A655" t="str">
-        <v>Saving...</v>
+        <v>Failed to update action</v>
       </c>
       <c r="B655" t="str">
-        <v>جاري الحفظ...</v>
+        <v>فشل في تحديث الإجراء</v>
       </c>
       <c r="C655" t="str">
-        <v>Saglabā...</v>
+        <v>Neizdevās atjaunināt darbību</v>
       </c>
     </row>
     <row r="656">
       <c r="A656" t="str">
-        <v>Save &amp; Resubmit</v>
+        <v>Saving...</v>
       </c>
       <c r="B656" t="str">
-        <v>حفظ وإعادة الإرسال</v>
+        <v>جاري الحفظ...</v>
       </c>
       <c r="C656" t="str">
-        <v>Saglabāt un iesniegt atkārtoti</v>
+        <v>Saglabā...</v>
       </c>
     </row>
     <row r="657">
       <c r="A657" t="str">
-        <v>Import Issues</v>
+        <v>Save &amp; Resubmit</v>
       </c>
       <c r="B657" t="str">
-        <v>استيراد القضايا</v>
+        <v>حفظ وإعادة الإرسال</v>
       </c>
       <c r="C657" t="str">
-        <v>Importēt problēmas</v>
+        <v>Saglabāt un iesniegt atkārtoti</v>
       </c>
     </row>
     <row r="658">
       <c r="A658" t="str">
-        <v>CSV file must have a header row and at least one data row</v>
+        <v>Import Issues</v>
       </c>
       <c r="B658" t="str">
-        <v>يجب أن يحتوي ملف CSV على صف رأس وصف بيانات واحد على الأقل</v>
+        <v>استيراد القضايا</v>
       </c>
       <c r="C658" t="str">
-        <v>CSV failam jābūt galvenes rindai un vismaz vienai datu rindai</v>
+        <v>Importēt problēmas</v>
       </c>
     </row>
     <row r="659">
       <c r="A659" t="str">
-        <v>CSV must have a "title" column</v>
+        <v>CSV file must have a header row and at least one data row</v>
       </c>
       <c r="B659" t="str">
-        <v>يجب أن يحتوي ملف CSV على عمود "title"</v>
+        <v>يجب أن يحتوي ملف CSV على صف رأس وصف بيانات واحد على الأقل</v>
       </c>
       <c r="C659" t="str">
-        <v>CSV ir jābūt kolonnai "title"</v>
+        <v>CSV failam jābūt galvenes rindai un vismaz vienai datu rindai</v>
       </c>
     </row>
     <row r="660">
       <c r="A660" t="str">
-        <v>Successfully imported</v>
+        <v>CSV must have a "title" column</v>
       </c>
       <c r="B660" t="str">
-        <v>تم الاستيراد بنجاح</v>
+        <v>يجب أن يحتوي ملف CSV على عمود "title"</v>
       </c>
       <c r="C660" t="str">
-        <v>Veiksmīgi importēts</v>
+        <v>CSV ir jābūt kolonnai "title"</v>
       </c>
     </row>
     <row r="661">
       <c r="A661" t="str">
-        <v>issues</v>
+        <v>Successfully imported</v>
       </c>
       <c r="B661" t="str">
-        <v>قضايا</v>
+        <v>تم الاستيراد بنجاح</v>
       </c>
       <c r="C661" t="str">
-        <v>problēmas</v>
+        <v>Veiksmīgi importēts</v>
       </c>
     </row>
     <row r="662">
       <c r="A662" t="str">
-        <v>Error importing issues. Please check the file format.</v>
+        <v>issues</v>
       </c>
       <c r="B662" t="str">
-        <v>خطأ في استيراد القضايا. يرجى التحقق من تنسيق الملف.</v>
+        <v>قضايا</v>
       </c>
       <c r="C662" t="str">
-        <v>Kļūda importējot problēmas. Lūdzu, pārbaudiet faila formātu.</v>
+        <v>problēmas</v>
       </c>
     </row>
     <row r="663">
       <c r="A663" t="str">
-        <v>File attached to action</v>
+        <v>Error importing issues. Please check the file format.</v>
       </c>
       <c r="B663" t="str">
-        <v>تم إرفاق الملف بالإجراء</v>
+        <v>خطأ في استيراد القضايا. يرجى التحقق من تنسيق الملف.</v>
       </c>
       <c r="C663" t="str">
-        <v>Fails pievienots darbībai</v>
+        <v>Kļūda importējot problēmas. Lūdzu, pārbaudiet faila formātu.</v>
       </c>
     </row>
     <row r="664">
       <c r="A664" t="str">
-        <v>Failed to attach file to action</v>
+        <v>File attached to action</v>
       </c>
       <c r="B664" t="str">
-        <v>فشل في إرفاق الملف بالإجراء</v>
+        <v>تم إرفاق الملف بالإجراء</v>
       </c>
       <c r="C664" t="str">
-        <v>Neizdevās pievienot failu darbībai</v>
+        <v>Fails pievienots darbībai</v>
       </c>
     </row>
     <row r="665">
       <c r="A665" t="str">
-        <v>File deleted successfully</v>
+        <v>Failed to attach file to action</v>
       </c>
       <c r="B665" t="str">
-        <v>تم حذف الملف بنجاح</v>
+        <v>فشل في إرفاق الملف بالإجراء</v>
       </c>
       <c r="C665" t="str">
-        <v>Fails veiksmīgi dzēsts</v>
+        <v>Neizdevās pievienot failu darbībai</v>
       </c>
     </row>
     <row r="666">
       <c r="A666" t="str">
-        <v>Failed to delete file</v>
+        <v>File deleted successfully</v>
       </c>
       <c r="B666" t="str">
-        <v>فشل في حذف الملف</v>
+        <v>تم حذف الملف بنجاح</v>
       </c>
       <c r="C666" t="str">
-        <v>Neizdevās dzēst failu</v>
+        <v>Fails veiksmīgi dzēsts</v>
       </c>
     </row>
     <row r="667">
       <c r="A667" t="str">
-        <v>Repository</v>
+        <v>Failed to delete file</v>
       </c>
       <c r="B667" t="str">
-        <v>المستودع</v>
+        <v>فشل في حذف الملف</v>
       </c>
       <c r="C667" t="str">
-        <v>Repozitorijs</v>
+        <v>Neizdevās dzēst failu</v>
       </c>
     </row>
     <row r="668">
       <c r="A668" t="str">
-        <v>Performance Dashboard</v>
+        <v>Repository</v>
       </c>
       <c r="B668" t="str">
-        <v>لوحة الأداء</v>
+        <v>المستودع</v>
       </c>
       <c r="C668" t="str">
-        <v>Veiktspējas panelis</v>
+        <v>Repozitorijs</v>
       </c>
     </row>
     <row r="669">
       <c r="A669" t="str">
-        <v>Search By Process ID, Name</v>
+        <v>Performance Dashboard</v>
       </c>
       <c r="B669" t="str">
-        <v>البحث بمعرف العملية أو الاسم</v>
+        <v>لوحة الأداء</v>
       </c>
       <c r="C669" t="str">
-        <v>Meklēt pēc procesa ID, nosaukuma</v>
+        <v>Veiktspējas panelis</v>
       </c>
     </row>
     <row r="670">
       <c r="A670" t="str">
-        <v>All Owners</v>
+        <v>Search By Process ID, Name</v>
       </c>
       <c r="B670" t="str">
-        <v>جميع المالكين</v>
+        <v>البحث بمعرف العملية أو الاسم</v>
       </c>
       <c r="C670" t="str">
-        <v>Visi īpašnieki</v>
+        <v>Meklēt pēc procesa ID, nosaukuma</v>
       </c>
     </row>
     <row r="671">
       <c r="A671" t="str">
-        <v>All Frequencies</v>
+        <v>All Owners</v>
       </c>
       <c r="B671" t="str">
-        <v>جميع الترددات</v>
+        <v>جميع المالكين</v>
       </c>
       <c r="C671" t="str">
-        <v>Visi biežumi</v>
+        <v>Visi īpašnieki</v>
       </c>
     </row>
     <row r="672">
       <c r="A672" t="str">
-        <v>Edit Process</v>
+        <v>All Frequencies</v>
       </c>
       <c r="B672" t="str">
-        <v>تعديل العملية</v>
+        <v>جميع الترددات</v>
       </c>
       <c r="C672" t="str">
-        <v>Rediģēt procesu</v>
+        <v>Visi biežumi</v>
       </c>
     </row>
     <row r="673">
       <c r="A673" t="str">
-        <v>Confirm Delete</v>
+        <v>Edit Process</v>
       </c>
       <c r="B673" t="str">
-        <v>تأكيد الحذف</v>
+        <v>تعديل العملية</v>
       </c>
       <c r="C673" t="str">
-        <v>Apstiprināt dzēšanu</v>
+        <v>Rediģēt procesu</v>
       </c>
     </row>
     <row r="674">
       <c r="A674" t="str">
-        <v>Are you sure you want to delete this process? This action cannot be undone.</v>
+        <v>Confirm Delete</v>
       </c>
       <c r="B674" t="str">
-        <v>هل أنت متأكد أنك تريد حذف هذه العملية؟ لا يمكن التراجع عن هذا الإجراء.</v>
+        <v>تأكيد الحذف</v>
       </c>
       <c r="C674" t="str">
-        <v>Vai tiešām vēlaties dzēst šo procesu? Šo darbību nevar atsaukt.</v>
+        <v>Apstiprināt dzēšanu</v>
       </c>
     </row>
     <row r="675">
       <c r="A675" t="str">
-        <v>Add New Process</v>
+        <v>Are you sure you want to delete this process? This action cannot be undone.</v>
       </c>
       <c r="B675" t="str">
-        <v>إضافة عملية جديدة</v>
+        <v>هل أنت متأكد أنك تريد حذف هذه العملية؟ لا يمكن التراجع عن هذا الإجراء.</v>
       </c>
       <c r="C675" t="str">
-        <v>Pievienot jaunu procesu</v>
+        <v>Vai tiešām vēlaties dzēst šo procesu? Šo darbību nevar atsaukt.</v>
       </c>
     </row>
     <row r="676">
       <c r="A676" t="str">
-        <v>Basic Information</v>
+        <v>Add New Process</v>
       </c>
       <c r="B676" t="str">
-        <v>المعلومات الأساسية</v>
+        <v>إضافة عملية جديدة</v>
       </c>
       <c r="C676" t="str">
-        <v>Pamatinformācija</v>
+        <v>Pievienot jaunu procesu</v>
       </c>
     </row>
     <row r="677">
       <c r="A677" t="str">
-        <v>Process Details</v>
+        <v>Basic Information</v>
       </c>
       <c r="B677" t="str">
-        <v>تفاصيل العملية</v>
+        <v>المعلومات الأساسية</v>
       </c>
       <c r="C677" t="str">
-        <v>Procesa detaļas</v>
+        <v>Pamatinformācija</v>
       </c>
     </row>
     <row r="678">
       <c r="A678" t="str">
-        <v>Dependencies &amp; Options</v>
+        <v>Process Details</v>
       </c>
       <c r="B678" t="str">
-        <v>التبعيات والخيارات</v>
+        <v>تفاصيل العملية</v>
       </c>
       <c r="C678" t="str">
-        <v>Atkarības un opcijas</v>
+        <v>Procesa detaļas</v>
       </c>
     </row>
     <row r="679">
       <c r="A679" t="str">
-        <v>RACI Matrix</v>
+        <v>Dependencies &amp; Options</v>
       </c>
       <c r="B679" t="str">
-        <v>مصفوفة RACI</v>
+        <v>التبعيات والخيارات</v>
       </c>
       <c r="C679" t="str">
-        <v>RACI matrica</v>
+        <v>Atkarības un opcijas</v>
       </c>
     </row>
     <row r="680">
       <c r="A680" t="str">
-        <v>Enter process name</v>
+        <v>RACI Matrix</v>
       </c>
       <c r="B680" t="str">
-        <v>أدخل اسم العملية</v>
+        <v>مصفوفة RACI</v>
       </c>
       <c r="C680" t="str">
-        <v>Ievadiet procesa nosaukumu</v>
+        <v>RACI matrica</v>
       </c>
     </row>
     <row r="681">
       <c r="A681" t="str">
-        <v>Enter process description</v>
+        <v>Enter process name</v>
       </c>
       <c r="B681" t="str">
-        <v>أدخل وصف العملية</v>
+        <v>أدخل اسم العملية</v>
       </c>
       <c r="C681" t="str">
-        <v>Ievadiet procesa aprakstu</v>
+        <v>Ievadiet procesa nosaukumu</v>
       </c>
     </row>
     <row r="682">
       <c r="A682" t="str">
-        <v>Nature of Implementation</v>
+        <v>Enter process description</v>
       </c>
       <c r="B682" t="str">
-        <v>طبيعة التنفيذ</v>
+        <v>أدخل وصف العملية</v>
       </c>
       <c r="C682" t="str">
-        <v>Ieviešanas veids</v>
+        <v>Ievadiet procesa aprakstu</v>
       </c>
     </row>
     <row r="683">
       <c r="A683" t="str">
-        <v>Select implementation type</v>
+        <v>Nature of Implementation</v>
       </c>
       <c r="B683" t="str">
-        <v>اختر نوع التنفيذ</v>
+        <v>طبيعة التنفيذ</v>
       </c>
       <c r="C683" t="str">
-        <v>Izvēlieties ieviešanas tipu</v>
+        <v>Ieviešanas veids</v>
       </c>
     </row>
     <row r="684">
       <c r="A684" t="str">
-        <v>Select location</v>
+        <v>Select implementation type</v>
       </c>
       <c r="B684" t="str">
-        <v>اختر الموقع</v>
+        <v>اختر نوع التنفيذ</v>
       </c>
       <c r="C684" t="str">
-        <v>Izvēlieties atrašanās vietu</v>
+        <v>Izvēlieties ieviešanas tipu</v>
       </c>
     </row>
     <row r="685">
       <c r="A685" t="str">
-        <v>Operational Complexity</v>
+        <v>Select location</v>
       </c>
       <c r="B685" t="str">
-        <v>التعقيد التشغيلي</v>
+        <v>اختر الموقع</v>
       </c>
       <c r="C685" t="str">
-        <v>Operacionālā sarežģītība</v>
+        <v>Izvēlieties atrašanās vietu</v>
       </c>
     </row>
     <row r="686">
       <c r="A686" t="str">
-        <v>Select complexity</v>
+        <v>Operational Complexity</v>
       </c>
       <c r="B686" t="str">
-        <v>اختر التعقيد</v>
+        <v>التعقيد التشغيلي</v>
       </c>
       <c r="C686" t="str">
-        <v>Izvēlieties sarežģītību</v>
+        <v>Operacionālā sarežģītība</v>
       </c>
     </row>
     <row r="687">
       <c r="A687" t="str">
-        <v>Asset Dependency</v>
+        <v>Select complexity</v>
       </c>
       <c r="B687" t="str">
-        <v>تبعية الأصول</v>
+        <v>اختر التعقيد</v>
       </c>
       <c r="C687" t="str">
-        <v>Aktīvu atkarība</v>
+        <v>Izvēlieties sarežģītību</v>
       </c>
     </row>
     <row r="688">
       <c r="A688" t="str">
-        <v>External Dependency</v>
+        <v>Asset Dependency</v>
       </c>
       <c r="B688" t="str">
-        <v>تبعية خارجية</v>
+        <v>تبعية الأصول</v>
       </c>
       <c r="C688" t="str">
-        <v>Ārējā atkarība</v>
+        <v>Aktīvu atkarība</v>
       </c>
     </row>
     <row r="689">
       <c r="A689" t="str">
-        <v>KPI Measurement Required</v>
+        <v>External Dependency</v>
       </c>
       <c r="B689" t="str">
-        <v>قياس مؤشرات الأداء مطلوب</v>
+        <v>تبعية خارجية</v>
       </c>
       <c r="C689" t="str">
-        <v>Nepieciešams KPI mērījums</v>
+        <v>Ārējā atkarība</v>
       </c>
     </row>
     <row r="690">
       <c r="A690" t="str">
-        <v>PII Capture</v>
+        <v>KPI Measurement Required</v>
       </c>
       <c r="B690" t="str">
-        <v>التقاط البيانات الشخصية</v>
+        <v>قياس مؤشرات الأداء مطلوب</v>
       </c>
       <c r="C690" t="str">
-        <v>PII uztveršana</v>
+        <v>Nepieciešams KPI mērījums</v>
       </c>
     </row>
     <row r="691">
       <c r="A691" t="str">
-        <v>Auto-generated</v>
+        <v>PII Capture</v>
       </c>
       <c r="B691" t="str">
-        <v>يتم إنشاؤه تلقائياً</v>
+        <v>التقاط البيانات الشخصية</v>
       </c>
       <c r="C691" t="str">
-        <v>Automātiski ģenerēts</v>
+        <v>PII uztveršana</v>
       </c>
     </row>
     <row r="692">
       <c r="A692" t="str">
-        <v>Process created successfully</v>
+        <v>Auto-generated</v>
       </c>
       <c r="B692" t="str">
-        <v>تم إنشاء العملية بنجاح</v>
+        <v>يتم إنشاؤه تلقائياً</v>
       </c>
       <c r="C692" t="str">
-        <v>Process veiksmīgi izveidots</v>
+        <v>Automātiski ģenerēts</v>
       </c>
     </row>
     <row r="693">
       <c r="A693" t="str">
-        <v>Failed to create process</v>
+        <v>Auto-generated if left empty</v>
       </c>
       <c r="B693" t="str">
-        <v>فشل في إنشاء العملية</v>
+        <v>يتم إنشاؤه تلقائياً إذا تُرك فارغاً</v>
       </c>
       <c r="C693" t="str">
-        <v>Neizdevās izveidot procesu</v>
+        <v>Automātiski ģenerēts, ja atstāts tukšs</v>
       </c>
     </row>
     <row r="694">
       <c r="A694" t="str">
-        <v>Process updated successfully</v>
+        <v>Risk name is required</v>
       </c>
       <c r="B694" t="str">
-        <v>تم تحديث العملية بنجاح</v>
+        <v>اسم المخاطرة مطلوب</v>
       </c>
       <c r="C694" t="str">
-        <v>Process veiksmīgi atjaunināts</v>
+        <v>Riska nosaukums ir obligāts</v>
       </c>
     </row>
     <row r="695">
       <c r="A695" t="str">
-        <v>Failed to update process</v>
+        <v>Risk description is required</v>
       </c>
       <c r="B695" t="str">
-        <v>فشل في تحديث العملية</v>
+        <v>وصف المخاطرة مطلوب</v>
       </c>
       <c r="C695" t="str">
-        <v>Neizdevās atjaunināt procesu</v>
+        <v>Riska apraksts ir obligāts</v>
       </c>
     </row>
     <row r="696">
       <c r="A696" t="str">
-        <v>Please fill in required fields (Name and Process Type)</v>
+        <v>Inherent likelihood is required</v>
       </c>
       <c r="B696" t="str">
-        <v>يرجى ملء الحقول المطلوبة (الاسم ونوع العملية)</v>
+        <v>احتمالية المخاطر الكامنة مطلوبة</v>
       </c>
       <c r="C696" t="str">
-        <v>Lūdzu, aizpildiet obligātos laukus (Nosaukums un procesa tips)</v>
+        <v>Iedzimtā varbūtība ir obligāta</v>
       </c>
     </row>
     <row r="697">
       <c r="A697" t="str">
-        <v>Save Changes</v>
+        <v>Inherent impact is required</v>
       </c>
       <c r="B697" t="str">
-        <v>حفظ التغييرات</v>
+        <v>تأثير المخاطر الكامنة مطلوب</v>
       </c>
       <c r="C697" t="str">
-        <v>Saglabāt izmaiņas</v>
+        <v>Iedzimtā ietekme ir obligāta</v>
       </c>
     </row>
     <row r="698">
       <c r="A698" t="str">
-        <v>Reference ID</v>
+        <v>Residual likelihood is required</v>
       </c>
       <c r="B698" t="str">
-        <v>المعرف المرجعي</v>
+        <v>احتمالية المخاطر المتبقية مطلوبة</v>
       </c>
       <c r="C698" t="str">
-        <v>Atsauces ID</v>
+        <v>Atlikušā varbūtība ir obligāta</v>
       </c>
     </row>
     <row r="699">
       <c r="A699" t="str">
-        <v>Process Criticality</v>
+        <v>Residual impact is required</v>
       </c>
       <c r="B699" t="str">
-        <v>أهمية العملية</v>
+        <v>تأثير المخاطر المتبقية مطلوب</v>
       </c>
       <c r="C699" t="str">
-        <v>Procesa kritiskums</v>
+        <v>Atlikušā ietekme ir obligāta</v>
       </c>
     </row>
     <row r="700">
       <c r="A700" t="str">
-        <v>Process Frequency</v>
+        <v>Process created successfully</v>
       </c>
       <c r="B700" t="str">
-        <v>تكرار العملية</v>
+        <v>تم إنشاء العملية بنجاح</v>
       </c>
       <c r="C700" t="str">
-        <v>Procesa biežums</v>
+        <v>Process veiksmīgi izveidots</v>
       </c>
     </row>
     <row r="701">
       <c r="A701" t="str">
-        <v>Nature Of Implementation</v>
+        <v>Failed to create process</v>
       </c>
       <c r="B701" t="str">
-        <v>طبيعة التنفيذ</v>
+        <v>فشل في إنشاء العملية</v>
       </c>
       <c r="C701" t="str">
-        <v>Ieviešanas veids</v>
+        <v>Neizdevās izveidot procesu</v>
       </c>
     </row>
     <row r="702">
       <c r="A702" t="str">
-        <v>AI Risk</v>
+        <v>Process updated successfully</v>
       </c>
       <c r="B702" t="str">
-        <v>مخاطر الذكاء الاصطناعي</v>
+        <v>تم تحديث العملية بنجاح</v>
       </c>
       <c r="C702" t="str">
-        <v>AI risks</v>
+        <v>Process veiksmīgi atjaunināts</v>
       </c>
     </row>
     <row r="703">
       <c r="A703" t="str">
-        <v>AI Risk Evaluation</v>
+        <v>Failed to update process</v>
       </c>
       <c r="B703" t="str">
-        <v>تقييم مخاطر الذكاء الاصطناعي</v>
+        <v>فشل في تحديث العملية</v>
       </c>
       <c r="C703" t="str">
-        <v>AI risku novērtējums</v>
+        <v>Neizdevās atjaunināt procesu</v>
       </c>
     </row>
     <row r="704">
       <c r="A704" t="str">
-        <v>AI is identifying potential risks...</v>
+        <v>Please fill in required fields (Name and Process Type)</v>
       </c>
       <c r="B704" t="str">
-        <v>الذكاء الاصطناعي يحدد المخاطر المحتملة...</v>
+        <v>يرجى ملء الحقول المطلوبة (الاسم ونوع العملية)</v>
       </c>
       <c r="C704" t="str">
-        <v>AI identificē potenciālos riskus...</v>
+        <v>Lūdzu, aizpildiet obligātos laukus (Nosaukums un procesa tips)</v>
       </c>
     </row>
     <row r="705">
       <c r="A705" t="str">
-        <v>This may take up to 30 seconds</v>
+        <v>Save Changes</v>
       </c>
       <c r="B705" t="str">
-        <v>قد يستغرق هذا ما يصل إلى 30 ثانية</v>
+        <v>حفظ التغييرات</v>
       </c>
       <c r="C705" t="str">
-        <v>Tas var aizņemt līdz 30 sekundēm</v>
+        <v>Saglabāt izmaiņas</v>
       </c>
     </row>
     <row r="706">
       <c r="A706" t="str">
-        <v>Detected Risks</v>
+        <v>Reference ID</v>
       </c>
       <c r="B706" t="str">
-        <v>المخاطر المكتشفة</v>
+        <v>المعرف المرجعي</v>
       </c>
       <c r="C706" t="str">
-        <v>Atklātie riski</v>
+        <v>Atsauces ID</v>
       </c>
     </row>
     <row r="707">
       <c r="A707" t="str">
-        <v>The AI has identified the following risks, threats, and suggested controls...</v>
+        <v>Process Criticality</v>
       </c>
       <c r="B707" t="str">
-        <v>حدد الذكاء الاصطناعي المخاطر والتهديدات والضوابط المقترحة التالية...</v>
+        <v>أهمية العملية</v>
       </c>
       <c r="C707" t="str">
-        <v>AI ir identificējis šādus riskus, draudus un ieteiktos kontroles...</v>
+        <v>Procesa kritiskums</v>
       </c>
     </row>
     <row r="708">
       <c r="A708" t="str">
-        <v>Threats</v>
+        <v>Process Frequency</v>
       </c>
       <c r="B708" t="str">
-        <v>التهديدات</v>
+        <v>تكرار العملية</v>
       </c>
       <c r="C708" t="str">
-        <v>Draudi</v>
+        <v>Procesa biežums</v>
       </c>
     </row>
     <row r="709">
       <c r="A709" t="str">
-        <v>Suggested Controls</v>
+        <v>Nature Of Implementation</v>
       </c>
       <c r="B709" t="str">
-        <v>الضوابط المقترحة</v>
+        <v>طبيعة التنفيذ</v>
       </c>
       <c r="C709" t="str">
-        <v>Ieteiktās kontroles</v>
+        <v>Ieviešanas veids</v>
       </c>
     </row>
     <row r="710">
       <c r="A710" t="str">
-        <v>No risks generated yet.</v>
+        <v>AI Risk</v>
       </c>
       <c r="B710" t="str">
-        <v>لم يتم إنشاء مخاطر بعد.</v>
+        <v>مخاطر الذكاء الاصطناعي</v>
       </c>
       <c r="C710" t="str">
-        <v>Vēl nav ģenerēti riski.</v>
+        <v>AI risks</v>
       </c>
     </row>
     <row r="711">
       <c r="A711" t="str">
-        <v>AI Risks Generated</v>
+        <v>AI Risk Evaluation</v>
       </c>
       <c r="B711" t="str">
-        <v>تم إنشاء مخاطر الذكاء الاصطناعي</v>
+        <v>تقييم مخاطر الذكاء الاصطناعي</v>
       </c>
       <c r="C711" t="str">
-        <v>AI riski ģenerēti</v>
+        <v>AI risku novērtējums</v>
       </c>
     </row>
     <row r="712">
       <c r="A712" t="str">
-        <v>AI Generation Failed</v>
+        <v>AI is identifying potential risks...</v>
       </c>
       <c r="B712" t="str">
-        <v>فشل إنشاء الذكاء الاصطناعي</v>
+        <v>الذكاء الاصطناعي يحدد المخاطر المحتملة...</v>
       </c>
       <c r="C712" t="str">
-        <v>AI ģenerēšana neizdevās</v>
+        <v>AI identificē potenciālos riskus...</v>
       </c>
     </row>
     <row r="713">
       <c r="A713" t="str">
-        <v>Communication with AI service failed.</v>
+        <v>This may take up to 30 seconds</v>
       </c>
       <c r="B713" t="str">
-        <v>فشل الاتصال بخدمة الذكاء الاصطناعي.</v>
+        <v>قد يستغرق هذا ما يصل إلى 30 ثانية</v>
       </c>
       <c r="C713" t="str">
-        <v>Saziņa ar AI servisu neizdevās.</v>
+        <v>Tas var aizņemt līdz 30 sekundēm</v>
       </c>
     </row>
     <row r="714">
       <c r="A714" t="str">
-        <v>Please try again later.</v>
+        <v>Detected Risks</v>
       </c>
       <c r="B714" t="str">
-        <v>يرجى المحاولة مرة أخرى لاحقاً.</v>
+        <v>المخاطر المكتشفة</v>
       </c>
       <c r="C714" t="str">
-        <v>Lūdzu, mēģiniet vēlreiz vēlāk.</v>
+        <v>Atklātie riski</v>
       </c>
     </row>
     <row r="715">
       <c r="A715" t="str">
-        <v>Go to Risk Register</v>
+        <v>The AI has identified the following risks, threats, and suggested controls...</v>
       </c>
       <c r="B715" t="str">
-        <v>الذهاب إلى سجل المخاطر</v>
+        <v>حدد الذكاء الاصطناعي المخاطر والتهديدات والضوابط المقترحة التالية...</v>
       </c>
       <c r="C715" t="str">
-        <v>Doties uz risku reģistru</v>
+        <v>AI ir identificējis šādus riskus, draudus un ieteiktos kontroles...</v>
       </c>
     </row>
     <row r="716">
       <c r="A716" t="str">
-        <v>Add to Risk Register</v>
+        <v>Threats</v>
       </c>
       <c r="B716" t="str">
-        <v>إضافة إلى سجل المخاطر</v>
+        <v>التهديدات</v>
       </c>
       <c r="C716" t="str">
-        <v>Pievienot risku reģistram</v>
+        <v>Draudi</v>
       </c>
     </row>
     <row r="717">
       <c r="A717" t="str">
-        <v>Adding...</v>
+        <v>Suggested Controls</v>
       </c>
       <c r="B717" t="str">
-        <v>جاري الإضافة...</v>
+        <v>الضوابط المقترحة</v>
       </c>
       <c r="C717" t="str">
-        <v>Pievieno...</v>
+        <v>Ieteiktās kontroles</v>
       </c>
     </row>
     <row r="718">
       <c r="A718" t="str">
-        <v>No risks to add</v>
+        <v>No risks generated yet.</v>
       </c>
       <c r="B718" t="str">
-        <v>لا توجد مخاطر للإضافة</v>
+        <v>لم يتم إنشاء مخاطر بعد.</v>
       </c>
       <c r="C718" t="str">
-        <v>Nav risku, ko pievienot</v>
+        <v>Vēl nav ģenerēti riski.</v>
       </c>
     </row>
     <row r="719">
       <c r="A719" t="str">
-        <v>Keep at least one risk before adding to the register.</v>
+        <v>AI Risks Generated</v>
       </c>
       <c r="B719" t="str">
-        <v>احتفظ بخطر واحد على الأقل قبل الإضافة إلى السجل.</v>
+        <v>تم إنشاء مخاطر الذكاء الاصطناعي</v>
       </c>
       <c r="C719" t="str">
-        <v>Paturiet vismaz vienu risku pirms pievienošanas reģistram.</v>
+        <v>AI riski ģenerēti</v>
       </c>
     </row>
     <row r="720">
       <c r="A720" t="str">
-        <v>Risks have been added to the Risk Register.</v>
+        <v>AI Generation Failed</v>
       </c>
       <c r="B720" t="str">
-        <v>تمت إضافة المخاطر إلى سجل المخاطر.</v>
+        <v>فشل إنشاء الذكاء الاصطناعي</v>
       </c>
       <c r="C720" t="str">
-        <v>Riski ir pievienoti risku reģistram.</v>
+        <v>AI ģenerēšana neizdevās</v>
       </c>
     </row>
     <row r="721">
       <c r="A721" t="str">
-        <v>Adding to risk register timed out. Please try again.</v>
+        <v>Communication with AI service failed.</v>
       </c>
       <c r="B721" t="str">
-        <v>انتهت مهلة الإضافة إلى سجل المخاطر. يرجى المحاولة مرة أخرى.</v>
+        <v>فشل الاتصال بخدمة الذكاء الاصطناعي.</v>
       </c>
       <c r="C721" t="str">
-        <v>Pievienošanas reģistram laiks beidzās. Lūdzu, mēģiniet vēlreiz.</v>
+        <v>Saziņa ar AI servisu neizdevās.</v>
       </c>
     </row>
     <row r="722">
       <c r="A722" t="str">
-        <v>Failed to add risks to register</v>
+        <v>Please try again later.</v>
       </c>
       <c r="B722" t="str">
-        <v>فشل في إضافة المخاطر إلى السجل</v>
+        <v>يرجى المحاولة مرة أخرى لاحقاً.</v>
       </c>
       <c r="C722" t="str">
-        <v>Neizdevās pievienot riskus reģistram</v>
+        <v>Lūdzu, mēģiniet vēlreiz vēlāk.</v>
       </c>
     </row>
     <row r="723">
       <c r="A723" t="str">
-        <v>Failed to register risks</v>
+        <v>Go to Risk Register</v>
       </c>
       <c r="B723" t="str">
-        <v>فشل في تسجيل المخاطر</v>
+        <v>الذهاب إلى سجل المخاطر</v>
       </c>
       <c r="C723" t="str">
-        <v>Neizdevās reģistrēt riskus</v>
+        <v>Doties uz risku reģistru</v>
       </c>
     </row>
     <row r="724">
       <c r="A724" t="str">
-        <v>No risks in semantic result to register</v>
+        <v>Add to Risk Register</v>
       </c>
       <c r="B724" t="str">
-        <v>لا توجد مخاطر في نتيجة البحث الدلالي للتسجيل</v>
+        <v>إضافة إلى سجل المخاطر</v>
       </c>
       <c r="C724" t="str">
-        <v>Nav risku semantiskajā rezultātā reģistrēšanai</v>
+        <v>Pievienot risku reģistram</v>
       </c>
     </row>
     <row r="725">
       <c r="A725" t="str">
-        <v>Failed to add to risk register</v>
+        <v>Adding...</v>
       </c>
       <c r="B725" t="str">
-        <v>فشل في الإضافة إلى سجل المخاطر</v>
+        <v>جاري الإضافة...</v>
       </c>
       <c r="C725" t="str">
-        <v>Neizdevās pievienot risku reģistram</v>
+        <v>Pievieno...</v>
       </c>
     </row>
     <row r="726">
       <c r="A726" t="str">
-        <v>Add to Audit Plan</v>
+        <v>No risks to add</v>
       </c>
       <c r="B726" t="str">
-        <v>إضافة إلى خطة التدقيق</v>
+        <v>لا توجد مخاطر للإضافة</v>
       </c>
       <c r="C726" t="str">
-        <v>Pievienot audita plānam</v>
+        <v>Nav risku, ko pievienot</v>
       </c>
     </row>
     <row r="727">
       <c r="A727" t="str">
-        <v>Department information missing</v>
+        <v>Keep at least one risk before adding to the register.</v>
       </c>
       <c r="B727" t="str">
-        <v>معلومات القسم مفقودة</v>
+        <v>احتفظ بخطر واحد على الأقل قبل الإضافة إلى السجل.</v>
       </c>
       <c r="C727" t="str">
-        <v>Trūkst nodaļas informācijas</v>
+        <v>Paturiet vismaz vienu risku pirms pievienošanas reģistram.</v>
       </c>
     </row>
     <row r="728">
       <c r="A728" t="str">
-        <v>Failed to add to audit plan</v>
+        <v>Risks have been added to the Risk Register.</v>
       </c>
       <c r="B728" t="str">
-        <v>فشل في الإضافة إلى خطة التدقيق</v>
+        <v>تمت إضافة المخاطر إلى سجل المخاطر.</v>
       </c>
       <c r="C728" t="str">
-        <v>Neizdevās pievienot audita plānam</v>
+        <v>Riski ir pievienoti risku reģistram.</v>
       </c>
     </row>
     <row r="729">
       <c r="A729" t="str">
-        <v>Successfully added to Audit Planning!</v>
+        <v>Adding to risk register timed out. Please try again.</v>
       </c>
       <c r="B729" t="str">
-        <v>تمت الإضافة بنجاح إلى تخطيط التدقيق!</v>
+        <v>انتهت مهلة الإضافة إلى سجل المخاطر. يرجى المحاولة مرة أخرى.</v>
       </c>
       <c r="C729" t="str">
-        <v>Veiksmīgi pievienots audita plānošanai!</v>
+        <v>Pievienošanas reģistram laiks beidzās. Lūdzu, mēģiniet vēlreiz.</v>
       </c>
     </row>
     <row r="730">
       <c r="A730" t="str">
-        <v>Already Added</v>
+        <v>Failed to add risks to register</v>
       </c>
       <c r="B730" t="str">
-        <v>تمت الإضافة بالفعل</v>
+        <v>فشل في إضافة المخاطر إلى السجل</v>
       </c>
       <c r="C730" t="str">
-        <v>Jau pievienots</v>
+        <v>Neizdevās pievienot riskus reģistram</v>
       </c>
     </row>
     <row r="731">
       <c r="A731" t="str">
-        <v>This audit plan has already been added to Audit Planning.</v>
+        <v>Failed to register risks</v>
       </c>
       <c r="B731" t="str">
-        <v>تمت إضافة خطة التدقيق هذه بالفعل إلى تخطيط التدقيق.</v>
+        <v>فشل في تسجيل المخاطر</v>
       </c>
       <c r="C731" t="str">
-        <v>Šis audita plāns jau ir pievienots audita plānošanai.</v>
+        <v>Neizdevās reģistrēt riskus</v>
       </c>
     </row>
     <row r="732">
       <c r="A732" t="str">
-        <v>Failed to check status</v>
+        <v>No risks in semantic result to register</v>
       </c>
       <c r="B732" t="str">
-        <v>فشل في التحقق من الحالة</v>
+        <v>لا توجد مخاطر في نتيجة البحث الدلالي للتسجيل</v>
       </c>
       <c r="C732" t="str">
-        <v>Neizdevās pārbaudīt statusu</v>
+        <v>Nav risku semantiskajā rezultātā reģistrēšanai</v>
       </c>
     </row>
     <row r="733">
       <c r="A733" t="str">
-        <v>Remove risk</v>
+        <v>Failed to add to risk register</v>
       </c>
       <c r="B733" t="str">
-        <v>إزالة الخطر</v>
+        <v>فشل في الإضافة إلى سجل المخاطر</v>
       </c>
       <c r="C733" t="str">
-        <v>Noņemt risku</v>
+        <v>Neizdevās pievienot risku reģistram</v>
       </c>
     </row>
     <row r="734">
       <c r="A734" t="str">
-        <v>Remove risks you do not need; only the remaining risks will be sent to the next step.</v>
+        <v>Add to Audit Plan</v>
       </c>
       <c r="B734" t="str">
-        <v>أزل المخاطر التي لا تحتاجها؛ فقط المخاطر المتبقية سيتم إرسالها إلى الخطوة التالية.</v>
+        <v>إضافة إلى خطة التدقيق</v>
       </c>
       <c r="C734" t="str">
-        <v>Noņemiet riskus, kas nav nepieciešami; tikai atlikušie riski tiks nosūtīti nākamajā solī.</v>
+        <v>Pievienot audita plānam</v>
       </c>
     </row>
     <row r="735">
       <c r="A735" t="str">
-        <v>Perform BIA</v>
+        <v>Department information missing</v>
       </c>
       <c r="B735" t="str">
-        <v>إجراء تحليل تأثير الأعمال</v>
+        <v>معلومات القسم مفقودة</v>
       </c>
       <c r="C735" t="str">
-        <v>Veikt BIA</v>
+        <v>Trūkst nodaļas informācijas</v>
       </c>
     </row>
     <row r="736">
       <c r="A736" t="str">
-        <v>Submit For Approval</v>
+        <v>Failed to add to audit plan</v>
       </c>
       <c r="B736" t="str">
-        <v>إرسال للموافقة</v>
+        <v>فشل في الإضافة إلى خطة التدقيق</v>
       </c>
       <c r="C736" t="str">
-        <v>Iesniegt apstiprināšanai</v>
+        <v>Neizdevās pievienot audita plānam</v>
       </c>
     </row>
     <row r="737">
       <c r="A737" t="str">
-        <v>Status &amp; Approval</v>
+        <v>Successfully added to Audit Planning!</v>
       </c>
       <c r="B737" t="str">
-        <v>الحالة والموافقة</v>
+        <v>تمت الإضافة بنجاح إلى تخطيط التدقيق!</v>
       </c>
       <c r="C737" t="str">
-        <v>Statuss un apstiprinājums</v>
+        <v>Veiksmīgi pievienots audita plānošanai!</v>
       </c>
     </row>
     <row r="738">
       <c r="A738" t="str">
-        <v>Impact Assessment</v>
+        <v>Already Added</v>
       </c>
       <c r="B738" t="str">
-        <v>تقييم التأثير</v>
+        <v>تمت الإضافة بالفعل</v>
       </c>
       <c r="C738" t="str">
-        <v>Ietekmes novērtējums</v>
+        <v>Jau pievienots</v>
       </c>
     </row>
     <row r="739">
       <c r="A739" t="str">
-        <v>Recovery Metrics</v>
+        <v>This audit plan has already been added to Audit Planning.</v>
       </c>
       <c r="B739" t="str">
-        <v>مقاييس الاستعادة</v>
+        <v>تمت إضافة خطة التدقيق هذه بالفعل إلى تخطيط التدقيق.</v>
       </c>
       <c r="C739" t="str">
-        <v>Atjaunošanas metrikas</v>
+        <v>Šis audita plāns jau ir pievienots audita plānošanai.</v>
       </c>
     </row>
     <row r="740">
       <c r="A740" t="str">
-        <v>BIA Rating</v>
+        <v>Suggest Risks with AI</v>
       </c>
       <c r="B740" t="str">
-        <v>تصنيف تحليل تأثير الأعمال</v>
+        <v>اقتراح المخاطر بالذكاء الاصطناعي</v>
       </c>
       <c r="C740" t="str">
-        <v>BIA vērtējums</v>
+        <v>Ieteikt riskus ar AI</v>
       </c>
     </row>
     <row r="741">
       <c r="A741" t="str">
-        <v>Impact Rating</v>
+        <v>Add to Register</v>
       </c>
       <c r="B741" t="str">
-        <v>تصنيف التأثير</v>
+        <v>إضافة إلى السجل</v>
       </c>
       <c r="C741" t="str">
-        <v>Ietekmes vērtējums</v>
+        <v>Pievienot reģistram</v>
       </c>
     </row>
     <row r="742">
       <c r="A742" t="str">
-        <v>Note: The highest rating will be taken</v>
+        <v>Please select a department first</v>
       </c>
       <c r="B742" t="str">
-        <v>ملاحظة: سيتم أخذ أعلى تصنيف</v>
+        <v>يرجى تحديد قسم أولاً</v>
       </c>
       <c r="C742" t="str">
-        <v>Piezīme: Tiks ņemts augstākais vērtējums</v>
+        <v>Lūdzu, vispirms izvēlieties nodaļu</v>
       </c>
     </row>
     <row r="743">
       <c r="A743" t="str">
-        <v>RTO (Recovery Time Objective) - Hours</v>
+        <v>Only Audit Head can suggest risks with AI</v>
       </c>
       <c r="B743" t="str">
-        <v>هدف وقت الاستعادة - ساعات</v>
+        <v>فقط رئيس التدقيق يمكنه اقتراح المخاطر بالذكاء الاصطناعي</v>
       </c>
       <c r="C743" t="str">
-        <v>RTO (Atjaunošanas laika mērķis) - Stundas</v>
+        <v>Tikai audita vadītājs var ieteikt riskus ar AI</v>
       </c>
     </row>
     <row r="744">
       <c r="A744" t="str">
-        <v>RPO (Recovery Point Objective) - Hours</v>
+        <v>Only Audit Head can add risks to register</v>
       </c>
       <c r="B744" t="str">
-        <v>هدف نقطة الاستعادة - ساعات</v>
+        <v>فقط رئيس التدقيق يمكنه إضافة المخاطر إلى السجل</v>
       </c>
       <c r="C744" t="str">
-        <v>RPO (Atjaunošanas punkta mērķis) - Stundas</v>
+        <v>Tikai audita vadītājs var pievienot riskus reģistram</v>
       </c>
     </row>
     <row r="745">
       <c r="A745" t="str">
-        <v>N/A</v>
+        <v>Failed to check status</v>
       </c>
       <c r="B745" t="str">
-        <v>غير متاح</v>
+        <v>فشل في التحقق من الحالة</v>
       </c>
       <c r="C745" t="str">
-        <v>Nav piemērojams</v>
+        <v>Neizdevās pārbaudīt statusu</v>
       </c>
     </row>
     <row r="746">
       <c r="A746" t="str">
-        <v>KPI Details</v>
+        <v>Remove risk</v>
       </c>
       <c r="B746" t="str">
-        <v>تفاصيل مؤشرات الأداء</v>
+        <v>إزالة الخطر</v>
       </c>
       <c r="C746" t="str">
-        <v>KPI detaļas</v>
+        <v>Noņemt risku</v>
       </c>
     </row>
     <row r="747">
       <c r="A747" t="str">
-        <v>Performance Chart</v>
+        <v>Remove risks you do not need; only the remaining risks will be sent to the next step.</v>
       </c>
       <c r="B747" t="str">
-        <v>مخطط الأداء</v>
+        <v>أزل المخاطر التي لا تحتاجها؛ فقط المخاطر المتبقية سيتم إرسالها إلى الخطوة التالية.</v>
       </c>
       <c r="C747" t="str">
-        <v>Veiktspējas diagramma</v>
+        <v>Noņemiet riskus, kas nav nepieciešami; tikai atlikušie riski tiks nosūtīti nākamajā solī.</v>
       </c>
     </row>
     <row r="748">
       <c r="A748" t="str">
-        <v>KPI Configuration</v>
+        <v>Perform BIA</v>
       </c>
       <c r="B748" t="str">
-        <v>إعدادات مؤشرات الأداء</v>
+        <v>إجراء تحليل تأثير الأعمال</v>
       </c>
       <c r="C748" t="str">
-        <v>KPI konfigurācija</v>
+        <v>Veikt BIA</v>
       </c>
     </row>
     <row r="749">
       <c r="A749" t="str">
-        <v>KPI Records</v>
+        <v>Submit For Approval</v>
       </c>
       <c r="B749" t="str">
-        <v>سجلات مؤشرات الأداء</v>
+        <v>إرسال للموافقة</v>
       </c>
       <c r="C749" t="str">
-        <v>KPI ieraksti</v>
+        <v>Iesniegt apstiprināšanai</v>
       </c>
     </row>
     <row r="750">
       <c r="A750" t="str">
-        <v>Year</v>
+        <v>Status &amp; Approval</v>
       </c>
       <c r="B750" t="str">
-        <v>السنة</v>
+        <v>الحالة والموافقة</v>
       </c>
       <c r="C750" t="str">
-        <v>Gads</v>
+        <v>Statuss un apstiprinājums</v>
       </c>
     </row>
     <row r="751">
       <c r="A751" t="str">
-        <v>Achieved Value</v>
+        <v>Impact Assessment</v>
       </c>
       <c r="B751" t="str">
-        <v>القيمة المحققة</v>
+        <v>تقييم التأثير</v>
       </c>
       <c r="C751" t="str">
-        <v>Sasniegtā vērtība</v>
+        <v>Ietekmes novērtējums</v>
       </c>
     </row>
     <row r="752">
       <c r="A752" t="str">
-        <v>Expected Value</v>
+        <v>Recovery Metrics</v>
       </c>
       <c r="B752" t="str">
-        <v>القيمة المتوقعة</v>
+        <v>مقاييس الاستعادة</v>
       </c>
       <c r="C752" t="str">
-        <v>Gaidāmā vērtība</v>
+        <v>Atjaunošanas metrikas</v>
       </c>
     </row>
     <row r="753">
       <c r="A753" t="str">
-        <v>KPI Objective</v>
+        <v>BIA Rating</v>
       </c>
       <c r="B753" t="str">
-        <v>هدف مؤشر الأداء</v>
+        <v>تصنيف تحليل تأثير الأعمال</v>
       </c>
       <c r="C753" t="str">
-        <v>KPI mērķis</v>
+        <v>BIA vērtējums</v>
       </c>
     </row>
     <row r="754">
       <c r="A754" t="str">
-        <v>Enter Objective</v>
+        <v>Impact Rating</v>
       </c>
       <c r="B754" t="str">
-        <v>أدخل الهدف</v>
+        <v>تصنيف التأثير</v>
       </c>
       <c r="C754" t="str">
-        <v>Ievadiet mērķi</v>
+        <v>Ietekmes vērtējums</v>
       </c>
     </row>
     <row r="755">
       <c r="A755" t="str">
-        <v>KPI Description</v>
+        <v>Note: The highest rating will be taken</v>
       </c>
       <c r="B755" t="str">
-        <v>وصف مؤشر الأداء</v>
+        <v>ملاحظة: سيتم أخذ أعلى تصنيف</v>
       </c>
       <c r="C755" t="str">
-        <v>KPI apraksts</v>
+        <v>Piezīme: Tiks ņemts augstākais vērtējums</v>
       </c>
     </row>
     <row r="756">
       <c r="A756" t="str">
-        <v>Enter Description</v>
+        <v>RTO (Recovery Time Objective) - Hours</v>
       </c>
       <c r="B756" t="str">
-        <v>أدخل الوصف</v>
+        <v>هدف وقت الاستعادة - ساعات</v>
       </c>
       <c r="C756" t="str">
-        <v>Ievadiet aprakstu</v>
+        <v>RTO (Atjaunošanas laika mērķis) - Stundas</v>
       </c>
     </row>
     <row r="757">
       <c r="A757" t="str">
-        <v>KPI Data Source</v>
+        <v>RPO (Recovery Point Objective) - Hours</v>
       </c>
       <c r="B757" t="str">
-        <v>مصدر بيانات مؤشر الأداء</v>
+        <v>هدف نقطة الاستعادة - ساعات</v>
       </c>
       <c r="C757" t="str">
-        <v>KPI datu avots</v>
+        <v>RPO (Atjaunošanas punkta mērķis) - Stundas</v>
       </c>
     </row>
     <row r="758">
       <c r="A758" t="str">
-        <v>Enter Data Source</v>
+        <v>N/A</v>
       </c>
       <c r="B758" t="str">
-        <v>أدخل مصدر البيانات</v>
+        <v>غير متاح</v>
       </c>
       <c r="C758" t="str">
-        <v>Ievadiet datu avotu</v>
+        <v>Nav piemērojams</v>
       </c>
     </row>
     <row r="759">
       <c r="A759" t="str">
-        <v>KPI Measurement Formula</v>
+        <v>KPI Details</v>
       </c>
       <c r="B759" t="str">
-        <v>صيغة قياس مؤشر الأداء</v>
+        <v>تفاصيل مؤشرات الأداء</v>
       </c>
       <c r="C759" t="str">
-        <v>KPI mērīšanas formula</v>
+        <v>KPI detaļas</v>
       </c>
     </row>
     <row r="760">
       <c r="A760" t="str">
-        <v>Enter the KPI Calculation Formula</v>
+        <v>Performance Chart</v>
       </c>
       <c r="B760" t="str">
-        <v>أدخل صيغة حساب مؤشر الأداء</v>
+        <v>مخطط الأداء</v>
       </c>
       <c r="C760" t="str">
-        <v>Ievadiet KPI aprēķina formulu</v>
+        <v>Veiktspējas diagramma</v>
       </c>
     </row>
     <row r="761">
       <c r="A761" t="str">
-        <v>Targeted Achieved Value</v>
+        <v>KPI Configuration</v>
       </c>
       <c r="B761" t="str">
-        <v>القيمة المستهدفة المحققة</v>
+        <v>إعدادات مؤشرات الأداء</v>
       </c>
       <c r="C761" t="str">
-        <v>Mērķa sasniegtā vērtība</v>
+        <v>KPI konfigurācija</v>
       </c>
     </row>
     <row r="762">
       <c r="A762" t="str">
-        <v>No KPI records yet</v>
+        <v>KPI Records</v>
       </c>
       <c r="B762" t="str">
-        <v>لا توجد سجلات مؤشرات أداء بعد</v>
+        <v>سجلات مؤشرات الأداء</v>
       </c>
       <c r="C762" t="str">
-        <v>Vēl nav KPI ierakstu</v>
+        <v>KPI ieraksti</v>
       </c>
     </row>
     <row r="763">
       <c r="A763" t="str">
-        <v>No KPI Data</v>
+        <v>Year</v>
       </c>
       <c r="B763" t="str">
-        <v>لا توجد بيانات مؤشرات أداء</v>
+        <v>السنة</v>
       </c>
       <c r="C763" t="str">
-        <v>Nav KPI datu</v>
+        <v>Gads</v>
       </c>
     </row>
     <row r="764">
       <c r="A764" t="str">
-        <v>No processes have KPI measurement enabled...</v>
+        <v>Achieved Value</v>
       </c>
       <c r="B764" t="str">
-        <v>لم يتم تمكين قياس مؤشرات الأداء لأي عملية...</v>
+        <v>القيمة المحققة</v>
       </c>
       <c r="C764" t="str">
-        <v>Nevienam procesam nav iespējots KPI mērījums...</v>
+        <v>Sasniegtā vērtība</v>
       </c>
     </row>
     <row r="765">
       <c r="A765" t="str">
-        <v>Unassigned</v>
+        <v>Expected Value</v>
       </c>
       <c r="B765" t="str">
-        <v>غير معين</v>
+        <v>القيمة المتوقعة</v>
       </c>
       <c r="C765" t="str">
-        <v>Nepiešķirts</v>
+        <v>Gaidāmā vērtība</v>
       </c>
     </row>
     <row r="766">
       <c r="A766" t="str">
-        <v>Primary</v>
+        <v>KPI Objective</v>
       </c>
       <c r="B766" t="str">
-        <v>أساسي</v>
+        <v>هدف مؤشر الأداء</v>
       </c>
       <c r="C766" t="str">
-        <v>Primārais</v>
+        <v>KPI mērķis</v>
       </c>
     </row>
     <row r="767">
       <c r="A767" t="str">
-        <v>Supporting</v>
+        <v>Enter Objective</v>
       </c>
       <c r="B767" t="str">
-        <v>داعم</v>
+        <v>أدخل الهدف</v>
       </c>
       <c r="C767" t="str">
-        <v>Atbalsta</v>
+        <v>Ievadiet mērķi</v>
       </c>
     </row>
     <row r="768">
       <c r="A768" t="str">
-        <v>Manual</v>
+        <v>KPI Description</v>
       </c>
       <c r="B768" t="str">
-        <v>يدوي</v>
+        <v>وصف مؤشر الأداء</v>
       </c>
       <c r="C768" t="str">
-        <v>Manuāls</v>
+        <v>KPI apraksts</v>
       </c>
     </row>
     <row r="769">
       <c r="A769" t="str">
-        <v>Automated</v>
+        <v>Enter Description</v>
       </c>
       <c r="B769" t="str">
-        <v>آلي</v>
+        <v>أدخل الوصف</v>
       </c>
       <c r="C769" t="str">
-        <v>Automatizēts</v>
+        <v>Ievadiet aprakstu</v>
       </c>
     </row>
     <row r="770">
       <c r="A770" t="str">
-        <v>Manual + Automated</v>
+        <v>KPI Data Source</v>
       </c>
       <c r="B770" t="str">
-        <v>يدوي + آلي</v>
+        <v>مصدر بيانات مؤشر الأداء</v>
       </c>
       <c r="C770" t="str">
-        <v>Manuāls + Automatizēts</v>
+        <v>KPI datu avots</v>
       </c>
     </row>
     <row r="771">
       <c r="A771" t="str">
-        <v>Branch Office</v>
+        <v>Enter Data Source</v>
       </c>
       <c r="B771" t="str">
-        <v>فرع المكتب</v>
+        <v>أدخل مصدر البيانات</v>
       </c>
       <c r="C771" t="str">
-        <v>Filiāles birojs</v>
+        <v>Ievadiet datu avotu</v>
       </c>
     </row>
     <row r="772">
       <c r="A772" t="str">
-        <v>Remote</v>
+        <v>KPI Measurement Formula</v>
       </c>
       <c r="B772" t="str">
-        <v>عن بعد</v>
+        <v>صيغة قياس مؤشر الأداء</v>
       </c>
       <c r="C772" t="str">
-        <v>Attālināti</v>
+        <v>KPI mērīšanas formula</v>
       </c>
     </row>
     <row r="773">
       <c r="A773" t="str">
-        <v>Select frequency</v>
+        <v>Enter the KPI Calculation Formula</v>
       </c>
       <c r="B773" t="str">
-        <v>اختر التكرار</v>
+        <v>أدخل صيغة حساب مؤشر الأداء</v>
       </c>
       <c r="C773" t="str">
-        <v>Izvēlieties biežumu</v>
+        <v>Ievadiet KPI aprēķina formulu</v>
       </c>
     </row>
     <row r="774">
       <c r="A774" t="str">
-        <v>Bi-annually</v>
+        <v>Targeted Achieved Value</v>
       </c>
       <c r="B774" t="str">
-        <v>نصف سنوي</v>
+        <v>القيمة المستهدفة المحققة</v>
       </c>
       <c r="C774" t="str">
-        <v>Divreiz gadā</v>
+        <v>Mērķa sasniegtā vērtība</v>
       </c>
     </row>
     <row r="775">
       <c r="A775" t="str">
+        <v>No KPI records yet</v>
+      </c>
+      <c r="B775" t="str">
+        <v>لا توجد سجلات مؤشرات أداء بعد</v>
+      </c>
+      <c r="C775" t="str">
+        <v>Vēl nav KPI ierakstu</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="str">
+        <v>No KPI Data</v>
+      </c>
+      <c r="B776" t="str">
+        <v>لا توجد بيانات مؤشرات أداء</v>
+      </c>
+      <c r="C776" t="str">
+        <v>Nav KPI datu</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="str">
+        <v>No processes have KPI measurement enabled...</v>
+      </c>
+      <c r="B777" t="str">
+        <v>لم يتم تمكين قياس مؤشرات الأداء لأي عملية...</v>
+      </c>
+      <c r="C777" t="str">
+        <v>Nevienam procesam nav iespējots KPI mērījums...</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="str">
+        <v>Unassigned</v>
+      </c>
+      <c r="B778" t="str">
+        <v>غير معين</v>
+      </c>
+      <c r="C778" t="str">
+        <v>Nepiešķirts</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="str">
+        <v>Primary</v>
+      </c>
+      <c r="B779" t="str">
+        <v>أساسي</v>
+      </c>
+      <c r="C779" t="str">
+        <v>Primārais</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="str">
+        <v>Supporting</v>
+      </c>
+      <c r="B780" t="str">
+        <v>داعم</v>
+      </c>
+      <c r="C780" t="str">
+        <v>Atbalsta</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="B781" t="str">
+        <v>يدوي</v>
+      </c>
+      <c r="C781" t="str">
+        <v>Manuāls</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="str">
+        <v>Automated</v>
+      </c>
+      <c r="B782" t="str">
+        <v>آلي</v>
+      </c>
+      <c r="C782" t="str">
+        <v>Automatizēts</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="str">
+        <v>Manual + Automated</v>
+      </c>
+      <c r="B783" t="str">
+        <v>يدوي + آلي</v>
+      </c>
+      <c r="C783" t="str">
+        <v>Manuāls + Automatizēts</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="str">
+        <v>Branch Office</v>
+      </c>
+      <c r="B784" t="str">
+        <v>فرع المكتب</v>
+      </c>
+      <c r="C784" t="str">
+        <v>Filiāles birojs</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="str">
+        <v>Remote</v>
+      </c>
+      <c r="B785" t="str">
+        <v>عن بعد</v>
+      </c>
+      <c r="C785" t="str">
+        <v>Attālināti</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="str">
+        <v>Select frequency</v>
+      </c>
+      <c r="B786" t="str">
+        <v>اختر التكرار</v>
+      </c>
+      <c r="C786" t="str">
+        <v>Izvēlieties biežumu</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="str">
+        <v>Bi-annually</v>
+      </c>
+      <c r="B787" t="str">
+        <v>نصف سنوي</v>
+      </c>
+      <c r="C787" t="str">
+        <v>Divreiz gadā</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="str">
         <v>As needed</v>
       </c>
-      <c r="B775" t="str">
+      <c r="B788" t="str">
         <v>حسب الحاجة</v>
       </c>
-      <c r="C775" t="str">
+      <c r="C788" t="str">
         <v>Pēc vajadzības</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="str">
+        <v>Imported</v>
+      </c>
+      <c r="B789" t="str">
+        <v>تم استيراد</v>
+      </c>
+      <c r="C789" t="str">
+        <v>Importēts</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="str">
+        <v>categories</v>
+      </c>
+      <c r="B790" t="str">
+        <v>فئات</v>
+      </c>
+      <c r="C790" t="str">
+        <v>kategorijas</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="str">
+        <v>sub-categories</v>
+      </c>
+      <c r="B791" t="str">
+        <v>فئات فرعية</v>
+      </c>
+      <c r="C791" t="str">
+        <v>apakškategorijas</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="str">
+        <v>groups</v>
+      </c>
+      <c r="B792" t="str">
+        <v>مجموعات</v>
+      </c>
+      <c r="C792" t="str">
+        <v>grupas</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="str">
+        <v>sensitivities</v>
+      </c>
+      <c r="B793" t="str">
+        <v>حساسيات</v>
+      </c>
+      <c r="C793" t="str">
+        <v>jutīgumi</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="str">
+        <v>assets</v>
+      </c>
+      <c r="B794" t="str">
+        <v>أصول</v>
+      </c>
+      <c r="C794" t="str">
+        <v>aktīvi</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="str">
+        <v>lifecycle statuses</v>
+      </c>
+      <c r="B795" t="str">
+        <v>حالات دورة الحياة</v>
+      </c>
+      <c r="C795" t="str">
+        <v>dzīves cikla statusi</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="str">
+        <v>failed</v>
+      </c>
+      <c r="B796" t="str">
+        <v>فشل</v>
+      </c>
+      <c r="C796" t="str">
+        <v>neizdevās</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="str">
+        <v>category not found</v>
+      </c>
+      <c r="B797" t="str">
+        <v>الفئة غير موجودة</v>
+      </c>
+      <c r="C797" t="str">
+        <v>kategorija nav atrasta</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C775"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C797"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add RTL support for Evidence dashboard and Arabic translations for Governance/Evidence pages
- Add RTL direction, Tabs dir, and dialog RTL support to Evidence dashboard
- Translate recurrence options (Weekly/Monthly/Quarterly/Yearly) in Governance detail page
- Add 70+ missing Arabic/Latvian translations for Evidence and Governance detail pages
- Fix documentType Badge in Link Governance dialog to use t() wrapper

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1137"/>
+  <dimension ref="A1:C1403"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -12911,9 +12911,2935 @@
         <v>Nodaļas nosaukums</v>
       </c>
     </row>
+    <row r="1138">
+      <c r="A1138" t="str">
+        <v>Integrated Frameworks</v>
+      </c>
+      <c r="B1138" t="str">
+        <v>الأطر المتكاملة</v>
+      </c>
+      <c r="C1138" t="str">
+        <v>Integrētie ietvari</v>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="str">
+        <v>New Framework</v>
+      </c>
+      <c r="B1139" t="str">
+        <v>إطار جديد</v>
+      </c>
+      <c r="C1139" t="str">
+        <v>Jauns ietvars</v>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="str">
+        <v>New Framework (AI)</v>
+      </c>
+      <c r="B1140" t="str">
+        <v>إطار جديد (ذكاء اصطناعي)</v>
+      </c>
+      <c r="C1140" t="str">
+        <v>Jauns ietvars (MI)</v>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="str">
+        <v>Search frameworks...</v>
+      </c>
+      <c r="B1141" t="str">
+        <v>البحث في الأطر...</v>
+      </c>
+      <c r="C1141" t="str">
+        <v>Meklēt ietvarus...</v>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="str">
+        <v>All Statuses</v>
+      </c>
+      <c r="B1142" t="str">
+        <v>جميع الحالات</v>
+      </c>
+      <c r="C1142" t="str">
+        <v>Visi statusi</v>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="str">
+        <v>Grouping</v>
+      </c>
+      <c r="B1143" t="str">
+        <v>التصنيف</v>
+      </c>
+      <c r="C1143" t="str">
+        <v>Grupēšana</v>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="str">
+        <v>Function Grouping</v>
+      </c>
+      <c r="B1144" t="str">
+        <v>تصنيف الوظائف</v>
+      </c>
+      <c r="C1144" t="str">
+        <v>Funkciju grupēšana</v>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="str">
+        <v>No controls linked yet</v>
+      </c>
+      <c r="B1145" t="str">
+        <v>لا توجد ضوابط مرتبطة بعد</v>
+      </c>
+      <c r="C1145" t="str">
+        <v>Vēl nav saistītu kontroles pasākumu</v>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="str">
+        <v>Link controls to requirements in the framework to see them here</v>
+      </c>
+      <c r="B1146" t="str">
+        <v>اربط الضوابط بالمتطلبات في الإطار لرؤيتها هنا</v>
+      </c>
+      <c r="C1146" t="str">
+        <v>Saistiet kontroles pasākumus ar prasībām ietvarā, lai tos redzētu šeit</v>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="str">
+        <v>Policies</v>
+      </c>
+      <c r="B1147" t="str">
+        <v>السياسات</v>
+      </c>
+      <c r="C1147" t="str">
+        <v>Politikas</v>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="str">
+        <v>All Requirements</v>
+      </c>
+      <c r="B1148" t="str">
+        <v>جميع المتطلبات</v>
+      </c>
+      <c r="C1148" t="str">
+        <v>Visas prasības</v>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="str">
+        <v>SOA</v>
+      </c>
+      <c r="B1149" t="str">
+        <v>بيان التطبيق</v>
+      </c>
+      <c r="C1149" t="str">
+        <v>SOA</v>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="str">
+        <v>Audit Logs</v>
+      </c>
+      <c r="B1150" t="str">
+        <v>سجلات التدقيق</v>
+      </c>
+      <c r="C1150" t="str">
+        <v>Audita žurnāli</v>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="str">
+        <v>Search requirements...</v>
+      </c>
+      <c r="B1151" t="str">
+        <v>البحث في المتطلبات...</v>
+      </c>
+      <c r="C1151" t="str">
+        <v>Meklēt prasības...</v>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="str">
+        <v>New Requirement</v>
+      </c>
+      <c r="B1152" t="str">
+        <v>متطلب جديد</v>
+      </c>
+      <c r="C1152" t="str">
+        <v>Jauna prasība</v>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="str">
+        <v>Partial</v>
+      </c>
+      <c r="B1153" t="str">
+        <v>جزئي</v>
+      </c>
+      <c r="C1153" t="str">
+        <v>Daļējs</v>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="str">
+        <v>requirements</v>
+      </c>
+      <c r="B1154" t="str">
+        <v>متطلبات</v>
+      </c>
+      <c r="C1154" t="str">
+        <v>prasības</v>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="str">
+        <v>Requirement</v>
+      </c>
+      <c r="B1155" t="str">
+        <v>المتطلب</v>
+      </c>
+      <c r="C1155" t="str">
+        <v>Prasība</v>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="str">
+        <v>Requirement Name</v>
+      </c>
+      <c r="B1156" t="str">
+        <v>اسم المتطلب</v>
+      </c>
+      <c r="C1156" t="str">
+        <v>Prasības nosaukums</v>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="str">
+        <v>Requirement Category</v>
+      </c>
+      <c r="B1157" t="str">
+        <v>فئة المتطلب</v>
+      </c>
+      <c r="C1157" t="str">
+        <v>Prasības kategorija</v>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="str">
+        <v>Requirement Code</v>
+      </c>
+      <c r="B1158" t="str">
+        <v>رمز المتطلب</v>
+      </c>
+      <c r="C1158" t="str">
+        <v>Prasības kods</v>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="str">
+        <v>Requirement Description</v>
+      </c>
+      <c r="B1159" t="str">
+        <v>وصف المتطلب</v>
+      </c>
+      <c r="C1159" t="str">
+        <v>Prasības apraksts</v>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="str">
+        <v>Requirement Type</v>
+      </c>
+      <c r="B1160" t="str">
+        <v>نوع المتطلب</v>
+      </c>
+      <c r="C1160" t="str">
+        <v>Prasības veids</v>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="str">
+        <v>Chapter Type</v>
+      </c>
+      <c r="B1161" t="str">
+        <v>نوع الفصل</v>
+      </c>
+      <c r="C1161" t="str">
+        <v>Nodaļas veids</v>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="str">
+        <v>Add Requirement</v>
+      </c>
+      <c r="B1162" t="str">
+        <v>إضافة متطلب</v>
+      </c>
+      <c r="C1162" t="str">
+        <v>Pievienot prasību</v>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="str">
+        <v>Update Requirement</v>
+      </c>
+      <c r="B1163" t="str">
+        <v>تحديث المتطلب</v>
+      </c>
+      <c r="C1163" t="str">
+        <v>Atjaunināt prasību</v>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="str">
+        <v>Mandatory</v>
+      </c>
+      <c r="B1164" t="str">
+        <v>إلزامي</v>
+      </c>
+      <c r="C1164" t="str">
+        <v>Obligāts</v>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="str">
+        <v>Additional</v>
+      </c>
+      <c r="B1165" t="str">
+        <v>إضافي</v>
+      </c>
+      <c r="C1165" t="str">
+        <v>Papildu</v>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="str">
+        <v>Process Domain</v>
+      </c>
+      <c r="B1166" t="str">
+        <v>مجال العمليات</v>
+      </c>
+      <c r="C1166" t="str">
+        <v>Procesu domēns</v>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="str">
+        <v>Technical Domain</v>
+      </c>
+      <c r="B1167" t="str">
+        <v>المجال التقني</v>
+      </c>
+      <c r="C1167" t="str">
+        <v>Tehniskais domēns</v>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="str">
+        <v>Applicability</v>
+      </c>
+      <c r="B1168" t="str">
+        <v>قابلية التطبيق</v>
+      </c>
+      <c r="C1168" t="str">
+        <v>Piemērojamība</v>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="str">
+        <v>Implementation</v>
+      </c>
+      <c r="B1169" t="str">
+        <v>التنفيذ</v>
+      </c>
+      <c r="C1169" t="str">
+        <v>Ieviešana</v>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="str">
+        <v>Linked Controls</v>
+      </c>
+      <c r="B1170" t="str">
+        <v>الضوابط المرتبطة</v>
+      </c>
+      <c r="C1170" t="str">
+        <v>Saistītās kontroles</v>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="str">
+        <v>Link</v>
+      </c>
+      <c r="B1171" t="str">
+        <v>ربط</v>
+      </c>
+      <c r="C1171" t="str">
+        <v>Saistīt</v>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="str">
+        <v>No controls found</v>
+      </c>
+      <c r="B1172" t="str">
+        <v>لم يتم العثور على ضوابط</v>
+      </c>
+      <c r="C1172" t="str">
+        <v>Kontroles nav atrastas</v>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="str">
+        <v>Control Select</v>
+      </c>
+      <c r="B1173" t="str">
+        <v>اختيار الضوابط</v>
+      </c>
+      <c r="C1173" t="str">
+        <v>Kontroles izvēle</v>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="str">
+        <v>All Functions</v>
+      </c>
+      <c r="B1174" t="str">
+        <v>جميع الوظائف</v>
+      </c>
+      <c r="C1174" t="str">
+        <v>Visas funkcijas</v>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="str">
+        <v>Search by code, name</v>
+      </c>
+      <c r="B1175" t="str">
+        <v>البحث بالرمز أو الاسم</v>
+      </c>
+      <c r="C1175" t="str">
+        <v>Meklēt pēc koda, nosaukuma</v>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="str">
+        <v>Exception Code</v>
+      </c>
+      <c r="B1176" t="str">
+        <v>رمز الاستثناء</v>
+      </c>
+      <c r="C1176" t="str">
+        <v>Izņēmuma kods</v>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="str">
+        <v>Exception Name</v>
+      </c>
+      <c r="B1177" t="str">
+        <v>اسم الاستثناء</v>
+      </c>
+      <c r="C1177" t="str">
+        <v>Izņēmuma nosaukums</v>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="str">
+        <v>Description/Justification</v>
+      </c>
+      <c r="B1178" t="str">
+        <v>الوصف/المبرر</v>
+      </c>
+      <c r="C1178" t="str">
+        <v>Apraksts/Pamatojums</v>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="str">
+        <v>Provide justification for this exception</v>
+      </c>
+      <c r="B1179" t="str">
+        <v>قدم مبرراً لهذا الاستثناء</v>
+      </c>
+      <c r="C1179" t="str">
+        <v>Sniedziet pamatojumu šim izņēmumam</v>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="str">
+        <v>Authorised</v>
+      </c>
+      <c r="B1180" t="str">
+        <v>مصرح به</v>
+      </c>
+      <c r="C1180" t="str">
+        <v>Autorizēts</v>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="str">
+        <v>Submitted for Closure</v>
+      </c>
+      <c r="B1181" t="str">
+        <v>مقدم للإغلاق</v>
+      </c>
+      <c r="C1181" t="str">
+        <v>Iesniegts slēgšanai</v>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="str">
+        <v>Risk Accepted</v>
+      </c>
+      <c r="B1182" t="str">
+        <v>المخاطر مقبولة</v>
+      </c>
+      <c r="C1182" t="str">
+        <v>Risks pieņemts</v>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="str">
+        <v>Enter exception name</v>
+      </c>
+      <c r="B1183" t="str">
+        <v>أدخل اسم الاستثناء</v>
+      </c>
+      <c r="C1183" t="str">
+        <v>Ievadiet izņēmuma nosaukumu</v>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="str">
+        <v>Partial Compliant</v>
+      </c>
+      <c r="B1184" t="str">
+        <v>متوافق جزئياً</v>
+      </c>
+      <c r="C1184" t="str">
+        <v>Daļēji atbilstošs</v>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="str">
+        <v>No Requirements</v>
+      </c>
+      <c r="B1185" t="str">
+        <v>لا توجد متطلبات</v>
+      </c>
+      <c r="C1185" t="str">
+        <v>Nav prasību</v>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="str">
+        <v>Add your first requirement to get started.</v>
+      </c>
+      <c r="B1186" t="str">
+        <v>أضف أول متطلب للبدء.</v>
+      </c>
+      <c r="C1186" t="str">
+        <v>Pievienojiet savu pirmo prasību, lai sāktu.</v>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="str">
+        <v>Search logs...</v>
+      </c>
+      <c r="B1187" t="str">
+        <v>البحث في السجلات...</v>
+      </c>
+      <c r="C1187" t="str">
+        <v>Meklēt žurnālos...</v>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="str">
+        <v>All Actions</v>
+      </c>
+      <c r="B1188" t="str">
+        <v>جميع الإجراءات</v>
+      </c>
+      <c r="C1188" t="str">
+        <v>Visas darbības</v>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="str">
+        <v>Linked</v>
+      </c>
+      <c r="B1189" t="str">
+        <v>مرتبط</v>
+      </c>
+      <c r="C1189" t="str">
+        <v>Saistīts</v>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="str">
+        <v>Unlinked</v>
+      </c>
+      <c r="B1190" t="str">
+        <v>غير مرتبط</v>
+      </c>
+      <c r="C1190" t="str">
+        <v>Atsaistīts</v>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="str">
+        <v>Created</v>
+      </c>
+      <c r="B1191" t="str">
+        <v>تم الإنشاء</v>
+      </c>
+      <c r="C1191" t="str">
+        <v>Izveidots</v>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="str">
+        <v>Updated</v>
+      </c>
+      <c r="B1192" t="str">
+        <v>تم التحديث</v>
+      </c>
+      <c r="C1192" t="str">
+        <v>Atjaunināts</v>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="str">
+        <v>Deleted</v>
+      </c>
+      <c r="B1193" t="str">
+        <v>تم الحذف</v>
+      </c>
+      <c r="C1193" t="str">
+        <v>Dzēsts</v>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="str">
+        <v>Exported</v>
+      </c>
+      <c r="B1194" t="str">
+        <v>تم التصدير</v>
+      </c>
+      <c r="C1194" t="str">
+        <v>Eksportēts</v>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="str">
+        <v>SOA report exported successfully</v>
+      </c>
+      <c r="B1195" t="str">
+        <v>تم تصدير تقرير بيان التطبيق بنجاح</v>
+      </c>
+      <c r="C1195" t="str">
+        <v>SOA atskaite veiksmīgi eksportēta</v>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="str">
+        <v>Audit logs exported successfully</v>
+      </c>
+      <c r="B1196" t="str">
+        <v>تم تصدير سجلات التدقيق بنجاح</v>
+      </c>
+      <c r="C1196" t="str">
+        <v>Audita žurnāli veiksmīgi eksportēti</v>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="str">
+        <v>No audit logs match your search.</v>
+      </c>
+      <c r="B1197" t="str">
+        <v>لا توجد سجلات تدقيق تطابق بحثك.</v>
+      </c>
+      <c r="C1197" t="str">
+        <v>Neviens audita ieraksts neatbilst jūsu meklējumam.</v>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="str">
+        <v>No requirements match your search.</v>
+      </c>
+      <c r="B1198" t="str">
+        <v>لا توجد متطلبات تطابق بحثك.</v>
+      </c>
+      <c r="C1198" t="str">
+        <v>Neviena prasība neatbilst jūsu meklējumam.</v>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="str">
+        <v>No requirements match your filters.</v>
+      </c>
+      <c r="B1199" t="str">
+        <v>لا توجد متطلبات تطابق عوامل التصفية.</v>
+      </c>
+      <c r="C1199" t="str">
+        <v>Neviena prasība neatbilst jūsu filtriem.</v>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="str">
+        <v>Requirement name should not be empty.</v>
+      </c>
+      <c r="B1200" t="str">
+        <v>يجب ألا يكون اسم المتطلب فارغاً.</v>
+      </c>
+      <c r="C1200" t="str">
+        <v>Prasības nosaukums nedrīkst būt tukšs.</v>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="str">
+        <v>Requirement category should not be empty.</v>
+      </c>
+      <c r="B1201" t="str">
+        <v>يجب ألا تكون فئة المتطلب فارغة.</v>
+      </c>
+      <c r="C1201" t="str">
+        <v>Prasības kategorija nedrīkst būt tukša.</v>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="str">
+        <v>Requirement code should not be empty.</v>
+      </c>
+      <c r="B1202" t="str">
+        <v>يجب ألا يكون رمز المتطلب فارغاً.</v>
+      </c>
+      <c r="C1202" t="str">
+        <v>Prasības kods nedrīkst būt tukšs.</v>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="str">
+        <v>Enter Name</v>
+      </c>
+      <c r="B1203" t="str">
+        <v>أدخل الاسم</v>
+      </c>
+      <c r="C1203" t="str">
+        <v>Ievadiet nosaukumu</v>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="str">
+        <v>Enter Category</v>
+      </c>
+      <c r="B1204" t="str">
+        <v>أدخل الفئة</v>
+      </c>
+      <c r="C1204" t="str">
+        <v>Ievadiet kategoriju</v>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="str">
+        <v>Enter Code</v>
+      </c>
+      <c r="B1205" t="str">
+        <v>أدخل الرمز</v>
+      </c>
+      <c r="C1205" t="str">
+        <v>Ievadiet kodu</v>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="str">
+        <v>Type here</v>
+      </c>
+      <c r="B1206" t="str">
+        <v>اكتب هنا</v>
+      </c>
+      <c r="C1206" t="str">
+        <v>Rakstiet šeit</v>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="str">
+        <v>To add a requirement to this framework, please accurately fill in the fields below.</v>
+      </c>
+      <c r="B1207" t="str">
+        <v>لإضافة متطلب إلى هذا الإطار، يرجى ملء الحقول أدناه بدقة.</v>
+      </c>
+      <c r="C1207" t="str">
+        <v>Lai pievienotu prasību šim ietvaram, lūdzu, precīzi aizpildiet zemāk esošos laukus.</v>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="str">
+        <v>Applicable</v>
+      </c>
+      <c r="B1208" t="str">
+        <v>قابل للتطبيق</v>
+      </c>
+      <c r="C1208" t="str">
+        <v>Piemērojams</v>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="str">
+        <v>Justification</v>
+      </c>
+      <c r="B1209" t="str">
+        <v>المبرر</v>
+      </c>
+      <c r="C1209" t="str">
+        <v>Pamatojums</v>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="str">
+        <v>Enter justification...</v>
+      </c>
+      <c r="B1210" t="str">
+        <v>أدخل المبرر...</v>
+      </c>
+      <c r="C1210" t="str">
+        <v>Ievadiet pamatojumu...</v>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="str">
+        <v>Impl. Status</v>
+      </c>
+      <c r="B1211" t="str">
+        <v>حالة التنفيذ</v>
+      </c>
+      <c r="C1211" t="str">
+        <v>Ievieš. statuss</v>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="str">
+        <v>No SOA data available to export</v>
+      </c>
+      <c r="B1212" t="str">
+        <v>لا توجد بيانات بيان التطبيق للتصدير</v>
+      </c>
+      <c r="C1212" t="str">
+        <v>Nav SOA datu eksportēšanai</v>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="str">
+        <v>No audit logs available to export</v>
+      </c>
+      <c r="B1213" t="str">
+        <v>لا توجد سجلات تدقيق للتصدير</v>
+      </c>
+      <c r="C1213" t="str">
+        <v>Nav audita žurnālu eksportēšanai</v>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="str">
+        <v>Framework Not Subscribed</v>
+      </c>
+      <c r="B1214" t="str">
+        <v>الإطار غير مشترك</v>
+      </c>
+      <c r="C1214" t="str">
+        <v>Ietvars nav abonēts</v>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="str">
+        <v>You do not have access to this framework. Please subscribe to view its contents.</v>
+      </c>
+      <c r="B1215" t="str">
+        <v>ليس لديك صلاحية الوصول إلى هذا الإطار. يرجى الاشتراك لعرض محتوياته.</v>
+      </c>
+      <c r="C1215" t="str">
+        <v>Jums nav piekļuves šim ietvaram. Lūdzu, abonējiet, lai skatītu tā saturu.</v>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="str">
+        <v>Loading framework...</v>
+      </c>
+      <c r="B1216" t="str">
+        <v>جاري تحميل الإطار...</v>
+      </c>
+      <c r="C1216" t="str">
+        <v>Ielādē ietvaru...</v>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="str">
+        <v>Framework not found</v>
+      </c>
+      <c r="B1217" t="str">
+        <v>لم يتم العثور على الإطار</v>
+      </c>
+      <c r="C1217" t="str">
+        <v>Ietvars nav atrasts</v>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="str">
+        <v>The requested framework could not be loaded.</v>
+      </c>
+      <c r="B1218" t="str">
+        <v>تعذر تحميل الإطار المطلوب.</v>
+      </c>
+      <c r="C1218" t="str">
+        <v>Pieprasīto ietvaru nevarēja ielādēt.</v>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="str">
+        <v>Framework Details</v>
+      </c>
+      <c r="B1219" t="str">
+        <v>تفاصيل الإطار</v>
+      </c>
+      <c r="C1219" t="str">
+        <v>Ietvara detaļas</v>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="str">
+        <v>Date &amp; Time</v>
+      </c>
+      <c r="B1220" t="str">
+        <v>التاريخ والوقت</v>
+      </c>
+      <c r="C1220" t="str">
+        <v>Datums un laiks</v>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="str">
+        <v>Target</v>
+      </c>
+      <c r="B1221" t="str">
+        <v>الهدف</v>
+      </c>
+      <c r="C1221" t="str">
+        <v>Mērķis</v>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="str">
+        <v>Details</v>
+      </c>
+      <c r="B1222" t="str">
+        <v>التفاصيل</v>
+      </c>
+      <c r="C1222" t="str">
+        <v>Detaļas</v>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="str">
+        <v>Unlink control</v>
+      </c>
+      <c r="B1223" t="str">
+        <v>إلغاء ربط الضابط</v>
+      </c>
+      <c r="C1223" t="str">
+        <v>Atsaistīt kontroli</v>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="str">
+        <v>Add Exception</v>
+      </c>
+      <c r="B1224" t="str">
+        <v>إضافة استثناء</v>
+      </c>
+      <c r="C1224" t="str">
+        <v>Pievienot izņēmumu</v>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="str">
+        <v>Please enter the reason for exception</v>
+      </c>
+      <c r="B1225" t="str">
+        <v>يرجى إدخال سبب الاستثناء</v>
+      </c>
+      <c r="C1225" t="str">
+        <v>Lūdzu, ievadiet izņēmuma iemeslu</v>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="str">
+        <v>Please select the enddate</v>
+      </c>
+      <c r="B1226" t="str">
+        <v>يرجى اختيار تاريخ النهاية</v>
+      </c>
+      <c r="C1226" t="str">
+        <v>Lūdzu, izvēlieties beigu datumu</v>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="str">
+        <v>Search by name or code...</v>
+      </c>
+      <c r="B1227" t="str">
+        <v>البحث بالاسم أو الرمز...</v>
+      </c>
+      <c r="C1227" t="str">
+        <v>Meklēt pēc nosaukuma vai koda...</v>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="str">
+        <v>No items match your search</v>
+      </c>
+      <c r="B1228" t="str">
+        <v>لا توجد عناصر تطابق بحثك</v>
+      </c>
+      <c r="C1228" t="str">
+        <v>Neviens elements neatbilst jūsu meklējumam</v>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="str">
+        <v>No items found for this framework</v>
+      </c>
+      <c r="B1229" t="str">
+        <v>لم يتم العثور على عناصر لهذا الإطار</v>
+      </c>
+      <c r="C1229" t="str">
+        <v>Šim ietvaram nav atrasts neviens elements</v>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="str">
+        <v>Try adjusting your search term</v>
+      </c>
+      <c r="B1230" t="str">
+        <v>حاول تعديل مصطلح البحث</v>
+      </c>
+      <c r="C1230" t="str">
+        <v>Mēģiniet mainīt meklēšanas terminu</v>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="str">
+        <v>Items will appear here once linked to this framework</v>
+      </c>
+      <c r="B1231" t="str">
+        <v>ستظهر العناصر هنا بمجرد ربطها بهذا الإطار</v>
+      </c>
+      <c r="C1231" t="str">
+        <v>Elementi parādīsies šeit, kad tie tiks saistīti ar šo ietvaru</v>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="str">
+        <v>No items</v>
+      </c>
+      <c r="B1232" t="str">
+        <v>لا توجد عناصر</v>
+      </c>
+      <c r="C1232" t="str">
+        <v>Nav elementu</v>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="str">
+        <v>Search by name, domain or assignee...</v>
+      </c>
+      <c r="B1233" t="str">
+        <v>البحث بالاسم أو المجال أو المسؤول...</v>
+      </c>
+      <c r="C1233" t="str">
+        <v>Meklēt pēc nosaukuma, domēna vai atbildīgā...</v>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="str">
+        <v>Evidence Code</v>
+      </c>
+      <c r="B1234" t="str">
+        <v>رمز الدليل</v>
+      </c>
+      <c r="C1234" t="str">
+        <v>Pierādījuma kods</v>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="str">
+        <v>No evidence matches your search</v>
+      </c>
+      <c r="B1235" t="str">
+        <v>لا توجد أدلة تطابق بحثك</v>
+      </c>
+      <c r="C1235" t="str">
+        <v>Neviens pierādījums neatbilst jūsu meklējumam</v>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="str">
+        <v>No evidence records found for this framework</v>
+      </c>
+      <c r="B1236" t="str">
+        <v>لم يتم العثور على سجلات أدلة لهذا الإطار</v>
+      </c>
+      <c r="C1236" t="str">
+        <v>Šim ietvaram nav atrasti pierādījumu ieraksti</v>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="str">
+        <v>Try adjusting your search</v>
+      </c>
+      <c r="B1237" t="str">
+        <v>حاول تعديل البحث</v>
+      </c>
+      <c r="C1237" t="str">
+        <v>Mēģiniet mainīt meklējumu</v>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="str">
+        <v>Link evidence to controls in the framework to see them here</v>
+      </c>
+      <c r="B1238" t="str">
+        <v>اربط الأدلة بالضوابط في الإطار لرؤيتها هنا</v>
+      </c>
+      <c r="C1238" t="str">
+        <v>Saistiet pierādījumus ar kontrolēm ietvaram, lai tos redzētu šeit</v>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="str">
+        <v>No evidence</v>
+      </c>
+      <c r="B1239" t="str">
+        <v>لا توجد أدلة</v>
+      </c>
+      <c r="C1239" t="str">
+        <v>Nav pierādījumu</v>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="str">
+        <v>Showing {start} to {end} of {total}</v>
+      </c>
+      <c r="B1240" t="str">
+        <v>عرض {start} إلى {end} من {total}</v>
+      </c>
+      <c r="C1240" t="str">
+        <v>Rāda {start} līdz {end} no {total}</v>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="str">
+        <v>Create Integrated Framework</v>
+      </c>
+      <c r="B1241" t="str">
+        <v>إنشاء إطار متكامل</v>
+      </c>
+      <c r="C1241" t="str">
+        <v>Izveidot integrētu ietvaru</v>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="str">
+        <v>Create Integrated Framework (AI)</v>
+      </c>
+      <c r="B1242" t="str">
+        <v>إنشاء إطار متكامل (ذكاء اصطناعي)</v>
+      </c>
+      <c r="C1242" t="str">
+        <v>Izveidot integrētu ietvaru (AI)</v>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="str">
+        <v>Custom framework will be automatically added in grey color to differentiate between Subscribed Frameworks.</v>
+      </c>
+      <c r="B1243" t="str">
+        <v>سيتم إضافة الإطار المخصص تلقائياً باللون الرمادي للتمييز بين الأطر المشترك بها.</v>
+      </c>
+      <c r="C1243" t="str">
+        <v>Pielāgotais ietvars tiks automātiski pievienots pelēkā krāsā, lai atšķirtu no abonētajiem ietvariem.</v>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="str">
+        <v>Integrated Framework Name</v>
+      </c>
+      <c r="B1244" t="str">
+        <v>اسم الإطار المتكامل</v>
+      </c>
+      <c r="C1244" t="str">
+        <v>Integrētā ietvara nosaukums</v>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="str">
+        <v>Framework Type</v>
+      </c>
+      <c r="B1245" t="str">
+        <v>نوع الإطار</v>
+      </c>
+      <c r="C1245" t="str">
+        <v>Ietvara veids</v>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="str">
+        <v>Enter framework name</v>
+      </c>
+      <c r="B1246" t="str">
+        <v>أدخل اسم الإطار</v>
+      </c>
+      <c r="C1246" t="str">
+        <v>Ievadiet ietvara nosaukumu</v>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="str">
+        <v>Enter code</v>
+      </c>
+      <c r="B1247" t="str">
+        <v>أدخل الرمز</v>
+      </c>
+      <c r="C1247" t="str">
+        <v>Ievadiet kodu</v>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="str">
+        <v>Enter country</v>
+      </c>
+      <c r="B1248" t="str">
+        <v>أدخل الدولة</v>
+      </c>
+      <c r="C1248" t="str">
+        <v>Ievadiet valsti</v>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="str">
+        <v>Enter industry</v>
+      </c>
+      <c r="B1249" t="str">
+        <v>أدخل الصناعة</v>
+      </c>
+      <c r="C1249" t="str">
+        <v>Ievadiet nozari</v>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="str">
+        <v>Create &amp; Import</v>
+      </c>
+      <c r="B1250" t="str">
+        <v>إنشاء واستيراد</v>
+      </c>
+      <c r="C1250" t="str">
+        <v>Izveidot un importēt</v>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="str">
+        <v>Upload Support Document</v>
+      </c>
+      <c r="B1251" t="str">
+        <v>رفع مستند داعم</v>
+      </c>
+      <c r="C1251" t="str">
+        <v>Augšupielādēt atbalsta dokumentu</v>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="str">
+        <v>Click here, or drop files here to upload.</v>
+      </c>
+      <c r="B1252" t="str">
+        <v>انقر هنا، أو اسحب الملفات هنا للرفع.</v>
+      </c>
+      <c r="C1252" t="str">
+        <v>Noklikšķiniet šeit vai velciet failus šeit, lai augšupielādētu.</v>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="str">
+        <v>Import Framework Requirements</v>
+      </c>
+      <c r="B1253" t="str">
+        <v>استيراد متطلبات الإطار</v>
+      </c>
+      <c r="C1253" t="str">
+        <v>Importēt ietvara prasības</v>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="str">
+        <v>Upload an Excel file (.xlsx) containing your framework requirements.</v>
+      </c>
+      <c r="B1254" t="str">
+        <v>ارفع ملف إكسل (.xlsx) يحتوي على متطلبات الإطار.</v>
+      </c>
+      <c r="C1254" t="str">
+        <v>Augšupielādējiet Excel failu (.xlsx) ar ietvara prasībām.</v>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="str">
+        <v>You can download the sample template to see the required format.</v>
+      </c>
+      <c r="B1255" t="str">
+        <v>يمكنك تحميل القالب النموذجي لمعرفة التنسيق المطلوب.</v>
+      </c>
+      <c r="C1255" t="str">
+        <v>Varat lejupielādēt parauga veidni, lai redzētu nepieciešamo formātu.</v>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="str">
+        <v>Download Sample Template</v>
+      </c>
+      <c r="B1256" t="str">
+        <v>تحميل القالب النموذجي</v>
+      </c>
+      <c r="C1256" t="str">
+        <v>Lejupielādēt parauga veidni</v>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="str">
+        <v>Use this template to ensure correct column headers</v>
+      </c>
+      <c r="B1257" t="str">
+        <v>استخدم هذا القالب لضمان عناوين الأعمدة الصحيحة</v>
+      </c>
+      <c r="C1257" t="str">
+        <v>Izmantojiet šo veidni, lai nodrošinātu pareizus kolonnu virsrakstus</v>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="str">
+        <v>Upload Document</v>
+      </c>
+      <c r="B1258" t="str">
+        <v>رفع مستند</v>
+      </c>
+      <c r="C1258" t="str">
+        <v>Augšupielādēt dokumentu</v>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="str">
+        <v>Click to upload or drag and drop</v>
+      </c>
+      <c r="B1259" t="str">
+        <v>انقر للرفع أو اسحب وأفلت</v>
+      </c>
+      <c r="C1259" t="str">
+        <v>Noklikšķiniet, lai augšupielādētu, vai velciet un nometiet</v>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="str">
+        <v>Excel files only (.xlsx)</v>
+      </c>
+      <c r="B1260" t="str">
+        <v>ملفات إكسل فقط (.xlsx)</v>
+      </c>
+      <c r="C1260" t="str">
+        <v>Tikai Excel faili (.xlsx)</v>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="str">
+        <v>Required Column Headers:</v>
+      </c>
+      <c r="B1261" t="str">
+        <v>عناوين الأعمدة المطلوبة:</v>
+      </c>
+      <c r="C1261" t="str">
+        <v>Nepieciešamie kolonnu virsraksti:</v>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="str">
+        <v>Control Mapping</v>
+      </c>
+      <c r="B1262" t="str">
+        <v>ربط الضوابط</v>
+      </c>
+      <c r="C1262" t="str">
+        <v>Kontroles kartēšana</v>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="str">
+        <v>Skip</v>
+      </c>
+      <c r="B1263" t="str">
+        <v>تخطي</v>
+      </c>
+      <c r="C1263" t="str">
+        <v>Izlaist</v>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="str">
+        <v>Import Successful</v>
+      </c>
+      <c r="B1264" t="str">
+        <v>تم الاستيراد بنجاح</v>
+      </c>
+      <c r="C1264" t="str">
+        <v>Imports veiksmīgs</v>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="str">
+        <v>Import Failed</v>
+      </c>
+      <c r="B1265" t="str">
+        <v>فشل الاستيراد</v>
+      </c>
+      <c r="C1265" t="str">
+        <v>Imports neizdevās</v>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="str">
+        <v>Failed to import requirements</v>
+      </c>
+      <c r="B1266" t="str">
+        <v>فشل استيراد المتطلبات</v>
+      </c>
+      <c r="C1266" t="str">
+        <v>Neizdevās importēt prasības</v>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="str">
+        <v>Template Downloaded</v>
+      </c>
+      <c r="B1267" t="str">
+        <v>تم تحميل القالب</v>
+      </c>
+      <c r="C1267" t="str">
+        <v>Veidne lejupielādēta</v>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="str">
+        <v>Sample template has been downloaded successfully</v>
+      </c>
+      <c r="B1268" t="str">
+        <v>تم تحميل القالب النموذجي بنجاح</v>
+      </c>
+      <c r="C1268" t="str">
+        <v>Parauga veidne veiksmīgi lejupielādēta</v>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="str">
+        <v>Failed to download template</v>
+      </c>
+      <c r="B1269" t="str">
+        <v>فشل تحميل القالب</v>
+      </c>
+      <c r="C1269" t="str">
+        <v>Neizdevās lejupielādēt veidni</v>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="str">
+        <v>Invalid File</v>
+      </c>
+      <c r="B1270" t="str">
+        <v>ملف غير صالح</v>
+      </c>
+      <c r="C1270" t="str">
+        <v>Nederīgs fails</v>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="str">
+        <v>Please upload an Excel file (.xlsx)</v>
+      </c>
+      <c r="B1271" t="str">
+        <v>يرجى رفع ملف إكسل (.xlsx)</v>
+      </c>
+      <c r="C1271" t="str">
+        <v>Lūdzu, augšupielādējiet Excel failu (.xlsx)</v>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="str">
+        <v>Please enter Country</v>
+      </c>
+      <c r="B1272" t="str">
+        <v>يرجى إدخال الدولة</v>
+      </c>
+      <c r="C1272" t="str">
+        <v>Lūdzu, ievadiet valsti</v>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="str">
+        <v>Please enter Industry</v>
+      </c>
+      <c r="B1273" t="str">
+        <v>يرجى إدخال الصناعة</v>
+      </c>
+      <c r="C1273" t="str">
+        <v>Lūdzu, ievadiet nozari</v>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="str">
+        <v>Generating... (AI)</v>
+      </c>
+      <c r="B1274" t="str">
+        <v>جاري الإنشاء... (ذكاء اصطناعي)</v>
+      </c>
+      <c r="C1274" t="str">
+        <v>Ģenerē... (AI)</v>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="str">
+        <v>AI framework generation failed</v>
+      </c>
+      <c r="B1275" t="str">
+        <v>فشل إنشاء الإطار بالذكاء الاصطناعي</v>
+      </c>
+      <c r="C1275" t="str">
+        <v>AI ietvara ģenerēšana neizdevās</v>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="str">
+        <v>Polling failed</v>
+      </c>
+      <c r="B1276" t="str">
+        <v>فشل الاستعلام</v>
+      </c>
+      <c r="C1276" t="str">
+        <v>Aptauja neizdevās</v>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="str">
+        <v>Framework created successfully</v>
+      </c>
+      <c r="B1277" t="str">
+        <v>تم إنشاء الإطار بنجاح</v>
+      </c>
+      <c r="C1277" t="str">
+        <v>Ietvars veiksmīgi izveidots</v>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="str">
+        <v>Some warnings occurred during import. See details below.</v>
+      </c>
+      <c r="B1278" t="str">
+        <v>حدثت بعض التحذيرات أثناء الاستيراد. انظر التفاصيل أدناه.</v>
+      </c>
+      <c r="C1278" t="str">
+        <v>Importēšanas laikā radās daži brīdinājumi. Skatiet detaļas zemāk.</v>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="str">
+        <v>Warnings</v>
+      </c>
+      <c r="B1279" t="str">
+        <v>تحذيرات</v>
+      </c>
+      <c r="C1279" t="str">
+        <v>Brīdinājumi</v>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="str">
+        <v>Validation Errors</v>
+      </c>
+      <c r="B1280" t="str">
+        <v>أخطاء التحقق</v>
+      </c>
+      <c r="C1280" t="str">
+        <v>Validācijas kļūdas</v>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="str">
+        <v>Row</v>
+      </c>
+      <c r="B1281" t="str">
+        <v>صف</v>
+      </c>
+      <c r="C1281" t="str">
+        <v>Rinda</v>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="str">
+        <v>Country</v>
+      </c>
+      <c r="B1282" t="str">
+        <v>الدولة</v>
+      </c>
+      <c r="C1282" t="str">
+        <v>Valsts</v>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="str">
+        <v>Industry</v>
+      </c>
+      <c r="B1283" t="str">
+        <v>الصناعة</v>
+      </c>
+      <c r="C1283" t="str">
+        <v>Nozare</v>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="str">
+        <v>Total Controls</v>
+      </c>
+      <c r="B1284" t="str">
+        <v>إجمالي الضوابط</v>
+      </c>
+      <c r="C1284" t="str">
+        <v>Kopējās kontroles</v>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="str">
+        <v>Controls by Framework</v>
+      </c>
+      <c r="B1285" t="str">
+        <v>الضوابط حسب الإطار</v>
+      </c>
+      <c r="C1285" t="str">
+        <v>Kontroles pēc ietvara</v>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="str">
+        <v>Control Question</v>
+      </c>
+      <c r="B1286" t="str">
+        <v>سؤال الضابطة</v>
+      </c>
+      <c r="C1286" t="str">
+        <v>Kontroles jautājums</v>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="str">
+        <v>Control Information</v>
+      </c>
+      <c r="B1287" t="str">
+        <v>معلومات الضابطة</v>
+      </c>
+      <c r="C1287" t="str">
+        <v>Kontroles informācija</v>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="str">
+        <v>Domain Code</v>
+      </c>
+      <c r="B1288" t="str">
+        <v>رمز المجال</v>
+      </c>
+      <c r="C1288" t="str">
+        <v>Domēna kods</v>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="str">
+        <v>Create New Domain</v>
+      </c>
+      <c r="B1289" t="str">
+        <v>إنشاء مجال جديد</v>
+      </c>
+      <c r="C1289" t="str">
+        <v>Izveidot jaunu domēnu</v>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="str">
+        <v>Enter control name</v>
+      </c>
+      <c r="B1290" t="str">
+        <v>أدخل اسم الضابطة</v>
+      </c>
+      <c r="C1290" t="str">
+        <v>Ievadiet kontroles nosaukumu</v>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="str">
+        <v>Enter control question</v>
+      </c>
+      <c r="B1291" t="str">
+        <v>أدخل سؤال الضابطة</v>
+      </c>
+      <c r="C1291" t="str">
+        <v>Ievadiet kontroles jautājumu</v>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="str">
+        <v>Select grouping</v>
+      </c>
+      <c r="B1292" t="str">
+        <v>اختر التجميع</v>
+      </c>
+      <c r="C1292" t="str">
+        <v>Izvēlieties grupēšanu</v>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="str">
+        <v>Select assignee</v>
+      </c>
+      <c r="B1293" t="str">
+        <v>اختر المسؤول</v>
+      </c>
+      <c r="C1293" t="str">
+        <v>Izvēlieties atbildīgo</v>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="str">
+        <v>Assignment</v>
+      </c>
+      <c r="B1294" t="str">
+        <v>التعيين</v>
+      </c>
+      <c r="C1294" t="str">
+        <v>Piešķiršana</v>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="str">
+        <v>Review</v>
+      </c>
+      <c r="B1295" t="str">
+        <v>المراجعة</v>
+      </c>
+      <c r="C1295" t="str">
+        <v>Pārskatīšana</v>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="str">
+        <v>Assignment Details</v>
+      </c>
+      <c r="B1296" t="str">
+        <v>تفاصيل التعيين</v>
+      </c>
+      <c r="C1296" t="str">
+        <v>Piešķiršanas detaļas</v>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="str">
+        <v>Review Information</v>
+      </c>
+      <c r="B1297" t="str">
+        <v>مراجعة المعلومات</v>
+      </c>
+      <c r="C1297" t="str">
+        <v>Pārskatīt informāciju</v>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="str">
+        <v>e.g., GOV</v>
+      </c>
+      <c r="B1298" t="str">
+        <v>مثال: GOV</v>
+      </c>
+      <c r="C1298" t="str">
+        <v>piem., GOV</v>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="str">
+        <v>e.g., Governance</v>
+      </c>
+      <c r="B1299" t="str">
+        <v>مثال: الحوكمة</v>
+      </c>
+      <c r="C1299" t="str">
+        <v>piem., Pārvaldība</v>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="str">
+        <v>Please enter the question</v>
+      </c>
+      <c r="B1300" t="str">
+        <v>يرجى إدخال السؤال</v>
+      </c>
+      <c r="C1300" t="str">
+        <v>Lūdzu, ievadiet jautājumu</v>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="str">
+        <v>Please select the Functional Grouping</v>
+      </c>
+      <c r="B1301" t="str">
+        <v>يرجى اختيار التجميع الوظيفي</v>
+      </c>
+      <c r="C1301" t="str">
+        <v>Lūdzu, izvēlieties funkcionālo grupēšanu</v>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="str">
+        <v>No department reviewers found</v>
+      </c>
+      <c r="B1302" t="str">
+        <v>لم يتم العثور على مراجعين للقسم</v>
+      </c>
+      <c r="C1302" t="str">
+        <v>Nav atrasti nodaļas pārskatītāji</v>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="str">
+        <v>Information Security Vault</v>
+      </c>
+      <c r="B1303" t="str">
+        <v>خزنة أمن المعلومات</v>
+      </c>
+      <c r="C1303" t="str">
+        <v>Informācijas drošības glabātuve</v>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="str">
+        <v>Import Controls</v>
+      </c>
+      <c r="B1304" t="str">
+        <v>استيراد الضوابط</v>
+      </c>
+      <c r="C1304" t="str">
+        <v>Importēt kontroles</v>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="str">
+        <v>Upload a CSV file to import controls. You can download a template to see the required format.</v>
+      </c>
+      <c r="B1305" t="str">
+        <v>ارفع ملف CSV لاستيراد الضوابط. يمكنك تنزيل قالب لمعرفة التنسيق المطلوب.</v>
+      </c>
+      <c r="C1305" t="str">
+        <v>Augšupielādējiet CSV failu, lai importētu kontroles. Varat lejupielādēt veidni, lai redzētu nepieciešamo formātu.</v>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="str">
+        <v>Search by code, name, department...</v>
+      </c>
+      <c r="B1306" t="str">
+        <v>البحث بالرمز، الاسم، القسم...</v>
+      </c>
+      <c r="C1306" t="str">
+        <v>Meklēt pēc koda, nosaukuma, nodaļas...</v>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="str">
+        <v>Link Governance Documents</v>
+      </c>
+      <c r="B1307" t="str">
+        <v>ربط مستندات الحوكمة</v>
+      </c>
+      <c r="C1307" t="str">
+        <v>Saistīt pārvaldības dokumentus</v>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="str">
+        <v>Link Governance</v>
+      </c>
+      <c r="B1308" t="str">
+        <v>ربط الحوكمة</v>
+      </c>
+      <c r="C1308" t="str">
+        <v>Saistīt pārvaldību</v>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="str">
+        <v>Link Selected</v>
+      </c>
+      <c r="B1309" t="str">
+        <v>ربط المحدد</v>
+      </c>
+      <c r="C1309" t="str">
+        <v>Saistīt izvēlētos</v>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="str">
+        <v>Search by code or name...</v>
+      </c>
+      <c r="B1310" t="str">
+        <v>البحث بالرمز أو الاسم...</v>
+      </c>
+      <c r="C1310" t="str">
+        <v>Meklēt pēc koda vai nosaukuma...</v>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="str">
+        <v>selected</v>
+      </c>
+      <c r="B1311" t="str">
+        <v>محدد</v>
+      </c>
+      <c r="C1311" t="str">
+        <v>izvēlēts</v>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="str">
+        <v>No Documents</v>
+      </c>
+      <c r="B1312" t="str">
+        <v>لا توجد مستندات</v>
+      </c>
+      <c r="C1312" t="str">
+        <v>Nav dokumentu</v>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="str">
+        <v>Upload your first document to get started.</v>
+      </c>
+      <c r="B1313" t="str">
+        <v>ارفع أول مستند للبدء.</v>
+      </c>
+      <c r="C1313" t="str">
+        <v>Augšupielādējiet pirmo dokumentu, lai sāktu.</v>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="str">
+        <v>Drag and drop files here</v>
+      </c>
+      <c r="B1314" t="str">
+        <v>اسحب وأفلت الملفات هنا</v>
+      </c>
+      <c r="C1314" t="str">
+        <v>Velciet un nometiet failus šeit</v>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="str">
+        <v>or click to browse from your computer</v>
+      </c>
+      <c r="B1315" t="str">
+        <v>أو انقر للتصفح من جهازك</v>
+      </c>
+      <c r="C1315" t="str">
+        <v>vai noklikšķiniet, lai pārlūkotu no datora</v>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="str">
+        <v>Document ID</v>
+      </c>
+      <c r="B1316" t="str">
+        <v>معرّف المستند</v>
+      </c>
+      <c r="C1316" t="str">
+        <v>Dokumenta ID</v>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="str">
+        <v>Document Name</v>
+      </c>
+      <c r="B1317" t="str">
+        <v>اسم المستند</v>
+      </c>
+      <c r="C1317" t="str">
+        <v>Dokumenta nosaukums</v>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="str">
+        <v>Uploaded</v>
+      </c>
+      <c r="B1318" t="str">
+        <v>تاريخ الرفع</v>
+      </c>
+      <c r="C1318" t="str">
+        <v>Augšupielādēts</v>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="str">
+        <v>Edit Control</v>
+      </c>
+      <c r="B1319" t="str">
+        <v>تعديل الضابطة</v>
+      </c>
+      <c r="C1319" t="str">
+        <v>Rediģēt kontroli</v>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="str">
+        <v>Assigned To</v>
+      </c>
+      <c r="B1320" t="str">
+        <v>مُسند إلى</v>
+      </c>
+      <c r="C1320" t="str">
+        <v>Piešķirts</v>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="str">
+        <v>No risks linked</v>
+      </c>
+      <c r="B1321" t="str">
+        <v>لا توجد مخاطر مرتبطة</v>
+      </c>
+      <c r="C1321" t="str">
+        <v>Nav saistītu risku</v>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="str">
+        <v>No linked risks</v>
+      </c>
+      <c r="B1322" t="str">
+        <v>لا توجد مخاطر مرتبطة</v>
+      </c>
+      <c r="C1322" t="str">
+        <v>Nav saistītu risku</v>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="str">
+        <v>No linked exceptions</v>
+      </c>
+      <c r="B1323" t="str">
+        <v>لا توجد استثناءات مرتبطة</v>
+      </c>
+      <c r="C1323" t="str">
+        <v>Nav saistītu izņēmumu</v>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="str">
+        <v>No linked evidences</v>
+      </c>
+      <c r="B1324" t="str">
+        <v>لا توجد أدلة مرتبطة</v>
+      </c>
+      <c r="C1324" t="str">
+        <v>Nav saistītu pierādījumu</v>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="str">
+        <v>No linked requirements</v>
+      </c>
+      <c r="B1325" t="str">
+        <v>لا توجد متطلبات مرتبطة</v>
+      </c>
+      <c r="C1325" t="str">
+        <v>Nav saistītu prasību</v>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="str">
+        <v>No linked policies</v>
+      </c>
+      <c r="B1326" t="str">
+        <v>لا توجد سياسات مرتبطة</v>
+      </c>
+      <c r="C1326" t="str">
+        <v>Nav saistītu politiku</v>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="str">
+        <v>Select Risks</v>
+      </c>
+      <c r="B1327" t="str">
+        <v>اختر المخاطر</v>
+      </c>
+      <c r="C1327" t="str">
+        <v>Izvēlieties riskus</v>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="str">
+        <v>Select Requirements</v>
+      </c>
+      <c r="B1328" t="str">
+        <v>اختر المتطلبات</v>
+      </c>
+      <c r="C1328" t="str">
+        <v>Izvēlieties prasības</v>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="str">
+        <v>Select Policies</v>
+      </c>
+      <c r="B1329" t="str">
+        <v>اختر السياسات</v>
+      </c>
+      <c r="C1329" t="str">
+        <v>Izvēlieties politikas</v>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="str">
+        <v>Select Evidence</v>
+      </c>
+      <c r="B1330" t="str">
+        <v>اختر الأدلة</v>
+      </c>
+      <c r="C1330" t="str">
+        <v>Izvēlieties pierādījumus</v>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="str">
+        <v>Select Exceptions</v>
+      </c>
+      <c r="B1331" t="str">
+        <v>اختر الاستثناءات</v>
+      </c>
+      <c r="C1331" t="str">
+        <v>Izvēlieties izņēmumus</v>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="str">
+        <v>Linked Requirement</v>
+      </c>
+      <c r="B1332" t="str">
+        <v>المتطلبات المرتبطة</v>
+      </c>
+      <c r="C1332" t="str">
+        <v>Saistītā prasība</v>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="str">
+        <v>Linked Requirements</v>
+      </c>
+      <c r="B1333" t="str">
+        <v>المتطلبات المرتبطة</v>
+      </c>
+      <c r="C1333" t="str">
+        <v>Saistītās prasības</v>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="str">
+        <v>Add Selected</v>
+      </c>
+      <c r="B1334" t="str">
+        <v>إضافة المحدد</v>
+      </c>
+      <c r="C1334" t="str">
+        <v>Pievienot izvēlētos</v>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="str">
+        <v>Add Approver</v>
+      </c>
+      <c r="B1335" t="str">
+        <v>إضافة معتمد</v>
+      </c>
+      <c r="C1335" t="str">
+        <v>Pievienot apstiprinātāju</v>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="str">
+        <v>Select Approver</v>
+      </c>
+      <c r="B1336" t="str">
+        <v>اختر المعتمد</v>
+      </c>
+      <c r="C1336" t="str">
+        <v>Izvēlieties apstiprinātāju</v>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="str">
+        <v>Only Department Reviewers from the assigned department are shown.</v>
+      </c>
+      <c r="B1337" t="str">
+        <v>يتم عرض مراجعي القسم من القسم المعيّن فقط.</v>
+      </c>
+      <c r="C1337" t="str">
+        <v>Tiek rādīti tikai nodaļas pārskatītāji no piešķirtās nodaļas.</v>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="str">
+        <v>Select approver</v>
+      </c>
+      <c r="B1338" t="str">
+        <v>اختر المعتمد</v>
+      </c>
+      <c r="C1338" t="str">
+        <v>Izvēlieties apstiprinātāju</v>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="str">
+        <v>Linked Frameworks</v>
+      </c>
+      <c r="B1339" t="str">
+        <v>الأطر المرتبطة</v>
+      </c>
+      <c r="C1339" t="str">
+        <v>Saistītie ietvari</v>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="str">
+        <v>Policy Details</v>
+      </c>
+      <c r="B1340" t="str">
+        <v>تفاصيل السياسة</v>
+      </c>
+      <c r="C1340" t="str">
+        <v>Politikas detaļas</v>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="str">
+        <v>AI Review</v>
+      </c>
+      <c r="B1341" t="str">
+        <v>مراجعة الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1341" t="str">
+        <v>AI pārskatīšana</v>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="str">
+        <v>AI Review has not been performed yet</v>
+      </c>
+      <c r="B1342" t="str">
+        <v>لم تتم مراجعة الذكاء الاصطناعي بعد</v>
+      </c>
+      <c r="C1342" t="str">
+        <v>AI pārskatīšana vēl nav veikta</v>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="str">
+        <v>Start an AI review to analyze this document</v>
+      </c>
+      <c r="B1343" t="str">
+        <v>ابدأ مراجعة بالذكاء الاصطناعي لتحليل هذا المستند</v>
+      </c>
+      <c r="C1343" t="str">
+        <v>Sāciet AI pārskatīšanu, lai analizētu šo dokumentu</v>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="str">
+        <v>Attachments</v>
+      </c>
+      <c r="B1344" t="str">
+        <v>المرفقات</v>
+      </c>
+      <c r="C1344" t="str">
+        <v>Pielikumi</v>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="str">
+        <v>Link from Vault</v>
+      </c>
+      <c r="B1345" t="str">
+        <v>ربط من الخزنة</v>
+      </c>
+      <c r="C1345" t="str">
+        <v>Saistīt no glabātuves</v>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="str">
+        <v>Link existing vault documents</v>
+      </c>
+      <c r="B1346" t="str">
+        <v>ربط مستندات الخزنة الحالية</v>
+      </c>
+      <c r="C1346" t="str">
+        <v>Saistīt esošos glabātuves dokumentus</v>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="str">
+        <v>Generate Policy Using AI</v>
+      </c>
+      <c r="B1347" t="str">
+        <v>إنشاء سياسة باستخدام الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1347" t="str">
+        <v>Ģenerēt politiku ar AI</v>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="str">
+        <v>Create document with AI assistance</v>
+      </c>
+      <c r="B1348" t="str">
+        <v>إنشاء مستند بمساعدة الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1348" t="str">
+        <v>Izveidot dokumentu ar AI palīdzību</v>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="str">
+        <v>Upload Existing File</v>
+      </c>
+      <c r="B1349" t="str">
+        <v>رفع ملف موجود</v>
+      </c>
+      <c r="C1349" t="str">
+        <v>Augšupielādēt esošu failu</v>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="str">
+        <v>Upload document from your device</v>
+      </c>
+      <c r="B1350" t="str">
+        <v>رفع مستند من جهازك</v>
+      </c>
+      <c r="C1350" t="str">
+        <v>Augšupielādēt dokumentu no ierīces</v>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="str">
+        <v>Linked Documents</v>
+      </c>
+      <c r="B1351" t="str">
+        <v>المستندات المرتبطة</v>
+      </c>
+      <c r="C1351" t="str">
+        <v>Saistītie dokumenti</v>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="str">
+        <v>Linked Exception</v>
+      </c>
+      <c r="B1352" t="str">
+        <v>الاستثناء المرتبط</v>
+      </c>
+      <c r="C1352" t="str">
+        <v>Saistītais izņēmums</v>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="str">
+        <v>Linked Control</v>
+      </c>
+      <c r="B1353" t="str">
+        <v>الضابطة المرتبطة</v>
+      </c>
+      <c r="C1353" t="str">
+        <v>Saistītā kontrole</v>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="str">
+        <v>Link Control</v>
+      </c>
+      <c r="B1354" t="str">
+        <v>ربط ضابطة</v>
+      </c>
+      <c r="C1354" t="str">
+        <v>Saistīt kontroli</v>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="str">
+        <v>Control ID</v>
+      </c>
+      <c r="B1355" t="str">
+        <v>معرّف الضابطة</v>
+      </c>
+      <c r="C1355" t="str">
+        <v>Kontroles ID</v>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="str">
+        <v>No exceptions linked to this</v>
+      </c>
+      <c r="B1356" t="str">
+        <v>لا توجد استثناءات مرتبطة بهذا</v>
+      </c>
+      <c r="C1356" t="str">
+        <v>Nav izņēmumu saistītu ar šo</v>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="str">
+        <v>Link exceptions to track deviations</v>
+      </c>
+      <c r="B1357" t="str">
+        <v>ربط الاستثناءات لتتبع الانحرافات</v>
+      </c>
+      <c r="C1357" t="str">
+        <v>Saistīt izņēmumus, lai izsekotu novirzes</v>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="str">
+        <v>Link Exception</v>
+      </c>
+      <c r="B1358" t="str">
+        <v>ربط استثناء</v>
+      </c>
+      <c r="C1358" t="str">
+        <v>Saistīt izņēmumu</v>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="str">
+        <v>No documents linked to this</v>
+      </c>
+      <c r="B1359" t="str">
+        <v>لا توجد مستندات مرتبطة بهذا</v>
+      </c>
+      <c r="C1359" t="str">
+        <v>Nav dokumentu saistītu ar šo</v>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="str">
+        <v>Documents linked to this policy will appear here</v>
+      </c>
+      <c r="B1360" t="str">
+        <v>ستظهر المستندات المرتبطة بهذه السياسة هنا</v>
+      </c>
+      <c r="C1360" t="str">
+        <v>Ar šo politiku saistītie dokumenti parādīsies šeit</v>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="str">
+        <v>Start AI Review</v>
+      </c>
+      <c r="B1361" t="str">
+        <v>بدء مراجعة الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1361" t="str">
+        <v>Sākt AI pārskatīšanu</v>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="str">
+        <v>Publish</v>
+      </c>
+      <c r="B1362" t="str">
+        <v>نشر</v>
+      </c>
+      <c r="C1362" t="str">
+        <v>Publicēt</v>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="str">
+        <v>Select recurrence</v>
+      </c>
+      <c r="B1363" t="str">
+        <v>اختر التكرار</v>
+      </c>
+      <c r="C1363" t="str">
+        <v>Izvēlieties atkārtošanos</v>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="str">
+        <v>Review Date</v>
+      </c>
+      <c r="B1364" t="str">
+        <v>تاريخ المراجعة</v>
+      </c>
+      <c r="C1364" t="str">
+        <v>Pārskatīšanas datums</v>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="str">
+        <v>Recurrence</v>
+      </c>
+      <c r="B1365" t="str">
+        <v>التكرار</v>
+      </c>
+      <c r="C1365" t="str">
+        <v>Atkārtošanās</v>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="str">
+        <v>Edit Assignee</v>
+      </c>
+      <c r="B1366" t="str">
+        <v>تعديل المكلّف</v>
+      </c>
+      <c r="C1366" t="str">
+        <v>Rediģēt pilnvaroto</v>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="str">
+        <v>Select Assignee</v>
+      </c>
+      <c r="B1367" t="str">
+        <v>اختر المكلّف</v>
+      </c>
+      <c r="C1367" t="str">
+        <v>Izvēlieties pilnvaroto</v>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="str">
+        <v>Only Department Contributors and Department Reviewers from the assigned department are shown.</v>
+      </c>
+      <c r="B1368" t="str">
+        <v>يتم عرض مساهمي ومراجعي القسم من القسم المعيّن فقط.</v>
+      </c>
+      <c r="C1368" t="str">
+        <v>Tiek rādīti tikai nodaļas līdzstrādnieki un pārskatītāji no piešķirtās nodaļas.</v>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="str">
+        <v>Approvers</v>
+      </c>
+      <c r="B1369" t="str">
+        <v>المعتمدون</v>
+      </c>
+      <c r="C1369" t="str">
+        <v>Apstiprinātāji</v>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="str">
+        <v>Evidence Request List</v>
+      </c>
+      <c r="B1370" t="str">
+        <v>قائمة طلبات الأدلة</v>
+      </c>
+      <c r="C1370" t="str">
+        <v>Pierādījumu pieprasījumu saraksts</v>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="str">
+        <v>Artifacts</v>
+      </c>
+      <c r="B1371" t="str">
+        <v>المستندات المرفقة</v>
+      </c>
+      <c r="C1371" t="str">
+        <v>Artefakti</v>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="str">
+        <v>New Evidence</v>
+      </c>
+      <c r="B1372" t="str">
+        <v>دليل جديد</v>
+      </c>
+      <c r="C1372" t="str">
+        <v>Jauns pierādījums</v>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="str">
+        <v>Evidence Name</v>
+      </c>
+      <c r="B1373" t="str">
+        <v>اسم الدليل</v>
+      </c>
+      <c r="C1373" t="str">
+        <v>Pierādījuma nosaukums</v>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="str">
+        <v>Issue Identified By</v>
+      </c>
+      <c r="B1374" t="str">
+        <v>تم تحديد المشكلة بواسطة</v>
+      </c>
+      <c r="C1374" t="str">
+        <v>Problēmu identificēja</v>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="str">
+        <v>Submitted</v>
+      </c>
+      <c r="B1375" t="str">
+        <v>تم التقديم</v>
+      </c>
+      <c r="C1375" t="str">
+        <v>Iesniegts</v>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="str">
+        <v>Evidence Requirement</v>
+      </c>
+      <c r="B1376" t="str">
+        <v>متطلبات الدليل</v>
+      </c>
+      <c r="C1376" t="str">
+        <v>Pierādījuma prasība</v>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="str">
+        <v>Enter evidence requirement</v>
+      </c>
+      <c r="B1377" t="str">
+        <v>أدخل متطلبات الدليل</v>
+      </c>
+      <c r="C1377" t="str">
+        <v>Ievadiet pierādījuma prasību</v>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="str">
+        <v>Select Controls to Link</v>
+      </c>
+      <c r="B1378" t="str">
+        <v>اختر الضوابط للربط</v>
+      </c>
+      <c r="C1378" t="str">
+        <v>Izvēlieties kontroles saistīšanai</v>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="str">
+        <v>Search controls...</v>
+      </c>
+      <c r="B1379" t="str">
+        <v>البحث في الضوابط...</v>
+      </c>
+      <c r="C1379" t="str">
+        <v>Meklēt kontroles...</v>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="str">
+        <v>All Groupings</v>
+      </c>
+      <c r="B1380" t="str">
+        <v>جميع التصنيفات</v>
+      </c>
+      <c r="C1380" t="str">
+        <v>Visas grupas</v>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="str">
+        <v>controls</v>
+      </c>
+      <c r="B1381" t="str">
+        <v>ضوابط</v>
+      </c>
+      <c r="C1381" t="str">
+        <v>kontroles</v>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="str">
+        <v>Selected Controls</v>
+      </c>
+      <c r="B1382" t="str">
+        <v>الضوابط المحددة</v>
+      </c>
+      <c r="C1382" t="str">
+        <v>Izvēlētās kontroles</v>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="str">
+        <v>Create Evidence</v>
+      </c>
+      <c r="B1383" t="str">
+        <v>إنشاء دليل</v>
+      </c>
+      <c r="C1383" t="str">
+        <v>Izveidot pierādījumu</v>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="str">
+        <v>Delete All Evidence</v>
+      </c>
+      <c r="B1384" t="str">
+        <v>حذف جميع الأدلة</v>
+      </c>
+      <c r="C1384" t="str">
+        <v>Dzēst visus pierādījumus</v>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="str">
+        <v>Are you sure you want to delete all evidence records? This action cannot be undone.</v>
+      </c>
+      <c r="B1385" t="str">
+        <v>هل أنت متأكد أنك تريد حذف جميع سجلات الأدلة؟ لا يمكن التراجع عن هذا الإجراء.</v>
+      </c>
+      <c r="C1385" t="str">
+        <v>Vai tiešām vēlaties dzēst visus pierādījumu ierakstus? Šo darbību nevar atsaukt.</v>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="str">
+        <v>Import Evidence</v>
+      </c>
+      <c r="B1386" t="str">
+        <v>استيراد الأدلة</v>
+      </c>
+      <c r="C1386" t="str">
+        <v>Importēt pierādījumus</v>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="str">
+        <v>Upload a CSV or Excel file to import evidence records.</v>
+      </c>
+      <c r="B1387" t="str">
+        <v>ارفع ملف CSV أو Excel لاستيراد سجلات الأدلة.</v>
+      </c>
+      <c r="C1387" t="str">
+        <v>Augšupielādējiet CSV vai Excel failu, lai importētu pierādījumu ierakstus.</v>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="str">
+        <v>Drag and drop a file here, or click to browse</v>
+      </c>
+      <c r="B1388" t="str">
+        <v>اسحب وأفلت ملفاً هنا، أو انقر للتصفح</v>
+      </c>
+      <c r="C1388" t="str">
+        <v>Velciet un nometiet failu šeit vai noklikšķiniet, lai pārlūkotu</v>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="str">
+        <v>Search by Evidence Code, Name</v>
+      </c>
+      <c r="B1389" t="str">
+        <v>البحث برمز الدليل أو الاسم</v>
+      </c>
+      <c r="C1389" t="str">
+        <v>Meklēt pēc pierādījuma koda, nosaukuma</v>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="str">
+        <v>No evidences found</v>
+      </c>
+      <c r="B1390" t="str">
+        <v>لم يتم العثور على أدلة</v>
+      </c>
+      <c r="C1390" t="str">
+        <v>Nav atrasti pierādījumi</v>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="str">
+        <v>Link Evidences</v>
+      </c>
+      <c r="B1391" t="str">
+        <v>ربط الأدلة</v>
+      </c>
+      <c r="C1391" t="str">
+        <v>Saistīt pierādījumus</v>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="str">
+        <v>No evidence records found</v>
+      </c>
+      <c r="B1392" t="str">
+        <v>لم يتم العثور على سجلات أدلة</v>
+      </c>
+      <c r="C1392" t="str">
+        <v>Nav atrasti pierādījumu ieraksti</v>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="str">
+        <v>Create a new evidence record to get started</v>
+      </c>
+      <c r="B1393" t="str">
+        <v>أنشئ سجل دليل جديد للبدء</v>
+      </c>
+      <c r="C1393" t="str">
+        <v>Izveidojiet jaunu pierādījuma ierakstu, lai sāktu</v>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="str">
+        <v>Add Artifact</v>
+      </c>
+      <c r="B1394" t="str">
+        <v>إضافة مستند مرفق</v>
+      </c>
+      <c r="C1394" t="str">
+        <v>Pievienot artefaktu</v>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="str">
+        <v>AI Review Artifacts</v>
+      </c>
+      <c r="B1395" t="str">
+        <v>مراجعة المستندات بالذكاء الاصطناعي</v>
+      </c>
+      <c r="C1395" t="str">
+        <v>AI pārskatīt artefaktus</v>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="str">
+        <v>click to upload</v>
+      </c>
+      <c r="B1396" t="str">
+        <v>انقر للرفع</v>
+      </c>
+      <c r="C1396" t="str">
+        <v>noklikšķiniet, lai augšupielādētu</v>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="str">
+        <v>Supported formats: PDF, PNG, JPG, XLSX, DOC, DOCX</v>
+      </c>
+      <c r="B1397" t="str">
+        <v>الصيغ المدعومة: PDF، PNG، JPG، XLSX، DOC، DOCX</v>
+      </c>
+      <c r="C1397" t="str">
+        <v>Atbalstītie formāti: PDF, PNG, JPG, XLSX, DOC, DOCX</v>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="str">
+        <v>Uploaded Artifacts</v>
+      </c>
+      <c r="B1398" t="str">
+        <v>المستندات المرفقة المرفوعة</v>
+      </c>
+      <c r="C1398" t="str">
+        <v>Augšupielādētie artefakti</v>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="str">
+        <v>No artifacts uploaded yet</v>
+      </c>
+      <c r="B1399" t="str">
+        <v>لم يتم رفع مستندات مرفقة بعد</v>
+      </c>
+      <c r="C1399" t="str">
+        <v>Vēl nav augšupielādēti artefakti</v>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="str">
+        <v>Upload files above to get started</v>
+      </c>
+      <c r="B1400" t="str">
+        <v>ارفع الملفات أعلاه للبدء</v>
+      </c>
+      <c r="C1400" t="str">
+        <v>Augšupielādējiet failus iepriekš, lai sāktu</v>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="str">
+        <v>Link to Evidence</v>
+      </c>
+      <c r="B1401" t="str">
+        <v>ربط بالدليل</v>
+      </c>
+      <c r="C1401" t="str">
+        <v>Saistīt ar pierādījumu</v>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="str">
+        <v>Enter description</v>
+      </c>
+      <c r="B1402" t="str">
+        <v>أدخل الوصف</v>
+      </c>
+      <c r="C1402" t="str">
+        <v>Ievadiet aprakstu</v>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="str">
+        <v>Please select the recurrence</v>
+      </c>
+      <c r="B1403" t="str">
+        <v>يرجى اختيار التكرار</v>
+      </c>
+      <c r="C1403" t="str">
+        <v>Lūdzu izvēlieties atkārtošanos</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C1137"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C1403"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Arabic and Latvian translations for Evidence Details page
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1403"/>
+  <dimension ref="A1:C1536"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -15837,9 +15837,1472 @@
         <v>Lūdzu izvēlieties atkārtošanos</v>
       </c>
     </row>
+    <row r="1404">
+      <c r="A1404" t="str">
+        <v>Jan</v>
+      </c>
+      <c r="B1404" t="str">
+        <v>يناير</v>
+      </c>
+      <c r="C1404" t="str">
+        <v>Jan</v>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="str">
+        <v>Feb</v>
+      </c>
+      <c r="B1405" t="str">
+        <v>فبراير</v>
+      </c>
+      <c r="C1405" t="str">
+        <v>Feb</v>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="str">
+        <v>Mar</v>
+      </c>
+      <c r="B1406" t="str">
+        <v>مارس</v>
+      </c>
+      <c r="C1406" t="str">
+        <v>Mar</v>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="str">
+        <v>Apr</v>
+      </c>
+      <c r="B1407" t="str">
+        <v>أبريل</v>
+      </c>
+      <c r="C1407" t="str">
+        <v>Apr</v>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" t="str">
+        <v>May</v>
+      </c>
+      <c r="B1408" t="str">
+        <v>مايو</v>
+      </c>
+      <c r="C1408" t="str">
+        <v>Mai</v>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="str">
+        <v>Jun</v>
+      </c>
+      <c r="B1409" t="str">
+        <v>يونيو</v>
+      </c>
+      <c r="C1409" t="str">
+        <v>Jūn</v>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" t="str">
+        <v>Jul</v>
+      </c>
+      <c r="B1410" t="str">
+        <v>يوليو</v>
+      </c>
+      <c r="C1410" t="str">
+        <v>Jūl</v>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="str">
+        <v>Aug</v>
+      </c>
+      <c r="B1411" t="str">
+        <v>أغسطس</v>
+      </c>
+      <c r="C1411" t="str">
+        <v>Aug</v>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="str">
+        <v>Sep</v>
+      </c>
+      <c r="B1412" t="str">
+        <v>سبتمبر</v>
+      </c>
+      <c r="C1412" t="str">
+        <v>Sep</v>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="str">
+        <v>Oct</v>
+      </c>
+      <c r="B1413" t="str">
+        <v>أكتوبر</v>
+      </c>
+      <c r="C1413" t="str">
+        <v>Okt</v>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="str">
+        <v>Nov</v>
+      </c>
+      <c r="B1414" t="str">
+        <v>نوفمبر</v>
+      </c>
+      <c r="C1414" t="str">
+        <v>Nov</v>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="str">
+        <v>Dec</v>
+      </c>
+      <c r="B1415" t="str">
+        <v>ديسمبر</v>
+      </c>
+      <c r="C1415" t="str">
+        <v>Dec</v>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="str">
+        <v>Jan–Mar</v>
+      </c>
+      <c r="B1416" t="str">
+        <v>يناير–مارس</v>
+      </c>
+      <c r="C1416" t="str">
+        <v>Jan–Mar</v>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" t="str">
+        <v>Apr–Jun</v>
+      </c>
+      <c r="B1417" t="str">
+        <v>أبريل–يونيو</v>
+      </c>
+      <c r="C1417" t="str">
+        <v>Apr–Jūn</v>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" t="str">
+        <v>Jul–Sep</v>
+      </c>
+      <c r="B1418" t="str">
+        <v>يوليو–سبتمبر</v>
+      </c>
+      <c r="C1418" t="str">
+        <v>Jūl–Sep</v>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" t="str">
+        <v>Oct–Dec</v>
+      </c>
+      <c r="B1419" t="str">
+        <v>أكتوبر–ديسمبر</v>
+      </c>
+      <c r="C1419" t="str">
+        <v>Okt–Dec</v>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" t="str">
+        <v>Jan–Jun</v>
+      </c>
+      <c r="B1420" t="str">
+        <v>يناير–يونيو</v>
+      </c>
+      <c r="C1420" t="str">
+        <v>Jan–Jūn</v>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" t="str">
+        <v>Jul–Dec</v>
+      </c>
+      <c r="B1421" t="str">
+        <v>يوليو–ديسمبر</v>
+      </c>
+      <c r="C1421" t="str">
+        <v>Jūl–Dec</v>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" t="str">
+        <v>Jan–Dec</v>
+      </c>
+      <c r="B1422" t="str">
+        <v>يناير–ديسمبر</v>
+      </c>
+      <c r="C1422" t="str">
+        <v>Jan–Dec</v>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" t="str">
+        <v>Organization Wide</v>
+      </c>
+      <c r="B1423" t="str">
+        <v>على مستوى المنظمة</v>
+      </c>
+      <c r="C1423" t="str">
+        <v>Organizācijas mērogā</v>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" t="str">
+        <v>No attachments for</v>
+      </c>
+      <c r="B1424" t="str">
+        <v>لا توجد مرفقات لـ</v>
+      </c>
+      <c r="C1424" t="str">
+        <v>Nav pielikumu par</v>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" t="str">
+        <v>No attachments</v>
+      </c>
+      <c r="B1425" t="str">
+        <v>لا توجد مرفقات</v>
+      </c>
+      <c r="C1425" t="str">
+        <v>Nav pielikumu</v>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" t="str">
+        <v>Evidence Details</v>
+      </c>
+      <c r="B1426" t="str">
+        <v>تفاصيل الدليل</v>
+      </c>
+      <c r="C1426" t="str">
+        <v>Pierādījuma detaļas</v>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" t="str">
+        <v>Evidence not found</v>
+      </c>
+      <c r="B1427" t="str">
+        <v>لم يتم العثور على الدليل</v>
+      </c>
+      <c r="C1427" t="str">
+        <v>Pierādījums nav atrasts</v>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" t="str">
+        <v>Artifact</v>
+      </c>
+      <c r="B1428" t="str">
+        <v>المستند المرفق</v>
+      </c>
+      <c r="C1428" t="str">
+        <v>Artefakts</v>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" t="str">
+        <v>Review date</v>
+      </c>
+      <c r="B1429" t="str">
+        <v>تاريخ المراجعة</v>
+      </c>
+      <c r="C1429" t="str">
+        <v>Pārskatīšanas datums</v>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" t="str">
+        <v>Select review date</v>
+      </c>
+      <c r="B1430" t="str">
+        <v>اختر تاريخ المراجعة</v>
+      </c>
+      <c r="C1430" t="str">
+        <v>Izvēlieties pārskatīšanas datumu</v>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" t="str">
+        <v>Linked Artifact</v>
+      </c>
+      <c r="B1431" t="str">
+        <v>المستند المرتبط</v>
+      </c>
+      <c r="C1431" t="str">
+        <v>Saistītais artefakts</v>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" t="str">
+        <v>Linked Artifacts</v>
+      </c>
+      <c r="B1432" t="str">
+        <v>المستندات المرتبطة</v>
+      </c>
+      <c r="C1432" t="str">
+        <v>Saistītie artefakti</v>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" t="str">
+        <v>KPI Calculation Formula</v>
+      </c>
+      <c r="B1433" t="str">
+        <v>صيغة حساب مؤشر الأداء</v>
+      </c>
+      <c r="C1433" t="str">
+        <v>KPI aprēķina formula</v>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" t="str">
+        <v>Linked Frameworks:</v>
+      </c>
+      <c r="B1434" t="str">
+        <v>الأطر المرتبطة:</v>
+      </c>
+      <c r="C1434" t="str">
+        <v>Saistītie ietvari:</v>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" t="str">
+        <v>No controls linked to this evidence</v>
+      </c>
+      <c r="B1435" t="str">
+        <v>لا توجد ضوابط مرتبطة بهذا الدليل</v>
+      </c>
+      <c r="C1435" t="str">
+        <v>Nav kontroles saistītas ar šo pierādījumu</v>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" t="str">
+        <v>No artifacts linked to this evidence</v>
+      </c>
+      <c r="B1436" t="str">
+        <v>لا توجد مستندات مرتبطة بهذا الدليل</v>
+      </c>
+      <c r="C1436" t="str">
+        <v>Nav artefaktu saistītu ar šo pierādījumu</v>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" t="str">
+        <v>Assigned to</v>
+      </c>
+      <c r="B1437" t="str">
+        <v>مكلّف إلى</v>
+      </c>
+      <c r="C1437" t="str">
+        <v>Piešķirts</v>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" t="str">
+        <v>KPI Required</v>
+      </c>
+      <c r="B1438" t="str">
+        <v>مؤشر الأداء مطلوب</v>
+      </c>
+      <c r="C1438" t="str">
+        <v>KPI nepieciešams</v>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" t="str">
+        <v>KPI Expected Score (%)</v>
+      </c>
+      <c r="B1439" t="str">
+        <v>الدرجة المتوقعة لمؤشر الأداء (%)</v>
+      </c>
+      <c r="C1439" t="str">
+        <v>KPI sagaidāmais rezultāts (%)</v>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" t="str">
+        <v>KPI Actual Score</v>
+      </c>
+      <c r="B1440" t="str">
+        <v>الدرجة الفعلية لمؤشر الأداء</v>
+      </c>
+      <c r="C1440" t="str">
+        <v>KPI faktiskais rezultāts</v>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" t="str">
+        <v>Enter expected score</v>
+      </c>
+      <c r="B1441" t="str">
+        <v>أدخل الدرجة المتوقعة</v>
+      </c>
+      <c r="C1441" t="str">
+        <v>Ievadiet sagaidāmo rezultātu</v>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" t="str">
+        <v>Enter KPI Description</v>
+      </c>
+      <c r="B1442" t="str">
+        <v>أدخل وصف مؤشر الأداء</v>
+      </c>
+      <c r="C1442" t="str">
+        <v>Ievadiet KPI aprakstu</v>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" t="str">
+        <v>Enter actual score</v>
+      </c>
+      <c r="B1443" t="str">
+        <v>أدخل الدرجة الفعلية</v>
+      </c>
+      <c r="C1443" t="str">
+        <v>Ievadiet faktisko rezultātu</v>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" t="str">
+        <v>Save KPI details first</v>
+      </c>
+      <c r="B1444" t="str">
+        <v>احفظ تفاصيل مؤشر الأداء أولاً</v>
+      </c>
+      <c r="C1444" t="str">
+        <v>Vispirms saglabājiet KPI detaļas</v>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" t="str">
+        <v>Save actual score</v>
+      </c>
+      <c r="B1445" t="str">
+        <v>حفظ الدرجة الفعلية</v>
+      </c>
+      <c r="C1445" t="str">
+        <v>Saglabāt faktisko rezultātu</v>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" t="str">
+        <v>Edit actual score</v>
+      </c>
+      <c r="B1446" t="str">
+        <v>تعديل الدرجة الفعلية</v>
+      </c>
+      <c r="C1446" t="str">
+        <v>Rediģēt faktisko rezultātu</v>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" t="str">
+        <v>Save KPI details first to enable saving actual score</v>
+      </c>
+      <c r="B1447" t="str">
+        <v>احفظ تفاصيل مؤشر الأداء أولاً لتتمكن من حفظ الدرجة الفعلية</v>
+      </c>
+      <c r="C1447" t="str">
+        <v>Vispirms saglabājiet KPI detaļas, lai varētu saglabāt faktisko rezultātu</v>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" t="str">
+        <v>Unpublish</v>
+      </c>
+      <c r="B1448" t="str">
+        <v>إلغاء النشر</v>
+      </c>
+      <c r="C1448" t="str">
+        <v>Atcelt publicēšanu</v>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" t="str">
+        <v>Published On:</v>
+      </c>
+      <c r="B1449" t="str">
+        <v>تاريخ النشر:</v>
+      </c>
+      <c r="C1449" t="str">
+        <v>Publicēts:</v>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" t="str">
+        <v>No published files</v>
+      </c>
+      <c r="B1450" t="str">
+        <v>لا توجد ملفات منشورة</v>
+      </c>
+      <c r="C1450" t="str">
+        <v>Nav publicētu failu</v>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" t="str">
+        <v>Add Attachment</v>
+      </c>
+      <c r="B1451" t="str">
+        <v>إضافة مرفق</v>
+      </c>
+      <c r="C1451" t="str">
+        <v>Pievienot pielikumu</v>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" t="str">
+        <v>Add Evidence Attachment</v>
+      </c>
+      <c r="B1452" t="str">
+        <v>إضافة مرفق الدليل</v>
+      </c>
+      <c r="C1452" t="str">
+        <v>Pievienot pierādījuma pielikumu</v>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" t="str">
+        <v>Drag and drop or select file.</v>
+      </c>
+      <c r="B1453" t="str">
+        <v>اسحب وأفلت أو اختر ملفاً.</v>
+      </c>
+      <c r="C1453" t="str">
+        <v>Velciet un nometiet vai izvēlieties failu.</v>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" t="str">
+        <v>Submitting...</v>
+      </c>
+      <c r="B1454" t="str">
+        <v>جارٍ الإرسال...</v>
+      </c>
+      <c r="C1454" t="str">
+        <v>Iesniedz...</v>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" t="str">
+        <v>Link Artifacts</v>
+      </c>
+      <c r="B1455" t="str">
+        <v>ربط المستندات المرفقة</v>
+      </c>
+      <c r="C1455" t="str">
+        <v>Saistīt artefaktus</v>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" t="str">
+        <v>Search by Artifact Code or Name...</v>
+      </c>
+      <c r="B1456" t="str">
+        <v>البحث برمز المستند أو الاسم...</v>
+      </c>
+      <c r="C1456" t="str">
+        <v>Meklēt pēc artefakta koda vai nosaukuma...</v>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" t="str">
+        <v>No artifacts found matching your search</v>
+      </c>
+      <c r="B1457" t="str">
+        <v>لم يتم العثور على مستندات تطابق بحثك</v>
+      </c>
+      <c r="C1457" t="str">
+        <v>Nav atrasti artefakti, kas atbilst jūsu meklējumam</v>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" t="str">
+        <v>No available artifacts to link</v>
+      </c>
+      <c r="B1458" t="str">
+        <v>لا توجد مستندات متاحة للربط</v>
+      </c>
+      <c r="C1458" t="str">
+        <v>Nav pieejamu artefaktu saistīšanai</v>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" t="str">
+        <v>artifact(s) selected</v>
+      </c>
+      <c r="B1459" t="str">
+        <v>مستند(ات) محددة</v>
+      </c>
+      <c r="C1459" t="str">
+        <v>artefakts(-i) izvēlēti</v>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" t="str">
+        <v>Linking...</v>
+      </c>
+      <c r="B1460" t="str">
+        <v>جارٍ الربط...</v>
+      </c>
+      <c r="C1460" t="str">
+        <v>Saista...</v>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" t="str">
+        <v>Link Controls</v>
+      </c>
+      <c r="B1461" t="str">
+        <v>ربط الضوابط</v>
+      </c>
+      <c r="C1461" t="str">
+        <v>Saistīt kontroles</v>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" t="str">
+        <v>No controls found matching your filters</v>
+      </c>
+      <c r="B1462" t="str">
+        <v>لم يتم العثور على ضوابط تطابق عوامل التصفية</v>
+      </c>
+      <c r="C1462" t="str">
+        <v>Nav atrasti kontroli, kas atbilst jūsu filtriem</v>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" t="str">
+        <v>No available controls to link</v>
+      </c>
+      <c r="B1463" t="str">
+        <v>لا توجد ضوابط متاحة للربط</v>
+      </c>
+      <c r="C1463" t="str">
+        <v>Nav pieejamu kontrolu saistīšanai</v>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" t="str">
+        <v>Unlink</v>
+      </c>
+      <c r="B1464" t="str">
+        <v>إلغاء الربط</v>
+      </c>
+      <c r="C1464" t="str">
+        <v>Atsaistīt</v>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" t="str">
+        <v>Recent Comments</v>
+      </c>
+      <c r="B1465" t="str">
+        <v>التعليقات الأخيرة</v>
+      </c>
+      <c r="C1465" t="str">
+        <v>Jaunākie komentāri</v>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" t="str">
+        <v>Add Comment</v>
+      </c>
+      <c r="B1466" t="str">
+        <v>إضافة تعليق</v>
+      </c>
+      <c r="C1466" t="str">
+        <v>Pievienot komentāru</v>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" t="str">
+        <v>Add a comment</v>
+      </c>
+      <c r="B1467" t="str">
+        <v>أضف تعليقاً</v>
+      </c>
+      <c r="C1467" t="str">
+        <v>Pievienojiet komentāru</v>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" t="str">
+        <v>Type your comment...</v>
+      </c>
+      <c r="B1468" t="str">
+        <v>اكتب تعليقك...</v>
+      </c>
+      <c r="C1468" t="str">
+        <v>Rakstiet komentāru...</v>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" t="str">
+        <v>No comments yet</v>
+      </c>
+      <c r="B1469" t="str">
+        <v>لا توجد تعليقات بعد</v>
+      </c>
+      <c r="C1469" t="str">
+        <v>Vēl nav komentāru</v>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" t="str">
+        <v>Unknown User</v>
+      </c>
+      <c r="B1470" t="str">
+        <v>مستخدم غير معروف</v>
+      </c>
+      <c r="C1470" t="str">
+        <v>Nezināms lietotājs</v>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" t="str">
+        <v>View all</v>
+      </c>
+      <c r="B1471" t="str">
+        <v>عرض الكل</v>
+      </c>
+      <c r="C1471" t="str">
+        <v>Skatīt visus</v>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" t="str">
+        <v>comments</v>
+      </c>
+      <c r="B1472" t="str">
+        <v>تعليقات</v>
+      </c>
+      <c r="C1472" t="str">
+        <v>komentāri</v>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" t="str">
+        <v>View Comments</v>
+      </c>
+      <c r="B1473" t="str">
+        <v>عرض التعليقات</v>
+      </c>
+      <c r="C1473" t="str">
+        <v>Skatīt komentārus</v>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" t="str">
+        <v>Comment</v>
+      </c>
+      <c r="B1474" t="str">
+        <v>تعليق</v>
+      </c>
+      <c r="C1474" t="str">
+        <v>Komentārs</v>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" t="str">
+        <v>Enter your comment...</v>
+      </c>
+      <c r="B1475" t="str">
+        <v>أدخل تعليقك...</v>
+      </c>
+      <c r="C1475" t="str">
+        <v>Ievadiet komentāru...</v>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" t="str">
+        <v>Previous Comments</v>
+      </c>
+      <c r="B1476" t="str">
+        <v>التعليقات السابقة</v>
+      </c>
+      <c r="C1476" t="str">
+        <v>Iepriekšējie komentāri</v>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" t="str">
+        <v>Submit for Approval</v>
+      </c>
+      <c r="B1477" t="str">
+        <v>إرسال للموافقة</v>
+      </c>
+      <c r="C1477" t="str">
+        <v>Iesniegt apstiprināšanai</v>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" t="str">
+        <v>Validate</v>
+      </c>
+      <c r="B1478" t="str">
+        <v>تحقق</v>
+      </c>
+      <c r="C1478" t="str">
+        <v>Validēt</v>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" t="str">
+        <v>Send Back</v>
+      </c>
+      <c r="B1479" t="str">
+        <v>إرجاع</v>
+      </c>
+      <c r="C1479" t="str">
+        <v>Nosūtīt atpakaļ</v>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" t="str">
+        <v>Resubmit</v>
+      </c>
+      <c r="B1480" t="str">
+        <v>إعادة الإرسال</v>
+      </c>
+      <c r="C1480" t="str">
+        <v>Iesniegt atkārtoti</v>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" t="str">
+        <v>Resend</v>
+      </c>
+      <c r="B1481" t="str">
+        <v>إعادة الإرسال</v>
+      </c>
+      <c r="C1481" t="str">
+        <v>Nosūtīt atkārtoti</v>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" t="str">
+        <v>This cycle has been validated</v>
+      </c>
+      <c r="B1482" t="str">
+        <v>تم التحقق من هذه الدورة</v>
+      </c>
+      <c r="C1482" t="str">
+        <v>Šis cikls ir validēts</v>
+      </c>
+    </row>
+    <row r="1483">
+      <c r="A1483" t="str">
+        <v>This cycle has been sent back</v>
+      </c>
+      <c r="B1483" t="str">
+        <v>تم إرجاع هذه الدورة</v>
+      </c>
+      <c r="C1483" t="str">
+        <v>Šis cikls ir nosūtīts atpakaļ</v>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" t="str">
+        <v>Awaiting submission from Department Contributor</v>
+      </c>
+      <c r="B1484" t="str">
+        <v>في انتظار الإرسال من مساهم القسم</v>
+      </c>
+      <c r="C1484" t="str">
+        <v>Gaida iesniegumu no nodaļas līdzstrādnieka</v>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" t="str">
+        <v>Evidence Send Back</v>
+      </c>
+      <c r="B1485" t="str">
+        <v>إرجاع الدليل</v>
+      </c>
+      <c r="C1485" t="str">
+        <v>Pierādījuma nosūtīšana atpakaļ</v>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" t="str">
+        <v>Cannot Publish</v>
+      </c>
+      <c r="B1486" t="str">
+        <v>لا يمكن النشر</v>
+      </c>
+      <c r="C1486" t="str">
+        <v>Nevar publicēt</v>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" t="str">
+        <v>Current cycle:</v>
+      </c>
+      <c r="B1487" t="str">
+        <v>الدورة الحالية:</v>
+      </c>
+      <c r="C1487" t="str">
+        <v>Pašreizējais cikls:</v>
+      </c>
+    </row>
+    <row r="1488">
+      <c r="A1488" t="str">
+        <v>Are you sure you want to delete this evidence? This action cannot be undone.</v>
+      </c>
+      <c r="B1488" t="str">
+        <v>هل أنت متأكد أنك تريد حذف هذا الدليل؟ لا يمكن التراجع عن هذا الإجراء.</v>
+      </c>
+      <c r="C1488" t="str">
+        <v>Vai tiešām vēlaties dzēst šo pierādījumu? Šo darbību nevar atsaukt.</v>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" t="str">
+        <v>Status reverted to Draft: Current cycle is not validated.</v>
+      </c>
+      <c r="B1489" t="str">
+        <v>تم إرجاع الحالة إلى مسودة: الدورة الحالية غير مُتحقق منها.</v>
+      </c>
+      <c r="C1489" t="str">
+        <v>Statuss atgriezts uz Melnrakstu: Pašreizējais cikls nav validēts.</v>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" t="str">
+        <v>Please upload an attachment for this cycle first.</v>
+      </c>
+      <c r="B1490" t="str">
+        <v>يرجى رفع مرفق لهذه الدورة أولاً.</v>
+      </c>
+      <c r="C1490" t="str">
+        <v>Lūdzu vispirms augšupielādējiet pielikumu šim ciklam.</v>
+      </c>
+    </row>
+    <row r="1491">
+      <c r="A1491" t="str">
+        <v>Submitted for approval successfully.</v>
+      </c>
+      <c r="B1491" t="str">
+        <v>تم الإرسال للموافقة بنجاح.</v>
+      </c>
+      <c r="C1491" t="str">
+        <v>Veiksmīgi iesniegts apstiprināšanai.</v>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" t="str">
+        <v>cycle validated. Evidence status updated to Validated.</v>
+      </c>
+      <c r="B1492" t="str">
+        <v>تم التحقق من الدورة. تم تحديث حالة الدليل إلى مُتحقق.</v>
+      </c>
+      <c r="C1492" t="str">
+        <v>Cikls validēts. Pierādījuma statuss atjaunināts uz Validēts.</v>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" t="str">
+        <v>cycle validated successfully.</v>
+      </c>
+      <c r="B1493" t="str">
+        <v>تم التحقق من الدورة بنجاح.</v>
+      </c>
+      <c r="C1493" t="str">
+        <v>Cikls veiksmīgi validēts.</v>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" t="str">
+        <v>cycle sent back.</v>
+      </c>
+      <c r="B1494" t="str">
+        <v>تم إرجاع الدورة.</v>
+      </c>
+      <c r="C1494" t="str">
+        <v>Cikls nosūtīts atpakaļ.</v>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" t="str">
+        <v>Failed to send back.</v>
+      </c>
+      <c r="B1495" t="str">
+        <v>فشل الإرجاع.</v>
+      </c>
+      <c r="C1495" t="str">
+        <v>Neizdevās nosūtīt atpakaļ.</v>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" t="str">
+        <v>cycle resubmitted.</v>
+      </c>
+      <c r="B1496" t="str">
+        <v>تم إعادة إرسال الدورة.</v>
+      </c>
+      <c r="C1496" t="str">
+        <v>Cikls atkārtoti iesniegts.</v>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" t="str">
+        <v>Failed to resubmit.</v>
+      </c>
+      <c r="B1497" t="str">
+        <v>فشلت إعادة الإرسال.</v>
+      </c>
+      <c r="C1497" t="str">
+        <v>Neizdevās iesniegt atkārtoti.</v>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" t="str">
+        <v>Current cycle document is not validated.</v>
+      </c>
+      <c r="B1498" t="str">
+        <v>مستند الدورة الحالية غير مُتحقق منه.</v>
+      </c>
+      <c r="C1498" t="str">
+        <v>Pašreizējā cikla dokuments nav validēts.</v>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" t="str">
+        <v>Failed to save KPI details to evidence</v>
+      </c>
+      <c r="B1499" t="str">
+        <v>فشل حفظ تفاصيل مؤشر الأداء في الدليل</v>
+      </c>
+      <c r="C1499" t="str">
+        <v>Neizdevās saglabāt KPI detaļas pierādījumam</v>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" t="str">
+        <v>KPI updated successfully!</v>
+      </c>
+      <c r="B1500" t="str">
+        <v>تم تحديث مؤشر الأداء بنجاح!</v>
+      </c>
+      <c r="C1500" t="str">
+        <v>KPI veiksmīgi atjaunināts!</v>
+      </c>
+    </row>
+    <row r="1501">
+      <c r="A1501" t="str">
+        <v>KPI created successfully!</v>
+      </c>
+      <c r="B1501" t="str">
+        <v>تم إنشاء مؤشر الأداء بنجاح!</v>
+      </c>
+      <c r="C1501" t="str">
+        <v>KPI veiksmīgi izveidots!</v>
+      </c>
+    </row>
+    <row r="1502">
+      <c r="A1502" t="str">
+        <v>Failed to save KPI</v>
+      </c>
+      <c r="B1502" t="str">
+        <v>فشل حفظ مؤشر الأداء</v>
+      </c>
+      <c r="C1502" t="str">
+        <v>Neizdevās saglabāt KPI</v>
+      </c>
+    </row>
+    <row r="1503">
+      <c r="A1503" t="str">
+        <v>Please save KPI details first before saving actual score</v>
+      </c>
+      <c r="B1503" t="str">
+        <v>يرجى حفظ تفاصيل مؤشر الأداء أولاً قبل حفظ الدرجة الفعلية</v>
+      </c>
+      <c r="C1503" t="str">
+        <v>Lūdzu vispirms saglabājiet KPI detaļas pirms faktiskā rezultāta saglabāšanas</v>
+      </c>
+    </row>
+    <row r="1504">
+      <c r="A1504" t="str">
+        <v>KPI Actual Score saved successfully!</v>
+      </c>
+      <c r="B1504" t="str">
+        <v>تم حفظ الدرجة الفعلية لمؤشر الأداء بنجاح!</v>
+      </c>
+      <c r="C1504" t="str">
+        <v>KPI faktiskais rezultāts veiksmīgi saglabāts!</v>
+      </c>
+    </row>
+    <row r="1505">
+      <c r="A1505" t="str">
+        <v>Failed to save KPI Actual Score</v>
+      </c>
+      <c r="B1505" t="str">
+        <v>فشل حفظ الدرجة الفعلية لمؤشر الأداء</v>
+      </c>
+      <c r="C1505" t="str">
+        <v>Neizdevās saglabāt KPI faktisko rezultātu</v>
+      </c>
+    </row>
+    <row r="1506">
+      <c r="A1506" t="str">
+        <v>Attachment uploaded successfully!</v>
+      </c>
+      <c r="B1506" t="str">
+        <v>تم رفع المرفق بنجاح!</v>
+      </c>
+      <c r="C1506" t="str">
+        <v>Pielikums veiksmīgi augšupielādēts!</v>
+      </c>
+    </row>
+    <row r="1507">
+      <c r="A1507" t="str">
+        <v>Failed to upload attachment</v>
+      </c>
+      <c r="B1507" t="str">
+        <v>فشل رفع المرفق</v>
+      </c>
+      <c r="C1507" t="str">
+        <v>Neizdevās augšupielādēt pielikumu</v>
+      </c>
+    </row>
+    <row r="1508">
+      <c r="A1508" t="str">
+        <v>Attachment deleted successfully!</v>
+      </c>
+      <c r="B1508" t="str">
+        <v>تم حذف المرفق بنجاح!</v>
+      </c>
+      <c r="C1508" t="str">
+        <v>Pielikums veiksmīgi dzēsts!</v>
+      </c>
+    </row>
+    <row r="1509">
+      <c r="A1509" t="str">
+        <v>Artifacts linked successfully!</v>
+      </c>
+      <c r="B1509" t="str">
+        <v>تم ربط المستندات بنجاح!</v>
+      </c>
+      <c r="C1509" t="str">
+        <v>Artefakti veiksmīgi saistīti!</v>
+      </c>
+    </row>
+    <row r="1510">
+      <c r="A1510" t="str">
+        <v>Failed to link artifacts</v>
+      </c>
+      <c r="B1510" t="str">
+        <v>فشل ربط المستندات</v>
+      </c>
+      <c r="C1510" t="str">
+        <v>Neizdevās saistīt artefaktus</v>
+      </c>
+    </row>
+    <row r="1511">
+      <c r="A1511" t="str">
+        <v>Artifact unlinked successfully!</v>
+      </c>
+      <c r="B1511" t="str">
+        <v>تم إلغاء ربط المستند بنجاح!</v>
+      </c>
+      <c r="C1511" t="str">
+        <v>Artefakts veiksmīgi atsaistīts!</v>
+      </c>
+    </row>
+    <row r="1512">
+      <c r="A1512" t="str">
+        <v>Please upload evidence files first</v>
+      </c>
+      <c r="B1512" t="str">
+        <v>يرجى رفع ملفات الأدلة أولاً</v>
+      </c>
+      <c r="C1512" t="str">
+        <v>Lūdzu vispirms augšupielādējiet pierādījumu failus</v>
+      </c>
+    </row>
+    <row r="1513">
+      <c r="A1513" t="str">
+        <v>Failed to trigger AI ingest</v>
+      </c>
+      <c r="B1513" t="str">
+        <v>فشل بدء معالجة الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1513" t="str">
+        <v>Neizdevās aktivizēt AI apstrādi</v>
+      </c>
+    </row>
+    <row r="1514">
+      <c r="A1514" t="str">
+        <v>AI ingest started successfully</v>
+      </c>
+      <c r="B1514" t="str">
+        <v>بدأت معالجة الذكاء الاصطناعي بنجاح</v>
+      </c>
+      <c r="C1514" t="str">
+        <v>AI apstrāde veiksmīgi sākta</v>
+      </c>
+    </row>
+    <row r="1515">
+      <c r="A1515" t="str">
+        <v>Failed to trigger AI review</v>
+      </c>
+      <c r="B1515" t="str">
+        <v>فشل بدء مراجعة الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1515" t="str">
+        <v>Neizdevās aktivizēt AI pārskatīšanu</v>
+      </c>
+    </row>
+    <row r="1516">
+      <c r="A1516" t="str">
+        <v>AI review completed successfully</v>
+      </c>
+      <c r="B1516" t="str">
+        <v>اكتملت مراجعة الذكاء الاصطناعي بنجاح</v>
+      </c>
+      <c r="C1516" t="str">
+        <v>AI pārskatīšana veiksmīgi pabeigta</v>
+      </c>
+    </row>
+    <row r="1517">
+      <c r="A1517" t="str">
+        <v>Failed to clear AI review</v>
+      </c>
+      <c r="B1517" t="str">
+        <v>فشل مسح مراجعة الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1517" t="str">
+        <v>Neizdevās notīrīt AI pārskatīšanu</v>
+      </c>
+    </row>
+    <row r="1518">
+      <c r="A1518" t="str">
+        <v>AI review cleared successfully</v>
+      </c>
+      <c r="B1518" t="str">
+        <v>تم مسح مراجعة الذكاء الاصطناعي بنجاح</v>
+      </c>
+      <c r="C1518" t="str">
+        <v>AI pārskatīšana veiksmīgi notīrīta</v>
+      </c>
+    </row>
+    <row r="1519">
+      <c r="A1519" t="str">
+        <v>Clear AI Review</v>
+      </c>
+      <c r="B1519" t="str">
+        <v>مسح مراجعة الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1519" t="str">
+        <v>Notīrīt AI pārskatīšanu</v>
+      </c>
+    </row>
+    <row r="1520">
+      <c r="A1520" t="str">
+        <v>Upload evidence files and trigger AI processing to extract and analyze content.</v>
+      </c>
+      <c r="B1520" t="str">
+        <v>ارفع ملفات الأدلة وابدأ معالجة الذكاء الاصطناعي لاستخراج المحتوى وتحليله.</v>
+      </c>
+      <c r="C1520" t="str">
+        <v>Augšupielādējiet pierādījumu failus un aktivizējiet AI apstrādi, lai izvilktu un analizētu saturu.</v>
+      </c>
+    </row>
+    <row r="1521">
+      <c r="A1521" t="str">
+        <v>Starting AI Processing...</v>
+      </c>
+      <c r="B1521" t="str">
+        <v>جارٍ بدء معالجة الذكاء الاصطناعي...</v>
+      </c>
+      <c r="C1521" t="str">
+        <v>Sāk AI apstrādi...</v>
+      </c>
+    </row>
+    <row r="1522">
+      <c r="A1522" t="str">
+        <v>Start AI Processing</v>
+      </c>
+      <c r="B1522" t="str">
+        <v>بدء معالجة الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1522" t="str">
+        <v>Sākt AI apstrādi</v>
+      </c>
+    </row>
+    <row r="1523">
+      <c r="A1523" t="str">
+        <v>Upload evidence files first</v>
+      </c>
+      <c r="B1523" t="str">
+        <v>ارفع ملفات الأدلة أولاً</v>
+      </c>
+      <c r="C1523" t="str">
+        <v>Vispirms augšupielādējiet pierādījumu failus</v>
+      </c>
+    </row>
+    <row r="1524">
+      <c r="A1524" t="str">
+        <v>AI is processing your evidence files. This may take a few minutes...</v>
+      </c>
+      <c r="B1524" t="str">
+        <v>يقوم الذكاء الاصطناعي بمعالجة ملفات الأدلة الخاصة بك. قد يستغرق هذا بضع دقائق...</v>
+      </c>
+      <c r="C1524" t="str">
+        <v>AI apstrādā jūsu pierādījumu failus. Tas var aizņemt dažas minūtes...</v>
+      </c>
+    </row>
+    <row r="1525">
+      <c r="A1525" t="str">
+        <v>AI processing failed:</v>
+      </c>
+      <c r="B1525" t="str">
+        <v>فشلت معالجة الذكاء الاصطناعي:</v>
+      </c>
+      <c r="C1525" t="str">
+        <v>AI apstrāde neizdevās:</v>
+      </c>
+    </row>
+    <row r="1526">
+      <c r="A1526" t="str">
+        <v>AI review completed</v>
+      </c>
+      <c r="B1526" t="str">
+        <v>اكتملت مراجعة الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1526" t="str">
+        <v>AI pārskatīšana pabeigta</v>
+      </c>
+    </row>
+    <row r="1527">
+      <c r="A1527" t="str">
+        <v>AI review in progress...</v>
+      </c>
+      <c r="B1527" t="str">
+        <v>مراجعة الذكاء الاصطناعي جارية...</v>
+      </c>
+      <c r="C1527" t="str">
+        <v>AI pārskatīšana norit...</v>
+      </c>
+    </row>
+    <row r="1528">
+      <c r="A1528" t="str">
+        <v>Evidence processed and ready for AI review</v>
+      </c>
+      <c r="B1528" t="str">
+        <v>تمت معالجة الأدلة وهي جاهزة لمراجعة الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1528" t="str">
+        <v>Pierādījumi apstrādāti un gatavi AI pārskatīšanai</v>
+      </c>
+    </row>
+    <row r="1529">
+      <c r="A1529" t="str">
+        <v>AI Review Results</v>
+      </c>
+      <c r="B1529" t="str">
+        <v>نتائج مراجعة الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1529" t="str">
+        <v>AI pārskatīšanas rezultāti</v>
+      </c>
+    </row>
+    <row r="1530">
+      <c r="A1530" t="str">
+        <v>Compliance Score</v>
+      </c>
+      <c r="B1530" t="str">
+        <v>درجة الامتثال</v>
+      </c>
+      <c r="C1530" t="str">
+        <v>Atbilstības vērtējums</v>
+      </c>
+    </row>
+    <row r="1531">
+      <c r="A1531" t="str">
+        <v>AI Analysis</v>
+      </c>
+      <c r="B1531" t="str">
+        <v>تحليل الذكاء الاصطناعي</v>
+      </c>
+      <c r="C1531" t="str">
+        <v>AI analīze</v>
+      </c>
+    </row>
+    <row r="1532">
+      <c r="A1532" t="str">
+        <v>Identified Issues</v>
+      </c>
+      <c r="B1532" t="str">
+        <v>المشكلات المحددة</v>
+      </c>
+      <c r="C1532" t="str">
+        <v>Identificētās problēmas</v>
+      </c>
+    </row>
+    <row r="1533">
+      <c r="A1533" t="str">
+        <v>Severity</v>
+      </c>
+      <c r="B1533" t="str">
+        <v>الخطورة</v>
+      </c>
+      <c r="C1533" t="str">
+        <v>Smagums</v>
+      </c>
+    </row>
+    <row r="1534">
+      <c r="A1534" t="str">
+        <v>Control Assessment Details</v>
+      </c>
+      <c r="B1534" t="str">
+        <v>تفاصيل تقييم الضوابط</v>
+      </c>
+      <c r="C1534" t="str">
+        <v>Kontroles novērtējuma detaļas</v>
+      </c>
+    </row>
+    <row r="1535">
+      <c r="A1535" t="str">
+        <v>Control</v>
+      </c>
+      <c r="B1535" t="str">
+        <v>الضابطة</v>
+      </c>
+      <c r="C1535" t="str">
+        <v>Kontrole</v>
+      </c>
+    </row>
+    <row r="1536">
+      <c r="A1536" t="str">
+        <v>Reviewed</v>
+      </c>
+      <c r="B1536" t="str">
+        <v>تمت المراجعة</v>
+      </c>
+      <c r="C1536" t="str">
+        <v>Pārskatīts</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C1403"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C1536"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add dynamic translation support to Risk Control Matrix pages
- List page: translate risk names via useTranslatedData hook, translate ratings/status with t()
- Detail page: translate risk name, description, category, department, owner, controls via useTranslatedRecord/useTranslatedData
- Add 48 missing translation keys for Risk Control Matrix UI labels

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2533"/>
+  <dimension ref="A1:C2580"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -28267,9 +28267,526 @@
         <v>Neizdevās izveidot</v>
       </c>
     </row>
+    <row r="2534">
+      <c r="A2534" t="str">
+        <v>Risk Code</v>
+      </c>
+      <c r="B2534" t="str">
+        <v>رمز المخاطر</v>
+      </c>
+      <c r="C2534" t="str">
+        <v>Riska kods</v>
+      </c>
+    </row>
+    <row r="2535">
+      <c r="A2535" t="str">
+        <v>Inherent</v>
+      </c>
+      <c r="B2535" t="str">
+        <v>الأصيل</v>
+      </c>
+      <c r="C2535" t="str">
+        <v>Sākotnējais</v>
+      </c>
+    </row>
+    <row r="2536">
+      <c r="A2536" t="str">
+        <v>Sync from Risks</v>
+      </c>
+      <c r="B2536" t="str">
+        <v>مزامنة من المخاطر</v>
+      </c>
+      <c r="C2536" t="str">
+        <v>Sinhronizēt no riskiem</v>
+      </c>
+    </row>
+    <row r="2537">
+      <c r="A2537" t="str">
+        <v>Search by risk code, name, or owner...</v>
+      </c>
+      <c r="B2537" t="str">
+        <v>البحث برمز المخاطر أو الاسم أو المالك...</v>
+      </c>
+      <c r="C2537" t="str">
+        <v>Meklēt pēc riska koda, nosaukuma vai īpašnieka...</v>
+      </c>
+    </row>
+    <row r="2538">
+      <c r="A2538" t="str">
+        <v>Delete All Matrix Entries?</v>
+      </c>
+      <c r="B2538" t="str">
+        <v>حذف جميع إدخالات المصفوفة؟</v>
+      </c>
+      <c r="C2538" t="str">
+        <v>Dzēst visus matricas ierakstus?</v>
+      </c>
+    </row>
+    <row r="2539">
+      <c r="A2539" t="str">
+        <v>entry(ies) from the Risk Control Matrix.</v>
+      </c>
+      <c r="B2539" t="str">
+        <v>إدخال(ات) من مصفوفة التحكم في المخاطر.</v>
+      </c>
+      <c r="C2539" t="str">
+        <v>ierakstu(-s) no Risku kontroles matricas.</v>
+      </c>
+    </row>
+    <row r="2540">
+      <c r="A2540" t="str">
+        <v>The underlying Risk records will NOT be deleted.</v>
+      </c>
+      <c r="B2540" t="str">
+        <v>لن يتم حذف سجلات المخاطر الأساسية.</v>
+      </c>
+      <c r="C2540" t="str">
+        <v>Pamata risku ieraksti NETIKS dzēsti.</v>
+      </c>
+    </row>
+    <row r="2541">
+      <c r="A2541" t="str">
+        <v>Delete Matrix Entry?</v>
+      </c>
+      <c r="B2541" t="str">
+        <v>حذف إدخال المصفوفة؟</v>
+      </c>
+      <c r="C2541" t="str">
+        <v>Dzēst matricas ierakstu?</v>
+      </c>
+    </row>
+    <row r="2542">
+      <c r="A2542" t="str">
+        <v>This will remove entry</v>
+      </c>
+      <c r="B2542" t="str">
+        <v>سيؤدي هذا إلى إزالة الإدخال</v>
+      </c>
+      <c r="C2542" t="str">
+        <v>Tas noņems ierakstu</v>
+      </c>
+    </row>
+    <row r="2543">
+      <c r="A2543" t="str">
+        <v>from the Risk Control Matrix.</v>
+      </c>
+      <c r="B2543" t="str">
+        <v>من مصفوفة التحكم في المخاطر.</v>
+      </c>
+      <c r="C2543" t="str">
+        <v>no Risku kontroles matricas.</v>
+      </c>
+    </row>
+    <row r="2544">
+      <c r="A2544" t="str">
+        <v>The underlying Risk record will NOT be deleted.</v>
+      </c>
+      <c r="B2544" t="str">
+        <v>لن يتم حذف سجل المخاطر الأساسي.</v>
+      </c>
+      <c r="C2544" t="str">
+        <v>Pamata riska ieraksts NETIKS dzēsts.</v>
+      </c>
+    </row>
+    <row r="2545">
+      <c r="A2545" t="str">
+        <v>This will remove all</v>
+      </c>
+      <c r="B2545" t="str">
+        <v>سيؤدي هذا إلى إزالة جميع</v>
+      </c>
+      <c r="C2545" t="str">
+        <v>Tas noņems visus</v>
+      </c>
+    </row>
+    <row r="2546">
+      <c r="A2546" t="str">
+        <v>Deleting...</v>
+      </c>
+      <c r="B2546" t="str">
+        <v>جاري الحذف...</v>
+      </c>
+      <c r="C2546" t="str">
+        <v>Dzēš...</v>
+      </c>
+    </row>
+    <row r="2547">
+      <c r="A2547" t="str">
+        <v>risks to the matrix.</v>
+      </c>
+      <c r="B2547" t="str">
+        <v>المخاطر إلى المصفوفة.</v>
+      </c>
+      <c r="C2547" t="str">
+        <v>riski matricā.</v>
+      </c>
+    </row>
+    <row r="2548">
+      <c r="A2548" t="str">
+        <v>already existed.</v>
+      </c>
+      <c r="B2548" t="str">
+        <v>موجودة بالفعل.</v>
+      </c>
+      <c r="C2548" t="str">
+        <v>jau pastāvēja.</v>
+      </c>
+    </row>
+    <row r="2549">
+      <c r="A2549" t="str">
+        <v>Import failed</v>
+      </c>
+      <c r="B2549" t="str">
+        <v>فشل الاستيراد</v>
+      </c>
+      <c r="C2549" t="str">
+        <v>Imports neizdevās</v>
+      </c>
+    </row>
+    <row r="2550">
+      <c r="A2550" t="str">
+        <v>Failed to import risks.</v>
+      </c>
+      <c r="B2550" t="str">
+        <v>فشل في استيراد المخاطر.</v>
+      </c>
+      <c r="C2550" t="str">
+        <v>Neizdevās importēt riskus.</v>
+      </c>
+    </row>
+    <row r="2551">
+      <c r="A2551" t="str">
+        <v>Failed to import risks to matrix.</v>
+      </c>
+      <c r="B2551" t="str">
+        <v>فشل في استيراد المخاطر إلى المصفوفة.</v>
+      </c>
+      <c r="C2551" t="str">
+        <v>Neizdevās importēt riskus matricā.</v>
+      </c>
+    </row>
+    <row r="2552">
+      <c r="A2552" t="str">
+        <v>Entry deleted</v>
+      </c>
+      <c r="B2552" t="str">
+        <v>تم حذف الإدخال</v>
+      </c>
+      <c r="C2552" t="str">
+        <v>Ieraksts dzēsts</v>
+      </c>
+    </row>
+    <row r="2553">
+      <c r="A2553" t="str">
+        <v>The matrix entry has been removed. The underlying risk is NOT affected.</v>
+      </c>
+      <c r="B2553" t="str">
+        <v>تمت إزالة إدخال المصفوفة. لن يتأثر سجل المخاطر الأساسي.</v>
+      </c>
+      <c r="C2553" t="str">
+        <v>Matricas ieraksts ir noņemts. Pamata risks NAV ietekmēts.</v>
+      </c>
+    </row>
+    <row r="2554">
+      <c r="A2554" t="str">
+        <v>Failed to delete matrix entry.</v>
+      </c>
+      <c r="B2554" t="str">
+        <v>فشل في حذف إدخال المصفوفة.</v>
+      </c>
+      <c r="C2554" t="str">
+        <v>Neizdevās dzēst matricas ierakstu.</v>
+      </c>
+    </row>
+    <row r="2555">
+      <c r="A2555" t="str">
+        <v>All entries deleted</v>
+      </c>
+      <c r="B2555" t="str">
+        <v>تم حذف جميع الإدخالات</v>
+      </c>
+      <c r="C2555" t="str">
+        <v>Visi ieraksti dzēsti</v>
+      </c>
+    </row>
+    <row r="2556">
+      <c r="A2556" t="str">
+        <v>All matrix entries have been removed. The underlying risks are NOT affected.</v>
+      </c>
+      <c r="B2556" t="str">
+        <v>تمت إزالة جميع إدخالات المصفوفة. لن تتأثر سجلات المخاطر الأساسية.</v>
+      </c>
+      <c r="C2556" t="str">
+        <v>Visi matricas ieraksti ir noņemti. Pamata riski NAV ietekmēti.</v>
+      </c>
+    </row>
+    <row r="2557">
+      <c r="A2557" t="str">
+        <v>Failed to delete matrix entries.</v>
+      </c>
+      <c r="B2557" t="str">
+        <v>فشل في حذف إدخالات المصفوفة.</v>
+      </c>
+      <c r="C2557" t="str">
+        <v>Neizdevās dzēst matricas ierakstus.</v>
+      </c>
+    </row>
+    <row r="2558">
+      <c r="A2558" t="str">
+        <v>No entries in the Risk Control Matrix</v>
+      </c>
+      <c r="B2558" t="str">
+        <v>لا توجد إدخالات في مصفوفة التحكم في المخاطر</v>
+      </c>
+      <c r="C2558" t="str">
+        <v>Nav ierakstu Risku kontroles matricā</v>
+      </c>
+    </row>
+    <row r="2559">
+      <c r="A2559" t="str">
+        <v>Import risks from the risk register to get started</v>
+      </c>
+      <c r="B2559" t="str">
+        <v>استيراد المخاطر من سجل المخاطر للبدء</v>
+      </c>
+      <c r="C2559" t="str">
+        <v>Importējiet riskus no risku reģistra, lai sāktu</v>
+      </c>
+    </row>
+    <row r="2560">
+      <c r="A2560" t="str">
+        <v>Link Control to Risk</v>
+      </c>
+      <c r="B2560" t="str">
+        <v>ربط الضابط بالمخاطر</v>
+      </c>
+      <c r="C2560" t="str">
+        <v>Saistīt kontroli ar risku</v>
+      </c>
+    </row>
+    <row r="2561">
+      <c r="A2561" t="str">
+        <v>Select a control</v>
+      </c>
+      <c r="B2561" t="str">
+        <v>اختر ضابطاً</v>
+      </c>
+      <c r="C2561" t="str">
+        <v>Izvēlieties kontroli</v>
+      </c>
+    </row>
+    <row r="2562">
+      <c r="A2562" t="str">
+        <v>No controls linked to this risk</v>
+      </c>
+      <c r="B2562" t="str">
+        <v>لا توجد ضوابط مرتبطة بهذا الخطر</v>
+      </c>
+      <c r="C2562" t="str">
+        <v>Ar šo risku nav saistītas kontroles</v>
+      </c>
+    </row>
+    <row r="2563">
+      <c r="A2563" t="str">
+        <v>Link controls to show how this risk is being mitigated</v>
+      </c>
+      <c r="B2563" t="str">
+        <v>ربط الضوابط لإظهار كيفية تخفيف هذا الخطر</v>
+      </c>
+      <c r="C2563" t="str">
+        <v>Saistiet kontroles, lai parādītu, kā šis risks tiek mazināts</v>
+      </c>
+    </row>
+    <row r="2564">
+      <c r="A2564" t="str">
+        <v>No residual risk assessment available</v>
+      </c>
+      <c r="B2564" t="str">
+        <v>لا يوجد تقييم للمخاطر المتبقية</v>
+      </c>
+      <c r="C2564" t="str">
+        <v>Nav pieejams atlikušā riska novērtējums</v>
+      </c>
+    </row>
+    <row r="2565">
+      <c r="A2565" t="str">
+        <v>Edit the risk to add residual risk values</v>
+      </c>
+      <c r="B2565" t="str">
+        <v>حرر المخاطر لإضافة قيم المخاطر المتبقية</v>
+      </c>
+      <c r="C2565" t="str">
+        <v>Rediģējiet risku, lai pievienotu atlikušā riska vērtības</v>
+      </c>
+    </row>
+    <row r="2566">
+      <c r="A2566" t="str">
+        <v>Matrix Position</v>
+      </c>
+      <c r="B2566" t="str">
+        <v>موقع المصفوفة</v>
+      </c>
+      <c r="C2566" t="str">
+        <v>Matricas pozīcija</v>
+      </c>
+    </row>
+    <row r="2567">
+      <c r="A2567" t="str">
+        <v>Mitigating Controls</v>
+      </c>
+      <c r="B2567" t="str">
+        <v>ضوابط التخفيف</v>
+      </c>
+      <c r="C2567" t="str">
+        <v>Mazinošās kontroles</v>
+      </c>
+    </row>
+    <row r="2568">
+      <c r="A2568" t="str">
+        <v>After applying controls/mitigations</v>
+      </c>
+      <c r="B2568" t="str">
+        <v>بعد تطبيق الضوابط/التخفيفات</v>
+      </c>
+      <c r="C2568" t="str">
+        <v>Pēc kontroļu/mazinājumu piemērošanas</v>
+      </c>
+    </row>
+    <row r="2569">
+      <c r="A2569" t="str">
+        <v>L x I</v>
+      </c>
+      <c r="B2569" t="str">
+        <v>الاحتمالية × التأثير</v>
+      </c>
+      <c r="C2569" t="str">
+        <v>V x I</v>
+      </c>
+    </row>
+    <row r="2570">
+      <c r="A2570" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="B2570" t="str">
+        <v>تم التحقق</v>
+      </c>
+      <c r="C2570" t="str">
+        <v>Verificēts</v>
+      </c>
+    </row>
+    <row r="2571">
+      <c r="A2571" t="str">
+        <v>Inherent Risk Assessment</v>
+      </c>
+      <c r="B2571" t="str">
+        <v>تقييم المخاطر الأصيلة</v>
+      </c>
+      <c r="C2571" t="str">
+        <v>Sākotnējā riska novērtējums</v>
+      </c>
+    </row>
+    <row r="2572">
+      <c r="A2572" t="str">
+        <v>Residual Risk Assessment</v>
+      </c>
+      <c r="B2572" t="str">
+        <v>تقييم المخاطر المتبقية</v>
+      </c>
+      <c r="C2572" t="str">
+        <v>Atlikušā riska novērtējums</v>
+      </c>
+    </row>
+    <row r="2573">
+      <c r="A2573" t="str">
+        <v>Residual Likelihood</v>
+      </c>
+      <c r="B2573" t="str">
+        <v>الاحتمالية المتبقية</v>
+      </c>
+      <c r="C2573" t="str">
+        <v>Atlikušā iespējamība</v>
+      </c>
+    </row>
+    <row r="2574">
+      <c r="A2574" t="str">
+        <v>Residual Impact</v>
+      </c>
+      <c r="B2574" t="str">
+        <v>التأثير المتبقي</v>
+      </c>
+      <c r="C2574" t="str">
+        <v>Atlikušā ietekme</v>
+      </c>
+    </row>
+    <row r="2575">
+      <c r="A2575" t="str">
+        <v>Other Details</v>
+      </c>
+      <c r="B2575" t="str">
+        <v>تفاصيل أخرى</v>
+      </c>
+      <c r="C2575" t="str">
+        <v>Cita informācija</v>
+      </c>
+    </row>
+    <row r="2576">
+      <c r="A2576" t="str">
+        <v>Mitigation Status</v>
+      </c>
+      <c r="B2576" t="str">
+        <v>حالة التخفيف</v>
+      </c>
+      <c r="C2576" t="str">
+        <v>Mazināšanas statuss</v>
+      </c>
+    </row>
+    <row r="2577">
+      <c r="A2577" t="str">
+        <v>Select likelihood</v>
+      </c>
+      <c r="B2577" t="str">
+        <v>اختر الاحتمالية</v>
+      </c>
+      <c r="C2577" t="str">
+        <v>Izvēlieties iespējamību</v>
+      </c>
+    </row>
+    <row r="2578">
+      <c r="A2578" t="str">
+        <v>Select impact</v>
+      </c>
+      <c r="B2578" t="str">
+        <v>اختر التأثير</v>
+      </c>
+      <c r="C2578" t="str">
+        <v>Izvēlieties ietekmi</v>
+      </c>
+    </row>
+    <row r="2579">
+      <c r="A2579" t="str">
+        <v>Select due date</v>
+      </c>
+      <c r="B2579" t="str">
+        <v>اختر تاريخ الاستحقاق</v>
+      </c>
+      <c r="C2579" t="str">
+        <v>Izvēlieties izpildes datumu</v>
+      </c>
+    </row>
+    <row r="2580">
+      <c r="A2580" t="str">
+        <v>Implemented</v>
+      </c>
+      <c r="B2580" t="str">
+        <v>مُنفَّذ</v>
+      </c>
+      <c r="C2580" t="str">
+        <v>Ieviests</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2533"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C2580"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add auto-detect source language and 42 missing BIA/BCP translations
- Add detectSourceLocale() to translation-service.ts that auto-detects
  Arabic/Latvian/English from text content using Unicode character ranges
- translateRecord() now auto-detects source language when sourceLocale
  is not explicitly provided, enabling reverse translation (Arabic→English,
  Latvian→English) without modifying any of the 40+ API route callers
- Add 42 missing static translations to i18n/translations.xlsx for BIA
  Categories, BIA Methodology, BCP Labels, and Process pages
- Fix translate API endpoint to use auto-detection as fallback

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,12 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3136"/>
-  <cols>
-    <col min="1" max="1" width="60.83203125" customWidth="1"/>
-    <col min="2" max="2" width="60.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:C3178"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -34900,9 +34895,471 @@
         <v>risks(-i)</v>
       </c>
     </row>
+    <row r="3137">
+      <c r="A3137" t="str">
+        <v>Toggle Columns</v>
+      </c>
+      <c r="B3137" t="str">
+        <v>تبديل الأعمدة</v>
+      </c>
+      <c r="C3137" t="str">
+        <v>Pārslēgt kolonnas</v>
+      </c>
+    </row>
+    <row r="3138">
+      <c r="A3138" t="str">
+        <v>No Data</v>
+      </c>
+      <c r="B3138" t="str">
+        <v>لا توجد بيانات</v>
+      </c>
+      <c r="C3138" t="str">
+        <v>Nav datu</v>
+      </c>
+    </row>
+    <row r="3139">
+      <c r="A3139" t="str">
+        <v>RTO</v>
+      </c>
+      <c r="B3139" t="str">
+        <v>RTO</v>
+      </c>
+      <c r="C3139" t="str">
+        <v>RTO</v>
+      </c>
+    </row>
+    <row r="3140">
+      <c r="A3140" t="str">
+        <v>RPO</v>
+      </c>
+      <c r="B3140" t="str">
+        <v>RPO</v>
+      </c>
+      <c r="C3140" t="str">
+        <v>RPO</v>
+      </c>
+    </row>
+    <row r="3141">
+      <c r="A3141" t="str">
+        <v>Match with Library</v>
+      </c>
+      <c r="B3141" t="str">
+        <v>مطابقة مع المكتبة</v>
+      </c>
+      <c r="C3141" t="str">
+        <v>Saskaņot ar bibliotēku</v>
+      </c>
+    </row>
+    <row r="3142">
+      <c r="A3142" t="str">
+        <v>Choose File</v>
+      </c>
+      <c r="B3142" t="str">
+        <v>اختر ملف</v>
+      </c>
+      <c r="C3142" t="str">
+        <v>Izvēlēties failu</v>
+      </c>
+    </row>
+    <row r="3143">
+      <c r="A3143" t="str">
+        <v>No file chosen</v>
+      </c>
+      <c r="B3143" t="str">
+        <v>لم يتم اختيار ملف</v>
+      </c>
+      <c r="C3143" t="str">
+        <v>Nav izvēlēts fails</v>
+      </c>
+    </row>
+    <row r="3144">
+      <c r="A3144" t="str">
+        <v>Select Department First</v>
+      </c>
+      <c r="B3144" t="str">
+        <v>اختر القسم أولاً</v>
+      </c>
+      <c r="C3144" t="str">
+        <v>Vispirms atlasiet nodaļu</v>
+      </c>
+    </row>
+    <row r="3145">
+      <c r="A3145" t="str">
+        <v>Enable KPI Measurement Required when adding a process to see it here</v>
+      </c>
+      <c r="B3145" t="str">
+        <v>قم بتمكين خيار قياس مؤشرات الأداء عند إضافة عملية لرؤيتها هنا</v>
+      </c>
+      <c r="C3145" t="str">
+        <v>Iespējojiet KPI mērīšanu, pievienojot procesu, lai to redzētu šeit</v>
+      </c>
+    </row>
+    <row r="3146">
+      <c r="A3146" t="str">
+        <v>BIA Categories</v>
+      </c>
+      <c r="B3146" t="str">
+        <v>فئات تحليل تأثير الأعمال</v>
+      </c>
+      <c r="C3146" t="str">
+        <v>BIA kategorijas</v>
+      </c>
+    </row>
+    <row r="3147">
+      <c r="A3147" t="str">
+        <v>Add Category</v>
+      </c>
+      <c r="B3147" t="str">
+        <v>إضافة فئة</v>
+      </c>
+      <c r="C3147" t="str">
+        <v>Pievienot kategoriju</v>
+      </c>
+    </row>
+    <row r="3148">
+      <c r="A3148" t="str">
+        <v>Add BIA Category</v>
+      </c>
+      <c r="B3148" t="str">
+        <v>إضافة فئة تحليل تأثير الأعمال</v>
+      </c>
+      <c r="C3148" t="str">
+        <v>Pievienot BIA kategoriju</v>
+      </c>
+    </row>
+    <row r="3149">
+      <c r="A3149" t="str">
+        <v>Edit BIA Category</v>
+      </c>
+      <c r="B3149" t="str">
+        <v>تعديل فئة تحليل تأثير الأعمال</v>
+      </c>
+      <c r="C3149" t="str">
+        <v>Rediģēt BIA kategoriju</v>
+      </c>
+    </row>
+    <row r="3150">
+      <c r="A3150" t="str">
+        <v>Sort Order</v>
+      </c>
+      <c r="B3150" t="str">
+        <v>ترتيب الفرز</v>
+      </c>
+      <c r="C3150" t="str">
+        <v>Kārtošanas secība</v>
+      </c>
+    </row>
+    <row r="3151">
+      <c r="A3151" t="str">
+        <v>e.g., Financial, Reputational</v>
+      </c>
+      <c r="B3151" t="str">
+        <v>مثال: مالي، سمعة</v>
+      </c>
+      <c r="C3151" t="str">
+        <v>piem., Finanšu, Reputācijas</v>
+      </c>
+    </row>
+    <row r="3152">
+      <c r="A3152" t="str">
+        <v>Are you sure you want to delete this category? This action cannot be undone.</v>
+      </c>
+      <c r="B3152" t="str">
+        <v>هل أنت متأكد أنك تريد حذف هذه الفئة؟ لا يمكن التراجع عن هذا الإجراء.</v>
+      </c>
+      <c r="C3152" t="str">
+        <v>Vai tiešām vēlaties dzēst šo kategoriju? Šo darbību nevar atsaukt.</v>
+      </c>
+    </row>
+    <row r="3153">
+      <c r="A3153" t="str">
+        <v>Add a new impact category for Business Impact Analysis</v>
+      </c>
+      <c r="B3153" t="str">
+        <v>إضافة فئة تأثير جديدة لتحليل تأثير الأعمال</v>
+      </c>
+      <c r="C3153" t="str">
+        <v>Pievienojiet jaunu ietekmes kategoriju biznesa ietekmes analīzei</v>
+      </c>
+    </row>
+    <row r="3154">
+      <c r="A3154" t="str">
+        <v>Rating Label</v>
+      </c>
+      <c r="B3154" t="str">
+        <v>تسمية التقييم</v>
+      </c>
+      <c r="C3154" t="str">
+        <v>Novērtējuma etiķete</v>
+      </c>
+    </row>
+    <row r="3155">
+      <c r="A3155" t="str">
+        <v>Score Value</v>
+      </c>
+      <c r="B3155" t="str">
+        <v>قيمة النقاط</v>
+      </c>
+      <c r="C3155" t="str">
+        <v>Punktu vērtība</v>
+      </c>
+    </row>
+    <row r="3156">
+      <c r="A3156" t="str">
+        <v>Criticality Label</v>
+      </c>
+      <c r="B3156" t="str">
+        <v>تسمية الخطورة</v>
+      </c>
+      <c r="C3156" t="str">
+        <v>Kritiskuma etiķete</v>
+      </c>
+    </row>
+    <row r="3157">
+      <c r="A3157" t="str">
+        <v>Criticality Ranges</v>
+      </c>
+      <c r="B3157" t="str">
+        <v>نطاقات مستويات الخطورة</v>
+      </c>
+      <c r="C3157" t="str">
+        <v>Kritiskuma diapazoni</v>
+      </c>
+    </row>
+    <row r="3158">
+      <c r="A3158" t="str">
+        <v>Rating Methodology</v>
+      </c>
+      <c r="B3158" t="str">
+        <v>منهجية التقييم</v>
+      </c>
+      <c r="C3158" t="str">
+        <v>Novērtējuma metodika</v>
+      </c>
+    </row>
+    <row r="3159">
+      <c r="A3159" t="str">
+        <v>High of all (Maximum)</v>
+      </c>
+      <c r="B3159" t="str">
+        <v>الأعلى من الكل (الحد الأقصى)</v>
+      </c>
+      <c r="C3159" t="str">
+        <v>Augstākais no visiem (Maksimums)</v>
+      </c>
+    </row>
+    <row r="3160">
+      <c r="A3160" t="str">
+        <v>Addition of all (Sum)</v>
+      </c>
+      <c r="B3160" t="str">
+        <v>جمع الكل (المجموع)</v>
+      </c>
+      <c r="C3160" t="str">
+        <v>Visu pievienošana (Summa)</v>
+      </c>
+    </row>
+    <row r="3161">
+      <c r="A3161" t="str">
+        <v>Product of all (Multiply)</v>
+      </c>
+      <c r="B3161" t="str">
+        <v>حاصل ضرب الكل (الضرب)</v>
+      </c>
+      <c r="C3161" t="str">
+        <v>Visu reizinājums (Reizinājums)</v>
+      </c>
+    </row>
+    <row r="3162">
+      <c r="A3162" t="str">
+        <v>Add Rating</v>
+      </c>
+      <c r="B3162" t="str">
+        <v>إضافة تقييم</v>
+      </c>
+      <c r="C3162" t="str">
+        <v>Pievienot novērtējumu</v>
+      </c>
+    </row>
+    <row r="3163">
+      <c r="A3163" t="str">
+        <v>Add Range</v>
+      </c>
+      <c r="B3163" t="str">
+        <v>إضافة نطاق</v>
+      </c>
+      <c r="C3163" t="str">
+        <v>Pievienot diapazonu</v>
+      </c>
+    </row>
+    <row r="3164">
+      <c r="A3164" t="str">
+        <v>No limit</v>
+      </c>
+      <c r="B3164" t="str">
+        <v>بدون حد</v>
+      </c>
+      <c r="C3164" t="str">
+        <v>Bez ierobežojuma</v>
+      </c>
+    </row>
+    <row r="3165">
+      <c r="A3165" t="str">
+        <v>overlaps with</v>
+      </c>
+      <c r="B3165" t="str">
+        <v>يتداخل مع</v>
+      </c>
+      <c r="C3165" t="str">
+        <v>pārklājas ar</v>
+      </c>
+    </row>
+    <row r="3166">
+      <c r="A3166" t="str">
+        <v>Define a criticality level based on score range</v>
+      </c>
+      <c r="B3166" t="str">
+        <v>تحديد مستوى خطورة بناءً على نطاق النقاط</v>
+      </c>
+      <c r="C3166" t="str">
+        <v>Definējiet kritiskuma līmeni, pamatojoties uz punktu diapazonu</v>
+      </c>
+    </row>
+    <row r="3167">
+      <c r="A3167" t="str">
+        <v>Configure how the BIA impact rating is calculated from individual category scores</v>
+      </c>
+      <c r="B3167" t="str">
+        <v>تكوين كيفية حساب تقييم تأثير تحليل الأعمال من درجات الفئات الفردية</v>
+      </c>
+      <c r="C3167" t="str">
+        <v>Konfigurējiet, kā BIA ietekmes vērtējums tiek aprēķināts no atsevišķo kategoriju rādītājiem</v>
+      </c>
+    </row>
+    <row r="3168">
+      <c r="A3168" t="str">
+        <v>Define score ranges to determine process criticality levels</v>
+      </c>
+      <c r="B3168" t="str">
+        <v>تحديد نطاقات النقاط لتحديد مستويات خطورة العملية</v>
+      </c>
+      <c r="C3168" t="str">
+        <v>Definējiet punktu diapazonus, lai noteiktu procesa kritiskuma līmeņus</v>
+      </c>
+    </row>
+    <row r="3169">
+      <c r="A3169" t="str">
+        <v>Recovery Time Objective (RTO)</v>
+      </c>
+      <c r="B3169" t="str">
+        <v>الوقت المستهدف للاسترجاع (RTO)</v>
+      </c>
+      <c r="C3169" t="str">
+        <v>Atveseļošanas laika mērķis (RTO)</v>
+      </c>
+    </row>
+    <row r="3170">
+      <c r="A3170" t="str">
+        <v>Recovery Point Objective (RPO)</v>
+      </c>
+      <c r="B3170" t="str">
+        <v>نقطة استرجاع البيانات المستهدفة (RPO)</v>
+      </c>
+      <c r="C3170" t="str">
+        <v>Datu atveseļošanas punkta mērķis (RPO)</v>
+      </c>
+    </row>
+    <row r="3171">
+      <c r="A3171" t="str">
+        <v>RTO Labels</v>
+      </c>
+      <c r="B3171" t="str">
+        <v>تسميات الوقت المستهدف للاسترجاع</v>
+      </c>
+      <c r="C3171" t="str">
+        <v>RTO etiķetes</v>
+      </c>
+    </row>
+    <row r="3172">
+      <c r="A3172" t="str">
+        <v>RPO Labels</v>
+      </c>
+      <c r="B3172" t="str">
+        <v>تسميات نقطة استرجاع البيانات</v>
+      </c>
+      <c r="C3172" t="str">
+        <v>RPO etiķetes</v>
+      </c>
+    </row>
+    <row r="3173">
+      <c r="A3173" t="str">
+        <v>Add RTO Label</v>
+      </c>
+      <c r="B3173" t="str">
+        <v>إضافة تسمية الوقت المستهدف للاسترجاع</v>
+      </c>
+      <c r="C3173" t="str">
+        <v>Pievienot RTO etiķeti</v>
+      </c>
+    </row>
+    <row r="3174">
+      <c r="A3174" t="str">
+        <v>Add RPO Label</v>
+      </c>
+      <c r="B3174" t="str">
+        <v>إضافة تسمية نقطة استرجاع البيانات</v>
+      </c>
+      <c r="C3174" t="str">
+        <v>Pievienot RPO etiķeti</v>
+      </c>
+    </row>
+    <row r="3175">
+      <c r="A3175" t="str">
+        <v>RTO defines the maximum acceptable time to restore a process after a disruption. Configure labels to standardize RTO options across your organization.</v>
+      </c>
+      <c r="B3175" t="str">
+        <v>يحدد الوقت المستهدف للاسترجاع الحد الأقصى للوقت المقبول لاستعادة العملية بعد الانقطاع. قم بتكوين التسميات لتوحيد خيارات الوقت المستهدف للاسترجاع في جميع أنحاء مؤسستك.</v>
+      </c>
+      <c r="C3175" t="str">
+        <v>RTO definē maksimālo pieņemamo laiku procesa atjaunošanai pēc pārtraukuma. Konfigurējiet etiķetes, lai standartizētu RTO opcijas visā jūsu organizācijā.</v>
+      </c>
+    </row>
+    <row r="3176">
+      <c r="A3176" t="str">
+        <v>RPO defines the maximum acceptable data loss measured in time. Configure labels to standardize RPO options across your organization.</v>
+      </c>
+      <c r="B3176" t="str">
+        <v>تحدد نقطة استرجاع البيانات أقصى فقدان مقبول للبيانات يُقاس بالوقت. قم بتكوين التسميات لتوحيد خيارات نقطة استرجاع البيانات في جميع أنحاء مؤسستك.</v>
+      </c>
+      <c r="C3176" t="str">
+        <v>RPO definē maksimāli pieņemamo datu zudumu, ko mēra laikā. Konfigurējiet etiķetes, lai standartizētu RPO opcijas visā jūsu organizācijā.</v>
+      </c>
+    </row>
+    <row r="3177">
+      <c r="A3177" t="str">
+        <v>Email notifications enabled</v>
+      </c>
+      <c r="B3177" t="str">
+        <v>تم تفعيل إشعارات البريد الإلكتروني</v>
+      </c>
+      <c r="C3177" t="str">
+        <v>E-pasta paziņojumi iespējoti</v>
+      </c>
+    </row>
+    <row r="3178">
+      <c r="A3178" t="str">
+        <v>Email notifications disabled</v>
+      </c>
+      <c r="B3178" t="str">
+        <v>تم تعطيل إشعارات البريد الإلكتروني</v>
+      </c>
+      <c r="C3178" t="str">
+        <v>E-pasta paziņojumi atspējoti</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C3136"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3178"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix dynamic translations: prevent fallback storage, add missing fields, improve frontend overlays
- Prevent storing translations identical to source text when backend is down
- Filter out bad translations via sourceHash comparison in bulk/single endpoints
- Add missing translation fields: Service (serviceCategory, serviceItem), Regulation (version), Issue (domain, category), User (firstName, lastName, designation)
- Fix Users page: translate department names, reporting managers in all views/dropdowns/CSV
- Fix Context page: translate department names in issue/stakeholder display and CSV export
- Fix Organization profile: translate service categories and regulation versions
- Add auto-translate on fetch for single-record endpoint with retry
- Update translation hooks to remove English early-return, add retry for pending translations
- Add new static translations to Excel for Organization module pages

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3178"/>
+  <dimension ref="A1:C3189"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -35357,9 +35357,130 @@
         <v>E-pasta paziņojumi atspējoti</v>
       </c>
     </row>
+    <row r="3179">
+      <c r="A3179" t="str">
+        <v>BIA submitted for approval</v>
+      </c>
+      <c r="B3179" t="str">
+        <v>تم تقديم تحليل أثر الأعمال للموافقة</v>
+      </c>
+      <c r="C3179" t="str">
+        <v>BIA iesniegts apstiprināšanai</v>
+      </c>
+    </row>
+    <row r="3180">
+      <c r="A3180" t="str">
+        <v>BIA approved</v>
+      </c>
+      <c r="B3180" t="str">
+        <v>تمت الموافقة على تحليل أثر الأعمال</v>
+      </c>
+      <c r="C3180" t="str">
+        <v>BIA apstiprināts</v>
+      </c>
+    </row>
+    <row r="3181">
+      <c r="A3181" t="str">
+        <v>Failed to create rating</v>
+      </c>
+      <c r="B3181" t="str">
+        <v>فشل في إنشاء التصنيف</v>
+      </c>
+      <c r="C3181" t="str">
+        <v>Neizdevās izveidot vērtējumu</v>
+      </c>
+    </row>
+    <row r="3182">
+      <c r="A3182" t="str">
+        <v>Failed to update rating</v>
+      </c>
+      <c r="B3182" t="str">
+        <v>فشل في تحديث التصنيف</v>
+      </c>
+      <c r="C3182" t="str">
+        <v>Neizdevās atjaunināt vērtējumu</v>
+      </c>
+    </row>
+    <row r="3183">
+      <c r="A3183" t="str">
+        <v>Failed to create range</v>
+      </c>
+      <c r="B3183" t="str">
+        <v>فشل في إنشاء النطاق</v>
+      </c>
+      <c r="C3183" t="str">
+        <v>Neizdevās izveidot diapazonu</v>
+      </c>
+    </row>
+    <row r="3184">
+      <c r="A3184" t="str">
+        <v>Failed to create range. Please try again.</v>
+      </c>
+      <c r="B3184" t="str">
+        <v>فشل في إنشاء النطاق. يرجى المحاولة مرة أخرى.</v>
+      </c>
+      <c r="C3184" t="str">
+        <v>Neizdevās izveidot diapazonu. Lūdzu, mēģiniet vēlreiz.</v>
+      </c>
+    </row>
+    <row r="3185">
+      <c r="A3185" t="str">
+        <v>Failed to update range</v>
+      </c>
+      <c r="B3185" t="str">
+        <v>فشل في تحديث النطاق</v>
+      </c>
+      <c r="C3185" t="str">
+        <v>Neizdevās atjaunināt diapazonu</v>
+      </c>
+    </row>
+    <row r="3186">
+      <c r="A3186" t="str">
+        <v>Failed to update range. Please try again.</v>
+      </c>
+      <c r="B3186" t="str">
+        <v>فشل في تحديث النطاق. يرجى المحاولة مرة أخرى.</v>
+      </c>
+      <c r="C3186" t="str">
+        <v>Neizdevās atjaunināt diapazonu. Lūdzu, mēģiniet vēlreiz.</v>
+      </c>
+    </row>
+    <row r="3187">
+      <c r="A3187" t="str">
+        <v>Failed to create label</v>
+      </c>
+      <c r="B3187" t="str">
+        <v>فشل في إنشاء التسمية</v>
+      </c>
+      <c r="C3187" t="str">
+        <v>Neizdevās izveidot etiķeti</v>
+      </c>
+    </row>
+    <row r="3188">
+      <c r="A3188" t="str">
+        <v>Failed to update label</v>
+      </c>
+      <c r="B3188" t="str">
+        <v>فشل في تحديث التسمية</v>
+      </c>
+      <c r="C3188" t="str">
+        <v>Neizdevās atjaunināt etiķeti</v>
+      </c>
+    </row>
+    <row r="3189">
+      <c r="A3189" t="str">
+        <v>Select Process Type</v>
+      </c>
+      <c r="B3189" t="str">
+        <v>اختر نوع العملية</v>
+      </c>
+      <c r="C3189" t="str">
+        <v>Izvēlieties procesa veidu</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C3178"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3189"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Translate header topbar: user name, role, date/time with locale support
- Translate user display name using useTranslatedRecord hook
- Translate role names (Customer Administrator, Audit Head, etc.) with t()
- Use date-fns locale for Arabic/Latvian month names and AM/PM
- Add 7 role name translations to Excel and locale files

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3189"/>
+  <dimension ref="A1:C3196"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -35478,9 +35478,86 @@
         <v>Izvēlieties procesa veidu</v>
       </c>
     </row>
+    <row r="3190">
+      <c r="A3190" t="str">
+        <v>G R C Administrator</v>
+      </c>
+      <c r="B3190" t="str">
+        <v>مسؤول GRC</v>
+      </c>
+      <c r="C3190" t="str">
+        <v>GRC administrators</v>
+      </c>
+    </row>
+    <row r="3191">
+      <c r="A3191" t="str">
+        <v>Customer Administrator</v>
+      </c>
+      <c r="B3191" t="str">
+        <v>مسؤول العميل</v>
+      </c>
+      <c r="C3191" t="str">
+        <v>Klienta administrators</v>
+      </c>
+    </row>
+    <row r="3192">
+      <c r="A3192" t="str">
+        <v>Audit Manager</v>
+      </c>
+      <c r="B3192" t="str">
+        <v>مدير التدقيق</v>
+      </c>
+      <c r="C3192" t="str">
+        <v>Audita menedžeris</v>
+      </c>
+    </row>
+    <row r="3193">
+      <c r="A3193" t="str">
+        <v>Reviewer</v>
+      </c>
+      <c r="B3193" t="str">
+        <v>مراجع</v>
+      </c>
+      <c r="C3193" t="str">
+        <v>Pārskatītājs</v>
+      </c>
+    </row>
+    <row r="3194">
+      <c r="A3194" t="str">
+        <v>Contributor</v>
+      </c>
+      <c r="B3194" t="str">
+        <v>مساهم</v>
+      </c>
+      <c r="C3194" t="str">
+        <v>Līdzstrādnieks</v>
+      </c>
+    </row>
+    <row r="3195">
+      <c r="A3195" t="str">
+        <v>Department Reviewer</v>
+      </c>
+      <c r="B3195" t="str">
+        <v>مراجع القسم</v>
+      </c>
+      <c r="C3195" t="str">
+        <v>Nodaļas pārskatītājs</v>
+      </c>
+    </row>
+    <row r="3196">
+      <c r="A3196" t="str">
+        <v>Department Contributor</v>
+      </c>
+      <c r="B3196" t="str">
+        <v>مساهم القسم</v>
+      </c>
+      <c r="C3196" t="str">
+        <v>Nodaļas līdzstrādnieks</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C3189"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3196"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Help Chatbot with knowledge base, search engine, and audit scope isolation
- 73 Q&A articles covering General, Organization, Compliance, Risk, Asset, Internal Audit, TPRM, and GRC Admin modules
- Client-side keyword/fuzzy search engine with multi-strategy scoring (exact, token overlap, keyword, Levenshtein)
- Product scope separation: GRC, TPRM, Audit, Both - ensures audit-only users see only Internal Audit content
- Role-based article filtering and context-aware page suggestions
- RTL-aware Sheet panel with module browsing, chat interface, and F1 keyboard shortcut
- Implementation guide document for future AI Assistant/Agent roadmap
- Fix TPRM dashboard Recharts Tooltip type errors

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3891"/>
+  <dimension ref="A1:C3908"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="60.83203125" customWidth="1"/>
@@ -43205,9 +43205,196 @@
         <v>gads</v>
       </c>
     </row>
+    <row r="3892">
+      <c r="A3892" t="str">
+        <v>Help Assistant</v>
+      </c>
+      <c r="B3892" t="str">
+        <v>مساعد المساعدة</v>
+      </c>
+      <c r="C3892" t="str">
+        <v>Palīdzības asistents</v>
+      </c>
+    </row>
+    <row r="3893">
+      <c r="A3893" t="str">
+        <v>Need help?</v>
+      </c>
+      <c r="B3893" t="str">
+        <v>هل تحتاج مساعدة؟</v>
+      </c>
+      <c r="C3893" t="str">
+        <v>Vajadzīga palīdzība?</v>
+      </c>
+    </row>
+    <row r="3894">
+      <c r="A3894" t="str">
+        <v>Ask anything about the application</v>
+      </c>
+      <c r="B3894" t="str">
+        <v>اسأل أي شيء عن التطبيق</v>
+      </c>
+      <c r="C3894" t="str">
+        <v>Jautājiet jebko par lietojumprogrammu</v>
+      </c>
+    </row>
+    <row r="3895">
+      <c r="A3895" t="str">
+        <v>Type your question...</v>
+      </c>
+      <c r="B3895" t="str">
+        <v>اكتب سؤالك...</v>
+      </c>
+      <c r="C3895" t="str">
+        <v>Ierakstiet savu jautājumu...</v>
+      </c>
+    </row>
+    <row r="3896">
+      <c r="A3896" t="str">
+        <v>Clear chat</v>
+      </c>
+      <c r="B3896" t="str">
+        <v>مسح المحادثة</v>
+      </c>
+      <c r="C3896" t="str">
+        <v>Notīrīt sarunu</v>
+      </c>
+    </row>
+    <row r="3897">
+      <c r="A3897" t="str">
+        <v>Browse by Module</v>
+      </c>
+      <c r="B3897" t="str">
+        <v>تصفح حسب الوحدة</v>
+      </c>
+      <c r="C3897" t="str">
+        <v>Pārlūkot pēc moduļa</v>
+      </c>
+    </row>
+    <row r="3898">
+      <c r="A3898" t="str">
+        <v>Suggested for this page</v>
+      </c>
+      <c r="B3898" t="str">
+        <v>مقترح لهذه الصفحة</v>
+      </c>
+      <c r="C3898" t="str">
+        <v>Ieteikts šai lapai</v>
+      </c>
+    </row>
+    <row r="3899">
+      <c r="A3899" t="str">
+        <v>topics</v>
+      </c>
+      <c r="B3899" t="str">
+        <v>مواضيع</v>
+      </c>
+      <c r="C3899" t="str">
+        <v>tēmas</v>
+      </c>
+    </row>
+    <row r="3900">
+      <c r="A3900" t="str">
+        <v>Back to modules</v>
+      </c>
+      <c r="B3900" t="str">
+        <v>العودة للوحدات</v>
+      </c>
+      <c r="C3900" t="str">
+        <v>Atpakaļ uz moduļiem</v>
+      </c>
+    </row>
+    <row r="3901">
+      <c r="A3901" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="B3901" t="str">
+        <v>ملاحظات</v>
+      </c>
+      <c r="C3901" t="str">
+        <v>Piezīmes</v>
+      </c>
+    </row>
+    <row r="3902">
+      <c r="A3902" t="str">
+        <v>Related</v>
+      </c>
+      <c r="B3902" t="str">
+        <v>ذو صلة</v>
+      </c>
+      <c r="C3902" t="str">
+        <v>Saistītais</v>
+      </c>
+    </row>
+    <row r="3903">
+      <c r="A3903" t="str">
+        <v>Related Questions</v>
+      </c>
+      <c r="B3903" t="str">
+        <v>أسئلة ذات صلة</v>
+      </c>
+      <c r="C3903" t="str">
+        <v>Saistītie jautājumi</v>
+      </c>
+    </row>
+    <row r="3904">
+      <c r="A3904" t="str">
+        <v>Press</v>
+      </c>
+      <c r="B3904" t="str">
+        <v>اضغط</v>
+      </c>
+      <c r="C3904" t="str">
+        <v>Nospiediet</v>
+      </c>
+    </row>
+    <row r="3905">
+      <c r="A3905" t="str">
+        <v>to toggle help</v>
+      </c>
+      <c r="B3905" t="str">
+        <v>لفتح/إغلاق المساعدة</v>
+      </c>
+      <c r="C3905" t="str">
+        <v>lai pārslēgtu palīdzību</v>
+      </c>
+    </row>
+    <row r="3906">
+      <c r="A3906" t="str">
+        <v>General</v>
+      </c>
+      <c r="B3906" t="str">
+        <v>عام</v>
+      </c>
+      <c r="C3906" t="str">
+        <v>Vispārīgi</v>
+      </c>
+    </row>
+    <row r="3907">
+      <c r="A3907" t="str">
+        <v>TPRM</v>
+      </c>
+      <c r="B3907" t="str">
+        <v>إدارة مخاطر الطرف الثالث</v>
+      </c>
+      <c r="C3907" t="str">
+        <v>TPRM</v>
+      </c>
+    </row>
+    <row r="3908">
+      <c r="A3908" t="str">
+        <v>GRC Administration</v>
+      </c>
+      <c r="B3908" t="str">
+        <v>إدارة الحوكمة والمخاطر والامتثال</v>
+      </c>
+      <c r="C3908" t="str">
+        <v>GRC administrēšana</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C3891"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3908"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add vendor export/import with onboarding answer persistence across all TPRM pages
- Add 4 vendor management API routes: export-template, import-vendors, export-questions, import-questions
- Add onboardingAnswers field to TPRMVendor schema for persisting question responses
- Save onboarding answers on vendor create/edit in BO inventory, RM inventory, and monitoring pages
- Load existing answers when editing a vendor
- Populate stored answers in vendor risk rating questions export
- Display onboarding answers on vendor detail page
- Add Export/Import dropdown to vendor management page (CustomerAdministrator only)
- Add i18n translations for new UI strings

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,12 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4446"/>
-  <cols>
-    <col min="1" max="1" width="60.83203125" customWidth="1"/>
-    <col min="2" max="2" width="60.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:C4460"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -49310,9 +49305,163 @@
         <v>Izvēlnes</v>
       </c>
     </row>
+    <row r="4447">
+      <c r="A4447" t="str">
+        <v>Export/Import</v>
+      </c>
+      <c r="B4447" t="str">
+        <v>تصدير/استيراد</v>
+      </c>
+      <c r="C4447" t="str">
+        <v>Eksportēt/Importēt</v>
+      </c>
+    </row>
+    <row r="4448">
+      <c r="A4448" t="str">
+        <v>Download Vendor Profile Template</v>
+      </c>
+      <c r="B4448" t="str">
+        <v>تحميل نموذج ملف المورد</v>
+      </c>
+      <c r="C4448" t="str">
+        <v>Lejupielādēt piegādātāja profila veidni</v>
+      </c>
+    </row>
+    <row r="4449">
+      <c r="A4449" t="str">
+        <v>Import Vendor Profile</v>
+      </c>
+      <c r="B4449" t="str">
+        <v>استيراد ملف المورد</v>
+      </c>
+      <c r="C4449" t="str">
+        <v>Importēt piegādātāja profilu</v>
+      </c>
+    </row>
+    <row r="4450">
+      <c r="A4450" t="str">
+        <v>Export Vendor Risk Rating Questions</v>
+      </c>
+      <c r="B4450" t="str">
+        <v>تصدير أسئلة تصنيف مخاطر المورد</v>
+      </c>
+      <c r="C4450" t="str">
+        <v>Eksportēt piegādātāja riska vērtējuma jautājumus</v>
+      </c>
+    </row>
+    <row r="4451">
+      <c r="A4451" t="str">
+        <v>Import Responses for Questions</v>
+      </c>
+      <c r="B4451" t="str">
+        <v>استيراد ردود الأسئلة</v>
+      </c>
+      <c r="C4451" t="str">
+        <v>Importēt atbildes uz jautājumiem</v>
+      </c>
+    </row>
+    <row r="4452">
+      <c r="A4452" t="str">
+        <v>Import Complete</v>
+      </c>
+      <c r="B4452" t="str">
+        <v>اكتمل الاستيراد</v>
+      </c>
+      <c r="C4452" t="str">
+        <v>Importēšana pabeigta</v>
+      </c>
+    </row>
+    <row r="4453">
+      <c r="A4453" t="str">
+        <v>vendors created</v>
+      </c>
+      <c r="B4453" t="str">
+        <v>تم إنشاء الموردين</v>
+      </c>
+      <c r="C4453" t="str">
+        <v>piegādātāji izveidoti</v>
+      </c>
+    </row>
+    <row r="4454">
+      <c r="A4454" t="str">
+        <v>responses updated</v>
+      </c>
+      <c r="B4454" t="str">
+        <v>تم تحديث الردود</v>
+      </c>
+      <c r="C4454" t="str">
+        <v>atbildes atjauninātas</v>
+      </c>
+    </row>
+    <row r="4455">
+      <c r="A4455" t="str">
+        <v>ratings updated</v>
+      </c>
+      <c r="B4455" t="str">
+        <v>تم تحديث التصنيفات</v>
+      </c>
+      <c r="C4455" t="str">
+        <v>vērtējumi atjaunināti</v>
+      </c>
+    </row>
+    <row r="4456">
+      <c r="A4456" t="str">
+        <v>Failed to export questions</v>
+      </c>
+      <c r="B4456" t="str">
+        <v>فشل تصدير الأسئلة</v>
+      </c>
+      <c r="C4456" t="str">
+        <v>Neizdevās eksportēt jautājumus</v>
+      </c>
+    </row>
+    <row r="4457">
+      <c r="A4457" t="str">
+        <v>Failed to import vendors</v>
+      </c>
+      <c r="B4457" t="str">
+        <v>فشل استيراد الموردين</v>
+      </c>
+      <c r="C4457" t="str">
+        <v>Neizdevās importēt piegādātājus</v>
+      </c>
+    </row>
+    <row r="4458">
+      <c r="A4458" t="str">
+        <v>Failed to import responses</v>
+      </c>
+      <c r="B4458" t="str">
+        <v>فشل استيراد الردود</v>
+      </c>
+      <c r="C4458" t="str">
+        <v>Neizdevās importēt atbildes</v>
+      </c>
+    </row>
+    <row r="4459">
+      <c r="A4459" t="str">
+        <v>Upload the filled vendor profile template (.xlsx or .xls)</v>
+      </c>
+      <c r="B4459" t="str">
+        <v>ارفع نموذج ملف المورد المعبأ (.xlsx أو .xls)</v>
+      </c>
+      <c r="C4459" t="str">
+        <v>Augšupielādēt aizpildīto piegādātāja profila veidni (.xlsx vai .xls)</v>
+      </c>
+    </row>
+    <row r="4460">
+      <c r="A4460" t="str">
+        <v>Upload the filled vendor questionnaire with responses (.xlsx or .xls)</v>
+      </c>
+      <c r="B4460" t="str">
+        <v>ارفع استبيان المورد المعبأ بالردود (.xlsx أو .xls)</v>
+      </c>
+      <c r="C4460" t="str">
+        <v>Augšupielādēt aizpildīto piegādātāja anketu ar atbildēm (.xlsx vai .xls)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4446"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4460"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Compliance: add Technical Evidence Integration module
- New schema models: IntegrationCredential, TechnicalEvidenceCollection, TechnicalEvidenceRecord, TechnicalEvidenceControlMapping
- Platform connectors: Azure Entra, Azure Security, Google Cloud, Cisco/PaloAlto/FortiGate, ServiceNow, Tenable, Acunetix
- API routes: /api/integration-credentials, /api/technical-evidence (CRUD, collect, publish, AI-suggest, control mappings)
- UI pages: Technical Evidence dashboard, collection detail, integration settings per platform
- Auto-publish collected evidence to Evidence module with AI-suggested control mappings
- Extract generateEvidenceCode to shared lib (src/lib/evidence-utils.ts)
- Add compliance.technical-evidence and compliance.integration-credentials permissions and nav entries
- Update i18n translations for new strings

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,12 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5218"/>
-  <cols>
-    <col min="1" max="1" width="60.83203125" customWidth="1"/>
-    <col min="2" max="2" width="60.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:C5306"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -57802,9 +57797,977 @@
         <v>Dodieties uz Pamatdatu pārvaldība &gt; Jomas.</v>
       </c>
     </row>
+    <row r="5219">
+      <c r="A5219" t="str">
+        <v>Technical Evidence</v>
+      </c>
+      <c r="B5219" t="str">
+        <v>الأدلة التقنية</v>
+      </c>
+      <c r="C5219" t="str">
+        <v>Tehniskie pierādījumi</v>
+      </c>
+    </row>
+    <row r="5220">
+      <c r="A5220" t="str">
+        <v>Credential Vault</v>
+      </c>
+      <c r="B5220" t="str">
+        <v>خزنة بيانات الاعتماد</v>
+      </c>
+      <c r="C5220" t="str">
+        <v>Akreditācijas datu glabātuve</v>
+      </c>
+    </row>
+    <row r="5221">
+      <c r="A5221" t="str">
+        <v>Configure Credentials</v>
+      </c>
+      <c r="B5221" t="str">
+        <v>تكوين بيانات الاعتماد</v>
+      </c>
+      <c r="C5221" t="str">
+        <v>Konfigurēt akreditācijas datus</v>
+      </c>
+    </row>
+    <row r="5222">
+      <c r="A5222" t="str">
+        <v>Connect to live systems to pull real-time evidence. This data can be used to support automated checks and provide up-to-the-minute status for audits. Ensure your integrations are configured on the Settings page.</v>
+      </c>
+      <c r="B5222" t="str">
+        <v>الاتصال بالأنظمة المباشرة لسحب الأدلة في الوقت الفعلي. يمكن استخدام هذه البيانات لدعم عمليات التحقق الآلية وتوفير حالة محدثة للتدقيق.</v>
+      </c>
+      <c r="C5222" t="str">
+        <v>Savienojieties ar reāllaika sistēmām, lai iegūtu pierādījumus. Šos datus var izmantot automatizētu pārbaužu atbalstam.</v>
+      </c>
+    </row>
+    <row r="5223">
+      <c r="A5223" t="str">
+        <v>Microsoft Azure &amp; Defender</v>
+      </c>
+      <c r="B5223" t="str">
+        <v>مايكروسوفت أزور والمدافع</v>
+      </c>
+      <c r="C5223" t="str">
+        <v>Microsoft Azure un Defender</v>
+      </c>
+    </row>
+    <row r="5224">
+      <c r="A5224" t="str">
+        <v>Tenable</v>
+      </c>
+      <c r="B5224" t="str">
+        <v>تينابل</v>
+      </c>
+      <c r="C5224" t="str">
+        <v>Tenable</v>
+      </c>
+    </row>
+    <row r="5225">
+      <c r="A5225" t="str">
+        <v>Acunetix</v>
+      </c>
+      <c r="B5225" t="str">
+        <v>أكيونتكس</v>
+      </c>
+      <c r="C5225" t="str">
+        <v>Acunetix</v>
+      </c>
+    </row>
+    <row r="5226">
+      <c r="A5226" t="str">
+        <v>Service Desk</v>
+      </c>
+      <c r="B5226" t="str">
+        <v>مكتب الخدمة</v>
+      </c>
+      <c r="C5226" t="str">
+        <v>Pakalpojumu dienests</v>
+      </c>
+    </row>
+    <row r="5227">
+      <c r="A5227" t="str">
+        <v>Google Cloud Platform</v>
+      </c>
+      <c r="B5227" t="str">
+        <v>منصة جوجل السحابية</v>
+      </c>
+      <c r="C5227" t="str">
+        <v>Google mākoņa platforma</v>
+      </c>
+    </row>
+    <row r="5228">
+      <c r="A5228" t="str">
+        <v>No data sources configured</v>
+      </c>
+      <c r="B5228" t="str">
+        <v>لم يتم تكوين مصادر البيانات</v>
+      </c>
+      <c r="C5228" t="str">
+        <v>Nav konfigurēti datu avoti</v>
+      </c>
+    </row>
+    <row r="5229">
+      <c r="A5229" t="str">
+        <v>Configure credentials in Settings to enable data collection for this platform.</v>
+      </c>
+      <c r="B5229" t="str">
+        <v>قم بتكوين بيانات الاعتماد في الإعدادات لتمكين جمع البيانات لهذه المنصة.</v>
+      </c>
+      <c r="C5229" t="str">
+        <v>Konfigurējiet akreditācijas datus iestatījumos, lai iespējotu datu vākšanu šai platformai.</v>
+      </c>
+    </row>
+    <row r="5230">
+      <c r="A5230" t="str">
+        <v>Last Collected</v>
+      </c>
+      <c r="B5230" t="str">
+        <v>آخر جمع</v>
+      </c>
+      <c r="C5230" t="str">
+        <v>Pēdējoreiz savākts</v>
+      </c>
+    </row>
+    <row r="5231">
+      <c r="A5231" t="str">
+        <v>Never</v>
+      </c>
+      <c r="B5231" t="str">
+        <v>أبداً</v>
+      </c>
+      <c r="C5231" t="str">
+        <v>Nekad</v>
+      </c>
+    </row>
+    <row r="5232">
+      <c r="A5232" t="str">
+        <v>Collect</v>
+      </c>
+      <c r="B5232" t="str">
+        <v>جمع</v>
+      </c>
+      <c r="C5232" t="str">
+        <v>Savākt</v>
+      </c>
+    </row>
+    <row r="5233">
+      <c r="A5233" t="str">
+        <v>Recollect</v>
+      </c>
+      <c r="B5233" t="str">
+        <v>إعادة الجمع</v>
+      </c>
+      <c r="C5233" t="str">
+        <v>Atkārtoti savākt</v>
+      </c>
+    </row>
+    <row r="5234">
+      <c r="A5234" t="str">
+        <v>Record Count</v>
+      </c>
+      <c r="B5234" t="str">
+        <v>عدد السجلات</v>
+      </c>
+      <c r="C5234" t="str">
+        <v>Ierakstu skaits</v>
+      </c>
+    </row>
+    <row r="5235">
+      <c r="A5235" t="str">
+        <v>Collection failed</v>
+      </c>
+      <c r="B5235" t="str">
+        <v>فشل الجمع</v>
+      </c>
+      <c r="C5235" t="str">
+        <v>Savākšana neizdevās</v>
+      </c>
+    </row>
+    <row r="5236">
+      <c r="A5236" t="str">
+        <v>View Data</v>
+      </c>
+      <c r="B5236" t="str">
+        <v>عرض البيانات</v>
+      </c>
+      <c r="C5236" t="str">
+        <v>Skatīt datus</v>
+      </c>
+    </row>
+    <row r="5237">
+      <c r="A5237" t="str">
+        <v>Collecting...</v>
+      </c>
+      <c r="B5237" t="str">
+        <v>جاري الجمع...</v>
+      </c>
+      <c r="C5237" t="str">
+        <v>Savāc...</v>
+      </c>
+    </row>
+    <row r="5238">
+      <c r="A5238" t="str">
+        <v>Manage credentials for connecting to external platforms. Credentials are encrypted and stored securely.</v>
+      </c>
+      <c r="B5238" t="str">
+        <v>إدارة بيانات الاعتماد للاتصال بالمنصات الخارجية. يتم تشفير بيانات الاعتماد وتخزينها بأمان.</v>
+      </c>
+      <c r="C5238" t="str">
+        <v>Pārvaldiet akreditācijas datus savienojumam ar ārējām platformām. Akreditācijas dati tiek šifrēti un droši glabāti.</v>
+      </c>
+    </row>
+    <row r="5239">
+      <c r="A5239" t="str">
+        <v>Connected</v>
+      </c>
+      <c r="B5239" t="str">
+        <v>متصل</v>
+      </c>
+      <c r="C5239" t="str">
+        <v>Savienots</v>
+      </c>
+    </row>
+    <row r="5240">
+      <c r="A5240" t="str">
+        <v>Disconnected</v>
+      </c>
+      <c r="B5240" t="str">
+        <v>غير متصل</v>
+      </c>
+      <c r="C5240" t="str">
+        <v>Atvienots</v>
+      </c>
+    </row>
+    <row r="5241">
+      <c r="A5241" t="str">
+        <v>Not Configured</v>
+      </c>
+      <c r="B5241" t="str">
+        <v>غير مكوّن</v>
+      </c>
+      <c r="C5241" t="str">
+        <v>Nav konfigurēts</v>
+      </c>
+    </row>
+    <row r="5242">
+      <c r="A5242" t="str">
+        <v>Azure Entra (AD)</v>
+      </c>
+      <c r="B5242" t="str">
+        <v>أزور إنترا (AD)</v>
+      </c>
+      <c r="C5242" t="str">
+        <v>Azure Entra (AD)</v>
+      </c>
+    </row>
+    <row r="5243">
+      <c r="A5243" t="str">
+        <v>Azure Security</v>
+      </c>
+      <c r="B5243" t="str">
+        <v>أمن أزور</v>
+      </c>
+      <c r="C5243" t="str">
+        <v>Azure drošība</v>
+      </c>
+    </row>
+    <row r="5244">
+      <c r="A5244" t="str">
+        <v>Cisco</v>
+      </c>
+      <c r="B5244" t="str">
+        <v>سيسكو</v>
+      </c>
+      <c r="C5244" t="str">
+        <v>Cisco</v>
+      </c>
+    </row>
+    <row r="5245">
+      <c r="A5245" t="str">
+        <v>Palo Alto Networks</v>
+      </c>
+      <c r="B5245" t="str">
+        <v>شبكات بالو ألتو</v>
+      </c>
+      <c r="C5245" t="str">
+        <v>Palo Alto Networks</v>
+      </c>
+    </row>
+    <row r="5246">
+      <c r="A5246" t="str">
+        <v>FortiGate</v>
+      </c>
+      <c r="B5246" t="str">
+        <v>فورتي جيت</v>
+      </c>
+      <c r="C5246" t="str">
+        <v>FortiGate</v>
+      </c>
+    </row>
+    <row r="5247">
+      <c r="A5247" t="str">
+        <v>ServiceNow</v>
+      </c>
+      <c r="B5247" t="str">
+        <v>سيرفس ناو</v>
+      </c>
+      <c r="C5247" t="str">
+        <v>ServiceNow</v>
+      </c>
+    </row>
+    <row r="5248">
+      <c r="A5248" t="str">
+        <v>Connect to Azure Active Directory for user accounts, MFA status, dormant users, and password policies.</v>
+      </c>
+      <c r="B5248" t="str">
+        <v>الاتصال بـ Azure Active Directory للحصول على حسابات المستخدمين وحالة MFA والمستخدمين الخاملين وسياسات كلمات المرور.</v>
+      </c>
+      <c r="C5248" t="str">
+        <v>Savienojieties ar Azure Active Directory lietotāju kontiem, MFA statusam, neaktīviem lietotājiem un paroļu politikām.</v>
+      </c>
+    </row>
+    <row r="5249">
+      <c r="A5249" t="str">
+        <v>Connect to Azure Defender, Sentinel, Secure Score, and Cloud Security Posture Management.</v>
+      </c>
+      <c r="B5249" t="str">
+        <v>الاتصال بـ Azure Defender و Sentinel و Secure Score وإدارة وضع أمان السحابة.</v>
+      </c>
+      <c r="C5249" t="str">
+        <v>Savienojieties ar Azure Defender, Sentinel, Secure Score un mākoņa drošības pārvaldību.</v>
+      </c>
+    </row>
+    <row r="5250">
+      <c r="A5250" t="str">
+        <v>Connect to GCP Security Command Center for posture, findings, IAM, and cloud inventory.</v>
+      </c>
+      <c r="B5250" t="str">
+        <v>الاتصال بمركز أوامر أمان GCP للوضع الأمني والنتائج وIAM ومخزون السحابة.</v>
+      </c>
+      <c r="C5250" t="str">
+        <v>Savienojieties ar GCP drošības komandu centru.</v>
+      </c>
+    </row>
+    <row r="5251">
+      <c r="A5251" t="str">
+        <v>Connect to Cisco ASA/FTD firewalls for configuration analysis and compliance checks.</v>
+      </c>
+      <c r="B5251" t="str">
+        <v>الاتصال بجدران حماية Cisco ASA/FTD لتحليل التكوين وفحوصات الامتثال.</v>
+      </c>
+      <c r="C5251" t="str">
+        <v>Savienojieties ar Cisco ASA/FTD ugunsmūriem konfigurācijas analīzei.</v>
+      </c>
+    </row>
+    <row r="5252">
+      <c r="A5252" t="str">
+        <v>Connect to Palo Alto firewalls for security policy and configuration evidence.</v>
+      </c>
+      <c r="B5252" t="str">
+        <v>الاتصال بجدران حماية Palo Alto لأدلة سياسة الأمان والتكوين.</v>
+      </c>
+      <c r="C5252" t="str">
+        <v>Savienojieties ar Palo Alto ugunsmūriem drošības politikas pierādījumiem.</v>
+      </c>
+    </row>
+    <row r="5253">
+      <c r="A5253" t="str">
+        <v>Connect to FortiGate firewalls for network security compliance evidence.</v>
+      </c>
+      <c r="B5253" t="str">
+        <v>الاتصال بجدران حماية FortiGate لأدلة امتثال أمان الشبكة.</v>
+      </c>
+      <c r="C5253" t="str">
+        <v>Savienojieties ar FortiGate ugunsmūriem tīkla drošības pierādījumiem.</v>
+      </c>
+    </row>
+    <row r="5254">
+      <c r="A5254" t="str">
+        <v>Connect to ServiceNow for incidents, change requests, and service desk evidence.</v>
+      </c>
+      <c r="B5254" t="str">
+        <v>الاتصال بـ ServiceNow للحوادث وطلبات التغيير وأدلة مكتب الخدمة.</v>
+      </c>
+      <c r="C5254" t="str">
+        <v>Savienojieties ar ServiceNow incidentiem un izmaiņu pieprasījumiem.</v>
+      </c>
+    </row>
+    <row r="5255">
+      <c r="A5255" t="str">
+        <v>Connect to Tenable for vulnerability scan results and security assessment data.</v>
+      </c>
+      <c r="B5255" t="str">
+        <v>الاتصال بـ Tenable لنتائج فحص الثغرات وبيانات تقييم الأمان.</v>
+      </c>
+      <c r="C5255" t="str">
+        <v>Savienojieties ar Tenable ievainojamību skenēšanas rezultātiem.</v>
+      </c>
+    </row>
+    <row r="5256">
+      <c r="A5256" t="str">
+        <v>Connect to Acunetix for web application vulnerability scanning evidence.</v>
+      </c>
+      <c r="B5256" t="str">
+        <v>الاتصال بـ Acunetix لأدلة فحص ثغرات تطبيقات الويب.</v>
+      </c>
+      <c r="C5256" t="str">
+        <v>Savienojieties ar Acunetix tīmekļa ievainojamību skenēšanas pierādījumiem.</v>
+      </c>
+    </row>
+    <row r="5257">
+      <c r="A5257" t="str">
+        <v>Credential Name</v>
+      </c>
+      <c r="B5257" t="str">
+        <v>اسم بيانات الاعتماد</v>
+      </c>
+      <c r="C5257" t="str">
+        <v>Akreditācijas datu nosaukums</v>
+      </c>
+    </row>
+    <row r="5258">
+      <c r="A5258" t="str">
+        <v>Tenant ID</v>
+      </c>
+      <c r="B5258" t="str">
+        <v>معرف المستأجر</v>
+      </c>
+      <c r="C5258" t="str">
+        <v>Īrnieka ID</v>
+      </c>
+    </row>
+    <row r="5259">
+      <c r="A5259" t="str">
+        <v>Client ID</v>
+      </c>
+      <c r="B5259" t="str">
+        <v>معرف العميل</v>
+      </c>
+      <c r="C5259" t="str">
+        <v>Klienta ID</v>
+      </c>
+    </row>
+    <row r="5260">
+      <c r="A5260" t="str">
+        <v>Client Secret</v>
+      </c>
+      <c r="B5260" t="str">
+        <v>سر العميل</v>
+      </c>
+      <c r="C5260" t="str">
+        <v>Klienta noslēpums</v>
+      </c>
+    </row>
+    <row r="5261">
+      <c r="A5261" t="str">
+        <v>API Key</v>
+      </c>
+      <c r="B5261" t="str">
+        <v>مفتاح API</v>
+      </c>
+      <c r="C5261" t="str">
+        <v>API atslēga</v>
+      </c>
+    </row>
+    <row r="5262">
+      <c r="A5262" t="str">
+        <v>API Token</v>
+      </c>
+      <c r="B5262" t="str">
+        <v>رمز API</v>
+      </c>
+      <c r="C5262" t="str">
+        <v>API žetons</v>
+      </c>
+    </row>
+    <row r="5263">
+      <c r="A5263" t="str">
+        <v>Instance URL</v>
+      </c>
+      <c r="B5263" t="str">
+        <v>رابط المثيل</v>
+      </c>
+      <c r="C5263" t="str">
+        <v>Instances URL</v>
+      </c>
+    </row>
+    <row r="5264">
+      <c r="A5264" t="str">
+        <v>Access Key</v>
+      </c>
+      <c r="B5264" t="str">
+        <v>مفتاح الوصول</v>
+      </c>
+      <c r="C5264" t="str">
+        <v>Piekļuves atslēga</v>
+      </c>
+    </row>
+    <row r="5265">
+      <c r="A5265" t="str">
+        <v>Secret Key</v>
+      </c>
+      <c r="B5265" t="str">
+        <v>المفتاح السري</v>
+      </c>
+      <c r="C5265" t="str">
+        <v>Slepenā atslēga</v>
+      </c>
+    </row>
+    <row r="5266">
+      <c r="A5266" t="str">
+        <v>Host URL</v>
+      </c>
+      <c r="B5266" t="str">
+        <v>رابط المضيف</v>
+      </c>
+      <c r="C5266" t="str">
+        <v>Resursdatora URL</v>
+      </c>
+    </row>
+    <row r="5267">
+      <c r="A5267" t="str">
+        <v>Project ID</v>
+      </c>
+      <c r="B5267" t="str">
+        <v>معرف المشروع</v>
+      </c>
+      <c r="C5267" t="str">
+        <v>Projekta ID</v>
+      </c>
+    </row>
+    <row r="5268">
+      <c r="A5268" t="str">
+        <v>Service Account JSON</v>
+      </c>
+      <c r="B5268" t="str">
+        <v>ملف حساب الخدمة JSON</v>
+      </c>
+      <c r="C5268" t="str">
+        <v>Pakalpojuma konta JSON</v>
+      </c>
+    </row>
+    <row r="5269">
+      <c r="A5269" t="str">
+        <v>Save Credential</v>
+      </c>
+      <c r="B5269" t="str">
+        <v>حفظ بيانات الاعتماد</v>
+      </c>
+      <c r="C5269" t="str">
+        <v>Saglabāt akreditācijas datus</v>
+      </c>
+    </row>
+    <row r="5270">
+      <c r="A5270" t="str">
+        <v>Update Credential</v>
+      </c>
+      <c r="B5270" t="str">
+        <v>تحديث بيانات الاعتماد</v>
+      </c>
+      <c r="C5270" t="str">
+        <v>Atjaunināt akreditācijas datus</v>
+      </c>
+    </row>
+    <row r="5271">
+      <c r="A5271" t="str">
+        <v>Test Connection</v>
+      </c>
+      <c r="B5271" t="str">
+        <v>اختبار الاتصال</v>
+      </c>
+      <c r="C5271" t="str">
+        <v>Testēt savienojumu</v>
+      </c>
+    </row>
+    <row r="5272">
+      <c r="A5272" t="str">
+        <v>Connection successful</v>
+      </c>
+      <c r="B5272" t="str">
+        <v>الاتصال ناجح</v>
+      </c>
+      <c r="C5272" t="str">
+        <v>Savienojums veiksmīgs</v>
+      </c>
+    </row>
+    <row r="5273">
+      <c r="A5273" t="str">
+        <v>Connection Failed</v>
+      </c>
+      <c r="B5273" t="str">
+        <v>فشل الاتصال</v>
+      </c>
+      <c r="C5273" t="str">
+        <v>Savienojums neizdevās</v>
+      </c>
+    </row>
+    <row r="5274">
+      <c r="A5274" t="str">
+        <v>Credential saved and data sources initialized</v>
+      </c>
+      <c r="B5274" t="str">
+        <v>تم حفظ بيانات الاعتماد وتهيئة مصادر البيانات</v>
+      </c>
+      <c r="C5274" t="str">
+        <v>Akreditācijas dati saglabāti un datu avoti inicializēti</v>
+      </c>
+    </row>
+    <row r="5275">
+      <c r="A5275" t="str">
+        <v>Credential updated</v>
+      </c>
+      <c r="B5275" t="str">
+        <v>تم تحديث بيانات الاعتماد</v>
+      </c>
+      <c r="C5275" t="str">
+        <v>Akreditācijas dati atjaunināti</v>
+      </c>
+    </row>
+    <row r="5276">
+      <c r="A5276" t="str">
+        <v>Credential deleted</v>
+      </c>
+      <c r="B5276" t="str">
+        <v>تم حذف بيانات الاعتماد</v>
+      </c>
+      <c r="C5276" t="str">
+        <v>Akreditācijas dati dzēsti</v>
+      </c>
+    </row>
+    <row r="5277">
+      <c r="A5277" t="str">
+        <v>Are you sure you want to delete this credential? All associated collections and data will be removed.</v>
+      </c>
+      <c r="B5277" t="str">
+        <v>هل أنت متأكد من حذف بيانات الاعتماد هذه؟ سيتم إزالة جميع المجموعات والبيانات المرتبطة.</v>
+      </c>
+      <c r="C5277" t="str">
+        <v>Vai tiešām vēlaties dzēst šos akreditācijas datus? Visas saistītās kolekcijas un dati tiks noņemti.</v>
+      </c>
+    </row>
+    <row r="5278">
+      <c r="A5278" t="str">
+        <v>Missing required fields</v>
+      </c>
+      <c r="B5278" t="str">
+        <v>حقول مطلوبة مفقودة</v>
+      </c>
+      <c r="C5278" t="str">
+        <v>Trūkst obligāto lauku</v>
+      </c>
+    </row>
+    <row r="5279">
+      <c r="A5279" t="str">
+        <v>Leave empty to keep current value</v>
+      </c>
+      <c r="B5279" t="str">
+        <v>اتركه فارغاً للاحتفاظ بالقيمة الحالية</v>
+      </c>
+      <c r="C5279" t="str">
+        <v>Atstājiet tukšu, lai saglabātu pašreizējo vērtību</v>
+      </c>
+    </row>
+    <row r="5280">
+      <c r="A5280" t="str">
+        <v>Paste service account JSON here</v>
+      </c>
+      <c r="B5280" t="str">
+        <v>الصق ملف JSON لحساب الخدمة هنا</v>
+      </c>
+      <c r="C5280" t="str">
+        <v>Ielīmējiet pakalpojuma konta JSON šeit</v>
+      </c>
+    </row>
+    <row r="5281">
+      <c r="A5281" t="str">
+        <v>Unknown platform</v>
+      </c>
+      <c r="B5281" t="str">
+        <v>منصة غير معروفة</v>
+      </c>
+      <c r="C5281" t="str">
+        <v>Nezināma platforma</v>
+      </c>
+    </row>
+    <row r="5282">
+      <c r="A5282" t="str">
+        <v>No records collected yet</v>
+      </c>
+      <c r="B5282" t="str">
+        <v>لم يتم جمع سجلات بعد</v>
+      </c>
+      <c r="C5282" t="str">
+        <v>Vēl nav savākti ieraksti</v>
+      </c>
+    </row>
+    <row r="5283">
+      <c r="A5283" t="str">
+        <v>Click Recollect to fetch data from the source.</v>
+      </c>
+      <c r="B5283" t="str">
+        <v>انقر على إعادة الجمع لجلب البيانات من المصدر.</v>
+      </c>
+      <c r="C5283" t="str">
+        <v>Noklikšķiniet Atkārtoti savākt, lai iegūtu datus no avota.</v>
+      </c>
+    </row>
+    <row r="5284">
+      <c r="A5284" t="str">
+        <v>Control Mappings</v>
+      </c>
+      <c r="B5284" t="str">
+        <v>تعيينات الضوابط</v>
+      </c>
+      <c r="C5284" t="str">
+        <v>Kontroles kartējumi</v>
+      </c>
+    </row>
+    <row r="5285">
+      <c r="A5285" t="str">
+        <v>AI Suggest Controls</v>
+      </c>
+      <c r="B5285" t="str">
+        <v>اقتراح ضوابط بالذكاء الاصطناعي</v>
+      </c>
+      <c r="C5285" t="str">
+        <v>AI ieteikt kontroles</v>
+      </c>
+    </row>
+    <row r="5286">
+      <c r="A5286" t="str">
+        <v>No control mappings yet. Use AI Suggest to auto-map controls.</v>
+      </c>
+      <c r="B5286" t="str">
+        <v>لا توجد تعيينات ضوابط بعد. استخدم اقتراح AI لتعيين الضوابط تلقائياً.</v>
+      </c>
+      <c r="C5286" t="str">
+        <v>Vēl nav kontroles kartējumu. Izmantojiet AI ieteikumu automātiskai kartēšanai.</v>
+      </c>
+    </row>
+    <row r="5287">
+      <c r="A5287" t="str">
+        <v>Pending Confirmation</v>
+      </c>
+      <c r="B5287" t="str">
+        <v>في انتظار التأكيد</v>
+      </c>
+      <c r="C5287" t="str">
+        <v>Gaida apstiprinājumu</v>
+      </c>
+    </row>
+    <row r="5288">
+      <c r="A5288" t="str">
+        <v>Confirmed</v>
+      </c>
+      <c r="B5288" t="str">
+        <v>مؤكد</v>
+      </c>
+      <c r="C5288" t="str">
+        <v>Apstiprināts</v>
+      </c>
+    </row>
+    <row r="5289">
+      <c r="A5289" t="str">
+        <v>confidence</v>
+      </c>
+      <c r="B5289" t="str">
+        <v>الثقة</v>
+      </c>
+      <c r="C5289" t="str">
+        <v>pārliecība</v>
+      </c>
+    </row>
+    <row r="5290">
+      <c r="A5290" t="str">
+        <v>Reject</v>
+      </c>
+      <c r="B5290" t="str">
+        <v>رفض</v>
+      </c>
+      <c r="C5290" t="str">
+        <v>Noraidīt</v>
+      </c>
+    </row>
+    <row r="5291">
+      <c r="A5291" t="str">
+        <v>Mapping confirmed</v>
+      </c>
+      <c r="B5291" t="str">
+        <v>تم تأكيد التعيين</v>
+      </c>
+      <c r="C5291" t="str">
+        <v>Kartējums apstiprināts</v>
+      </c>
+    </row>
+    <row r="5292">
+      <c r="A5292" t="str">
+        <v>Mapping rejected</v>
+      </c>
+      <c r="B5292" t="str">
+        <v>تم رفض التعيين</v>
+      </c>
+      <c r="C5292" t="str">
+        <v>Kartējums noraidīts</v>
+      </c>
+    </row>
+    <row r="5293">
+      <c r="A5293" t="str">
+        <v>AI suggestion failed</v>
+      </c>
+      <c r="B5293" t="str">
+        <v>فشل اقتراح الذكاء الاصطناعي</v>
+      </c>
+      <c r="C5293" t="str">
+        <v>AI ieteikums neizdevās</v>
+      </c>
+    </row>
+    <row r="5294">
+      <c r="A5294" t="str">
+        <v>AI suggestions generated</v>
+      </c>
+      <c r="B5294" t="str">
+        <v>تم إنشاء اقتراحات الذكاء الاصطناعي</v>
+      </c>
+      <c r="C5294" t="str">
+        <v>AI ieteikumi ģenerēti</v>
+      </c>
+    </row>
+    <row r="5295">
+      <c r="A5295" t="str">
+        <v>Failed to confirm mapping</v>
+      </c>
+      <c r="B5295" t="str">
+        <v>فشل تأكيد التعيين</v>
+      </c>
+      <c r="C5295" t="str">
+        <v>Neizdevās apstiprināt kartējumu</v>
+      </c>
+    </row>
+    <row r="5296">
+      <c r="A5296" t="str">
+        <v>Failed to reject mapping</v>
+      </c>
+      <c r="B5296" t="str">
+        <v>فشل رفض التعيين</v>
+      </c>
+      <c r="C5296" t="str">
+        <v>Neizdevās noraidīt kartējumu</v>
+      </c>
+    </row>
+    <row r="5297">
+      <c r="A5297" t="str">
+        <v>You don't have permission to access Technical Evidence.</v>
+      </c>
+      <c r="B5297" t="str">
+        <v>ليس لديك صلاحية للوصول إلى الأدلة التقنية.</v>
+      </c>
+      <c r="C5297" t="str">
+        <v>Jums nav atļaujas piekļūt tehniskajiem pierādījumiem.</v>
+      </c>
+    </row>
+    <row r="5298">
+      <c r="A5298" t="str">
+        <v>You don't have permission to manage integration credentials.</v>
+      </c>
+      <c r="B5298" t="str">
+        <v>ليس لديك صلاحية لإدارة بيانات اعتماد التكامل.</v>
+      </c>
+      <c r="C5298" t="str">
+        <v>Jums nav atļaujas pārvaldīt integrācijas akreditācijas datus.</v>
+      </c>
+    </row>
+    <row r="5299">
+      <c r="A5299" t="str">
+        <v>You don't have permission to manage credentials.</v>
+      </c>
+      <c r="B5299" t="str">
+        <v>ليس لديك صلاحية لإدارة بيانات الاعتماد.</v>
+      </c>
+      <c r="C5299" t="str">
+        <v>Jums nav atļaujas pārvaldīt akreditācijas datus.</v>
+      </c>
+    </row>
+    <row r="5300">
+      <c r="A5300" t="str">
+        <v>You don't have permission to view this data.</v>
+      </c>
+      <c r="B5300" t="str">
+        <v>ليس لديك صلاحية لعرض هذه البيانات.</v>
+      </c>
+      <c r="C5300" t="str">
+        <v>Jums nav atļaujas skatīt šos datus.</v>
+      </c>
+    </row>
+    <row r="5301">
+      <c r="A5301" t="str">
+        <v>Configure Credential</v>
+      </c>
+      <c r="B5301" t="str">
+        <v>تكوين بيانات الاعتماد</v>
+      </c>
+      <c r="C5301" t="str">
+        <v>Konfigurēt akreditācijas datus</v>
+      </c>
+    </row>
+    <row r="5302">
+      <c r="A5302" t="str">
+        <v>Save the credential first before testing</v>
+      </c>
+      <c r="B5302" t="str">
+        <v>احفظ بيانات الاعتماد أولاً قبل الاختبار</v>
+      </c>
+      <c r="C5302" t="str">
+        <v>Vispirms saglabājiet akreditācijas datus pirms testēšanas</v>
+      </c>
+    </row>
+    <row r="5303">
+      <c r="A5303" t="str">
+        <v>Failed to save credential</v>
+      </c>
+      <c r="B5303" t="str">
+        <v>فشل حفظ بيانات الاعتماد</v>
+      </c>
+      <c r="C5303" t="str">
+        <v>Neizdevās saglabāt akreditācijas datus</v>
+      </c>
+    </row>
+    <row r="5304">
+      <c r="A5304" t="str">
+        <v>Failed to update</v>
+      </c>
+      <c r="B5304" t="str">
+        <v>فشل التحديث</v>
+      </c>
+      <c r="C5304" t="str">
+        <v>Neizdevās atjaunināt</v>
+      </c>
+    </row>
+    <row r="5305">
+      <c r="A5305" t="str">
+        <v>Failed to delete credential</v>
+      </c>
+      <c r="B5305" t="str">
+        <v>فشل حذف بيانات الاعتماد</v>
+      </c>
+      <c r="C5305" t="str">
+        <v>Neizdevās dzēst akreditācijas datus</v>
+      </c>
+    </row>
+    <row r="5306">
+      <c r="A5306" t="str">
+        <v>Connection test failed</v>
+      </c>
+      <c r="B5306" t="str">
+        <v>فشل اختبار الاتصال</v>
+      </c>
+      <c r="C5306" t="str">
+        <v>Savienojuma tests neizdevās</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5218"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5306"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Arabic and Latvian translations for engagement workflow UI
Localize all Phase 2/3 engagement-workflow strings (announcement, APM,
minutes of meeting, and the workflow hub) — 85 new phrases added to
translations.xlsx with Arabic and Latvian, locale files regenerated.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5306"/>
+  <dimension ref="A1:C5391"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -58765,9 +58765,944 @@
         <v>Savienojuma tests neizdevās</v>
       </c>
     </row>
+    <row r="5307">
+      <c r="A5307" t="str">
+        <v>Add Minutes</v>
+      </c>
+      <c r="B5307" t="str">
+        <v>إضافة محضر</v>
+      </c>
+      <c r="C5307" t="str">
+        <v>Pievienot protokolu</v>
+      </c>
+    </row>
+    <row r="5308">
+      <c r="A5308" t="str">
+        <v>Agenda</v>
+      </c>
+      <c r="B5308" t="str">
+        <v>جدول الأعمال</v>
+      </c>
+      <c r="C5308" t="str">
+        <v>Darba kārtība</v>
+      </c>
+    </row>
+    <row r="5309">
+      <c r="A5309" t="str">
+        <v>Announcement</v>
+      </c>
+      <c r="B5309" t="str">
+        <v>الإعلان</v>
+      </c>
+      <c r="C5309" t="str">
+        <v>Paziņojums</v>
+      </c>
+    </row>
+    <row r="5310">
+      <c r="A5310" t="str">
+        <v>Announcement message</v>
+      </c>
+      <c r="B5310" t="str">
+        <v>نص الإعلان</v>
+      </c>
+      <c r="C5310" t="str">
+        <v>Paziņojuma teksts</v>
+      </c>
+    </row>
+    <row r="5311">
+      <c r="A5311" t="str">
+        <v>Announcement saved</v>
+      </c>
+      <c r="B5311" t="str">
+        <v>تم حفظ الإعلان</v>
+      </c>
+      <c r="C5311" t="str">
+        <v>Paziņojums saglabāts</v>
+      </c>
+    </row>
+    <row r="5312">
+      <c r="A5312" t="str">
+        <v>Announcement sent</v>
+      </c>
+      <c r="B5312" t="str">
+        <v>تم إرسال الإعلان</v>
+      </c>
+      <c r="C5312" t="str">
+        <v>Paziņojums nosūtīts</v>
+      </c>
+    </row>
+    <row r="5313">
+      <c r="A5313" t="str">
+        <v>Announcement subject</v>
+      </c>
+      <c r="B5313" t="str">
+        <v>موضوع الإعلان</v>
+      </c>
+      <c r="C5313" t="str">
+        <v>Paziņojuma temats</v>
+      </c>
+    </row>
+    <row r="5314">
+      <c r="A5314" t="str">
+        <v>Are you sure you want to delete these minutes?</v>
+      </c>
+      <c r="B5314" t="str">
+        <v>هل أنت متأكد أنك تريد حذف هذا المحضر؟</v>
+      </c>
+      <c r="C5314" t="str">
+        <v>Vai tiešām vēlaties dzēst šo protokolu?</v>
+      </c>
+    </row>
+    <row r="5315">
+      <c r="A5315" t="str">
+        <v>Are you sure you want to delete this document?</v>
+      </c>
+      <c r="B5315" t="str">
+        <v>هل أنت متأكد أنك تريد حذف هذا المستند؟</v>
+      </c>
+      <c r="C5315" t="str">
+        <v>Vai tiešām vēlaties dzēst šo dokumentu?</v>
+      </c>
+    </row>
+    <row r="5316">
+      <c r="A5316" t="str">
+        <v>Attendees</v>
+      </c>
+      <c r="B5316" t="str">
+        <v>الحضور</v>
+      </c>
+      <c r="C5316" t="str">
+        <v>Dalībnieki</v>
+      </c>
+    </row>
+    <row r="5317">
+      <c r="A5317" t="str">
+        <v>Audit Announcement</v>
+      </c>
+      <c r="B5317" t="str">
+        <v>إعلان التدقيق</v>
+      </c>
+      <c r="C5317" t="str">
+        <v>Audita paziņojums</v>
+      </c>
+    </row>
+    <row r="5318">
+      <c r="A5318" t="str">
+        <v>audit engagement(s) generated from this plan</v>
+      </c>
+      <c r="B5318" t="str">
+        <v>مهمة (مهام) تدقيق تم إنشاؤها من هذه الخطة</v>
+      </c>
+      <c r="C5318" t="str">
+        <v>no šī plāna izveidotie audita uzdevumi</v>
+      </c>
+    </row>
+    <row r="5319">
+      <c r="A5319" t="str">
+        <v>Audit methodology</v>
+      </c>
+      <c r="B5319" t="str">
+        <v>منهجية التدقيق</v>
+      </c>
+      <c r="C5319" t="str">
+        <v>Audita metodoloģija</v>
+      </c>
+    </row>
+    <row r="5320">
+      <c r="A5320" t="str">
+        <v>Audit objectives</v>
+      </c>
+      <c r="B5320" t="str">
+        <v>أهداف التدقيق</v>
+      </c>
+      <c r="C5320" t="str">
+        <v>Audita mērķi</v>
+      </c>
+    </row>
+    <row r="5321">
+      <c r="A5321" t="str">
+        <v>Audit Planning Memorandum</v>
+      </c>
+      <c r="B5321" t="str">
+        <v>مذكرة تخطيط التدقيق</v>
+      </c>
+      <c r="C5321" t="str">
+        <v>Audita plānošanas memorands</v>
+      </c>
+    </row>
+    <row r="5322">
+      <c r="A5322" t="str">
+        <v>Audit planning memorandum saved</v>
+      </c>
+      <c r="B5322" t="str">
+        <v>تم حفظ مذكرة تخطيط التدقيق</v>
+      </c>
+      <c r="C5322" t="str">
+        <v>Audita plānošanas memorands saglabāts</v>
+      </c>
+    </row>
+    <row r="5323">
+      <c r="A5323" t="str">
+        <v>Audit Program</v>
+      </c>
+      <c r="B5323" t="str">
+        <v>برنامج التدقيق</v>
+      </c>
+      <c r="C5323" t="str">
+        <v>Audita programma</v>
+      </c>
+    </row>
+    <row r="5324">
+      <c r="A5324" t="str">
+        <v>Audit Program Documents</v>
+      </c>
+      <c r="B5324" t="str">
+        <v>مستندات برنامج التدقيق</v>
+      </c>
+      <c r="C5324" t="str">
+        <v>Audita programmas dokumenti</v>
+      </c>
+    </row>
+    <row r="5325">
+      <c r="A5325" t="str">
+        <v>Audit scope</v>
+      </c>
+      <c r="B5325" t="str">
+        <v>نطاق التدقيق</v>
+      </c>
+      <c r="C5325" t="str">
+        <v>Audita tvērums</v>
+      </c>
+    </row>
+    <row r="5326">
+      <c r="A5326" t="str">
+        <v>Audit timeline</v>
+      </c>
+      <c r="B5326" t="str">
+        <v>الجدول الزمني للتدقيق</v>
+      </c>
+      <c r="C5326" t="str">
+        <v>Audita laika grafiks</v>
+      </c>
+    </row>
+    <row r="5327">
+      <c r="A5327" t="str">
+        <v>Closing Meeting</v>
+      </c>
+      <c r="B5327" t="str">
+        <v>اجتماع الإغلاق</v>
+      </c>
+      <c r="C5327" t="str">
+        <v>Noslēguma sanāksme</v>
+      </c>
+    </row>
+    <row r="5328">
+      <c r="A5328" t="str">
+        <v>Commence Date</v>
+      </c>
+      <c r="B5328" t="str">
+        <v>تاريخ البدء</v>
+      </c>
+      <c r="C5328" t="str">
+        <v>Sākuma datums</v>
+      </c>
+    </row>
+    <row r="5329">
+      <c r="A5329" t="str">
+        <v>Current</v>
+      </c>
+      <c r="B5329" t="str">
+        <v>الحالي</v>
+      </c>
+      <c r="C5329" t="str">
+        <v>Pašreizējais</v>
+      </c>
+    </row>
+    <row r="5330">
+      <c r="A5330" t="str">
+        <v>Current step updated</v>
+      </c>
+      <c r="B5330" t="str">
+        <v>تم تحديث الخطوة الحالية</v>
+      </c>
+      <c r="C5330" t="str">
+        <v>Pašreizējais solis atjaunināts</v>
+      </c>
+    </row>
+    <row r="5331">
+      <c r="A5331" t="str">
+        <v>Decisions &amp; Action Plans</v>
+      </c>
+      <c r="B5331" t="str">
+        <v>القرارات وخطط العمل</v>
+      </c>
+      <c r="C5331" t="str">
+        <v>Lēmumi un rīcības plāni</v>
+      </c>
+    </row>
+    <row r="5332">
+      <c r="A5332" t="str">
+        <v>Delete Minutes</v>
+      </c>
+      <c r="B5332" t="str">
+        <v>حذف المحضر</v>
+      </c>
+      <c r="C5332" t="str">
+        <v>Dzēst protokolu</v>
+      </c>
+    </row>
+    <row r="5333">
+      <c r="A5333" t="str">
+        <v>Document deleted</v>
+      </c>
+      <c r="B5333" t="str">
+        <v>تم حذف المستند</v>
+      </c>
+      <c r="C5333" t="str">
+        <v>Dokuments dzēsts</v>
+      </c>
+    </row>
+    <row r="5334">
+      <c r="A5334" t="str">
+        <v>Documents uploaded</v>
+      </c>
+      <c r="B5334" t="str">
+        <v>تم رفع المستندات</v>
+      </c>
+      <c r="C5334" t="str">
+        <v>Dokumenti augšupielādēti</v>
+      </c>
+    </row>
+    <row r="5335">
+      <c r="A5335" t="str">
+        <v>Edit Minutes</v>
+      </c>
+      <c r="B5335" t="str">
+        <v>تعديل المحضر</v>
+      </c>
+      <c r="C5335" t="str">
+        <v>Rediģēt protokolu</v>
+      </c>
+    </row>
+    <row r="5336">
+      <c r="A5336" t="str">
+        <v>Email address</v>
+      </c>
+      <c r="B5336" t="str">
+        <v>البريد الإلكتروني</v>
+      </c>
+      <c r="C5336" t="str">
+        <v>E-pasta adrese</v>
+      </c>
+    </row>
+    <row r="5337">
+      <c r="A5337" t="str">
+        <v>Failed to delete minutes</v>
+      </c>
+      <c r="B5337" t="str">
+        <v>فشل حذف المحضر</v>
+      </c>
+      <c r="C5337" t="str">
+        <v>Neizdevās dzēst protokolu</v>
+      </c>
+    </row>
+    <row r="5338">
+      <c r="A5338" t="str">
+        <v>Failed to load announcement</v>
+      </c>
+      <c r="B5338" t="str">
+        <v>فشل تحميل الإعلان</v>
+      </c>
+      <c r="C5338" t="str">
+        <v>Neizdevās ielādēt paziņojumu</v>
+      </c>
+    </row>
+    <row r="5339">
+      <c r="A5339" t="str">
+        <v>Failed to load audit planning memorandum</v>
+      </c>
+      <c r="B5339" t="str">
+        <v>فشل تحميل مذكرة تخطيط التدقيق</v>
+      </c>
+      <c r="C5339" t="str">
+        <v>Neizdevās ielādēt audita plānošanas memorandu</v>
+      </c>
+    </row>
+    <row r="5340">
+      <c r="A5340" t="str">
+        <v>Failed to load documents</v>
+      </c>
+      <c r="B5340" t="str">
+        <v>فشل تحميل المستندات</v>
+      </c>
+      <c r="C5340" t="str">
+        <v>Neizdevās ielādēt dokumentus</v>
+      </c>
+    </row>
+    <row r="5341">
+      <c r="A5341" t="str">
+        <v>Failed to load meeting minutes</v>
+      </c>
+      <c r="B5341" t="str">
+        <v>فشل تحميل محضر الاجتماع</v>
+      </c>
+      <c r="C5341" t="str">
+        <v>Neizdevās ielādēt sanāksmes protokolu</v>
+      </c>
+    </row>
+    <row r="5342">
+      <c r="A5342" t="str">
+        <v>Failed to save announcement</v>
+      </c>
+      <c r="B5342" t="str">
+        <v>فشل حفظ الإعلان</v>
+      </c>
+      <c r="C5342" t="str">
+        <v>Neizdevās saglabāt paziņojumu</v>
+      </c>
+    </row>
+    <row r="5343">
+      <c r="A5343" t="str">
+        <v>Failed to save audit planning memorandum</v>
+      </c>
+      <c r="B5343" t="str">
+        <v>فشل حفظ مذكرة تخطيط التدقيق</v>
+      </c>
+      <c r="C5343" t="str">
+        <v>Neizdevās saglabāt audita plānošanas memorandu</v>
+      </c>
+    </row>
+    <row r="5344">
+      <c r="A5344" t="str">
+        <v>Failed to save minutes</v>
+      </c>
+      <c r="B5344" t="str">
+        <v>فشل حفظ المحضر</v>
+      </c>
+      <c r="C5344" t="str">
+        <v>Neizdevās saglabāt protokolu</v>
+      </c>
+    </row>
+    <row r="5345">
+      <c r="A5345" t="str">
+        <v>Failed to send announcement</v>
+      </c>
+      <c r="B5345" t="str">
+        <v>فشل إرسال الإعلان</v>
+      </c>
+      <c r="C5345" t="str">
+        <v>Neizdevās nosūtīt paziņojumu</v>
+      </c>
+    </row>
+    <row r="5346">
+      <c r="A5346" t="str">
+        <v>Failed to update workflow</v>
+      </c>
+      <c r="B5346" t="str">
+        <v>فشل تحديث سير العمل</v>
+      </c>
+      <c r="C5346" t="str">
+        <v>Neizdevās atjaunināt darbplūsmu</v>
+      </c>
+    </row>
+    <row r="5347">
+      <c r="A5347" t="str">
+        <v>Failed to upload documents</v>
+      </c>
+      <c r="B5347" t="str">
+        <v>فشل رفع المستندات</v>
+      </c>
+      <c r="C5347" t="str">
+        <v>Neizdevās augšupielādēt dokumentus</v>
+      </c>
+    </row>
+    <row r="5348">
+      <c r="A5348" t="str">
+        <v>Finalized</v>
+      </c>
+      <c r="B5348" t="str">
+        <v>نهائي</v>
+      </c>
+      <c r="C5348" t="str">
+        <v>Pabeigts</v>
+      </c>
+    </row>
+    <row r="5349">
+      <c r="A5349" t="str">
+        <v>Findings Discussion</v>
+      </c>
+      <c r="B5349" t="str">
+        <v>مناقشة الملاحظات</v>
+      </c>
+      <c r="C5349" t="str">
+        <v>Konstatējumu apspriešana</v>
+      </c>
+    </row>
+    <row r="5350">
+      <c r="A5350" t="str">
+        <v>Follow-up</v>
+      </c>
+      <c r="B5350" t="str">
+        <v>المتابعة</v>
+      </c>
+      <c r="C5350" t="str">
+        <v>Turpmākā uzraudzība</v>
+      </c>
+    </row>
+    <row r="5351">
+      <c r="A5351" t="str">
+        <v>List of attendees</v>
+      </c>
+      <c r="B5351" t="str">
+        <v>قائمة الحضور</v>
+      </c>
+      <c r="C5351" t="str">
+        <v>Dalībnieku saraksts</v>
+      </c>
+    </row>
+    <row r="5352">
+      <c r="A5352" t="str">
+        <v>Management contact</v>
+      </c>
+      <c r="B5352" t="str">
+        <v>جهة اتصال الإدارة</v>
+      </c>
+      <c r="C5352" t="str">
+        <v>Vadības kontaktpersona</v>
+      </c>
+    </row>
+    <row r="5353">
+      <c r="A5353" t="str">
+        <v>Mark complete &amp; continue</v>
+      </c>
+      <c r="B5353" t="str">
+        <v>وضع علامة كمكتمل والمتابعة</v>
+      </c>
+      <c r="C5353" t="str">
+        <v>Atzīmēt kā pabeigtu un turpināt</v>
+      </c>
+    </row>
+    <row r="5354">
+      <c r="A5354" t="str">
+        <v>Meeting</v>
+      </c>
+      <c r="B5354" t="str">
+        <v>اجتماع</v>
+      </c>
+      <c r="C5354" t="str">
+        <v>Sanāksme</v>
+      </c>
+    </row>
+    <row r="5355">
+      <c r="A5355" t="str">
+        <v>Meeting Date</v>
+      </c>
+      <c r="B5355" t="str">
+        <v>تاريخ الاجتماع</v>
+      </c>
+      <c r="C5355" t="str">
+        <v>Sanāksmes datums</v>
+      </c>
+    </row>
+    <row r="5356">
+      <c r="A5356" t="str">
+        <v>Meeting title</v>
+      </c>
+      <c r="B5356" t="str">
+        <v>عنوان الاجتماع</v>
+      </c>
+      <c r="C5356" t="str">
+        <v>Sanāksmes nosaukums</v>
+      </c>
+    </row>
+    <row r="5357">
+      <c r="A5357" t="str">
+        <v>Message</v>
+      </c>
+      <c r="B5357" t="str">
+        <v>الرسالة</v>
+      </c>
+      <c r="C5357" t="str">
+        <v>Ziņojums</v>
+      </c>
+    </row>
+    <row r="5358">
+      <c r="A5358" t="str">
+        <v>Methodology</v>
+      </c>
+      <c r="B5358" t="str">
+        <v>المنهجية</v>
+      </c>
+      <c r="C5358" t="str">
+        <v>Metodoloģija</v>
+      </c>
+    </row>
+    <row r="5359">
+      <c r="A5359" t="str">
+        <v>Minutes</v>
+      </c>
+      <c r="B5359" t="str">
+        <v>المحضر</v>
+      </c>
+      <c r="C5359" t="str">
+        <v>Protokols</v>
+      </c>
+    </row>
+    <row r="5360">
+      <c r="A5360" t="str">
+        <v>Minutes added</v>
+      </c>
+      <c r="B5360" t="str">
+        <v>تمت إضافة المحضر</v>
+      </c>
+      <c r="C5360" t="str">
+        <v>Protokols pievienots</v>
+      </c>
+    </row>
+    <row r="5361">
+      <c r="A5361" t="str">
+        <v>Minutes deleted</v>
+      </c>
+      <c r="B5361" t="str">
+        <v>تم حذف المحضر</v>
+      </c>
+      <c r="C5361" t="str">
+        <v>Protokols dzēsts</v>
+      </c>
+    </row>
+    <row r="5362">
+      <c r="A5362" t="str">
+        <v>Minutes updated</v>
+      </c>
+      <c r="B5362" t="str">
+        <v>تم تحديث المحضر</v>
+      </c>
+      <c r="C5362" t="str">
+        <v>Protokols atjaunināts</v>
+      </c>
+    </row>
+    <row r="5363">
+      <c r="A5363" t="str">
+        <v>No documents uploaded yet</v>
+      </c>
+      <c r="B5363" t="str">
+        <v>لم يتم رفع أي مستندات بعد</v>
+      </c>
+      <c r="C5363" t="str">
+        <v>Vēl nav augšupielādēts neviens dokuments</v>
+      </c>
+    </row>
+    <row r="5364">
+      <c r="A5364" t="str">
+        <v>No memorandum yet</v>
+      </c>
+      <c r="B5364" t="str">
+        <v>لا توجد مذكرة بعد</v>
+      </c>
+      <c r="C5364" t="str">
+        <v>Vēl nav memoranda</v>
+      </c>
+    </row>
+    <row r="5365">
+      <c r="A5365" t="str">
+        <v>No minutes recorded yet</v>
+      </c>
+      <c r="B5365" t="str">
+        <v>لم يتم تسجيل أي محضر بعد</v>
+      </c>
+      <c r="C5365" t="str">
+        <v>Vēl nav reģistrēts neviens protokols</v>
+      </c>
+    </row>
+    <row r="5366">
+      <c r="A5366" t="str">
+        <v>on</v>
+      </c>
+      <c r="B5366" t="str">
+        <v>بتاريخ</v>
+      </c>
+      <c r="C5366" t="str">
+        <v>datumā</v>
+      </c>
+    </row>
+    <row r="5367">
+      <c r="A5367" t="str">
+        <v>Opening Meeting</v>
+      </c>
+      <c r="B5367" t="str">
+        <v>اجتماع الافتتاح</v>
+      </c>
+      <c r="C5367" t="str">
+        <v>Atklāšanas sanāksme</v>
+      </c>
+    </row>
+    <row r="5368">
+      <c r="A5368" t="str">
+        <v>Recipient Email</v>
+      </c>
+      <c r="B5368" t="str">
+        <v>بريد المستلم الإلكتروني</v>
+      </c>
+      <c r="C5368" t="str">
+        <v>Saņēmēja e-pasts</v>
+      </c>
+    </row>
+    <row r="5369">
+      <c r="A5369" t="str">
+        <v>Recipient Name</v>
+      </c>
+      <c r="B5369" t="str">
+        <v>اسم المستلم</v>
+      </c>
+      <c r="C5369" t="str">
+        <v>Saņēmēja vārds</v>
+      </c>
+    </row>
+    <row r="5370">
+      <c r="A5370" t="str">
+        <v>Recorded by</v>
+      </c>
+      <c r="B5370" t="str">
+        <v>سُجِّل بواسطة</v>
+      </c>
+      <c r="C5370" t="str">
+        <v>Reģistrēja</v>
+      </c>
+    </row>
+    <row r="5371">
+      <c r="A5371" t="str">
+        <v>Save Draft</v>
+      </c>
+      <c r="B5371" t="str">
+        <v>حفظ المسودة</v>
+      </c>
+      <c r="C5371" t="str">
+        <v>Saglabāt melnrakstu</v>
+      </c>
+    </row>
+    <row r="5372">
+      <c r="A5372" t="str">
+        <v>Send Announcement</v>
+      </c>
+      <c r="B5372" t="str">
+        <v>إرسال الإعلان</v>
+      </c>
+      <c r="C5372" t="str">
+        <v>Nosūtīt paziņojumu</v>
+      </c>
+    </row>
+    <row r="5373">
+      <c r="A5373" t="str">
+        <v>Send this announcement to the auditee?</v>
+      </c>
+      <c r="B5373" t="str">
+        <v>إرسال هذا الإعلان إلى الجهة الخاضعة للتدقيق؟</v>
+      </c>
+      <c r="C5373" t="str">
+        <v>Nosūtīt šo paziņojumu auditējamai pusei?</v>
+      </c>
+    </row>
+    <row r="5374">
+      <c r="A5374" t="str">
+        <v>Sent</v>
+      </c>
+      <c r="B5374" t="str">
+        <v>تم الإرسال</v>
+      </c>
+      <c r="C5374" t="str">
+        <v>Nosūtīts</v>
+      </c>
+    </row>
+    <row r="5375">
+      <c r="A5375" t="str">
+        <v>Sent by</v>
+      </c>
+      <c r="B5375" t="str">
+        <v>أُرسل بواسطة</v>
+      </c>
+      <c r="C5375" t="str">
+        <v>Nosūtīja</v>
+      </c>
+    </row>
+    <row r="5376">
+      <c r="A5376" t="str">
+        <v>Set as current step</v>
+      </c>
+      <c r="B5376" t="str">
+        <v>تعيين كخطوة حالية</v>
+      </c>
+      <c r="C5376" t="str">
+        <v>Iestatīt kā pašreizējo soli</v>
+      </c>
+    </row>
+    <row r="5377">
+      <c r="A5377" t="str">
+        <v>Step marked complete</v>
+      </c>
+      <c r="B5377" t="str">
+        <v>تم وضع علامة على الخطوة كمكتملة</v>
+      </c>
+      <c r="C5377" t="str">
+        <v>Solis atzīmēts kā pabeigts</v>
+      </c>
+    </row>
+    <row r="5378">
+      <c r="A5378" t="str">
+        <v>steps complete</v>
+      </c>
+      <c r="B5378" t="str">
+        <v>خطوات مكتملة</v>
+      </c>
+      <c r="C5378" t="str">
+        <v>soļi pabeigti</v>
+      </c>
+    </row>
+    <row r="5379">
+      <c r="A5379" t="str">
+        <v>Subject</v>
+      </c>
+      <c r="B5379" t="str">
+        <v>الموضوع</v>
+      </c>
+      <c r="C5379" t="str">
+        <v>Temats</v>
+      </c>
+    </row>
+    <row r="5380">
+      <c r="A5380" t="str">
+        <v>This step will be available in a future update.</v>
+      </c>
+      <c r="B5380" t="str">
+        <v>ستتوفر هذه الخطوة في تحديث مستقبلي.</v>
+      </c>
+      <c r="C5380" t="str">
+        <v>Šis solis būs pieejams nākamajā atjauninājumā.</v>
+      </c>
+    </row>
+    <row r="5381">
+      <c r="A5381" t="str">
+        <v>Workflow</v>
+      </c>
+      <c r="B5381" t="str">
+        <v>سير العمل</v>
+      </c>
+      <c r="C5381" t="str">
+        <v>Darbplūsma</v>
+      </c>
+    </row>
+    <row r="5382">
+      <c r="A5382" t="str">
+        <v>Send the formal audit announcement to management with the preliminary information request (PBC) list.</v>
+      </c>
+      <c r="B5382" t="str">
+        <v>إرسال إعلان التدقيق الرسمي إلى الإدارة مع قائمة طلب المعلومات الأولية (PBC).</v>
+      </c>
+      <c r="C5382" t="str">
+        <v>Nosūtīt vadībai oficiālu audita paziņojumu kopā ar sākotnējo informācijas pieprasījuma (PBC) sarakstu.</v>
+      </c>
+    </row>
+    <row r="5383">
+      <c r="A5383" t="str">
+        <v>Define audit scope, objectives, methodology and timeline; attach detailed audit program documents.</v>
+      </c>
+      <c r="B5383" t="str">
+        <v>تحديد نطاق التدقيق وأهدافه ومنهجيته وجدوله الزمني؛ وإرفاق مستندات برنامج التدقيق التفصيلية.</v>
+      </c>
+      <c r="C5383" t="str">
+        <v>Definēt audita tvērumu, mērķus, metodoloģiju un laika grafiku; pievienot detalizētus audita programmas dokumentus.</v>
+      </c>
+    </row>
+    <row r="5384">
+      <c r="A5384" t="str">
+        <v>Walk through objectives, scope, timeline and key contacts; capture the Minutes of Meeting.</v>
+      </c>
+      <c r="B5384" t="str">
+        <v>استعراض الأهداف والنطاق والجدول الزمني وجهات الاتصال الرئيسية؛ وتسجيل محضر الاجتماع.</v>
+      </c>
+      <c r="C5384" t="str">
+        <v>Pārrunāt mērķus, tvērumu, laika grafiku un galvenās kontaktpersonas; reģistrēt sanāksmes protokolu.</v>
+      </c>
+    </row>
+    <row r="5385">
+      <c r="A5385" t="str">
+        <v>Review the audit program overview and prepare workpapers before fieldwork begins.</v>
+      </c>
+      <c r="B5385" t="str">
+        <v>مراجعة نظرة عامة على برنامج التدقيق وإعداد أوراق العمل قبل بدء العمل الميداني.</v>
+      </c>
+      <c r="C5385" t="str">
+        <v>Pārskatīt audita programmas kopsavilkumu un sagatavot darba dokumentus pirms lauka darba sākuma.</v>
+      </c>
+    </row>
+    <row r="5386">
+      <c r="A5386" t="str">
+        <v>Run walkthroughs and control testing, manage workpapers, and collect evidence.</v>
+      </c>
+      <c r="B5386" t="str">
+        <v>إجراء الاستعراضات واختبار الضوابط وإدارة أوراق العمل وجمع الأدلة.</v>
+      </c>
+      <c r="C5386" t="str">
+        <v>Veikt caurskates un kontroļu testēšanu, pārvaldīt darba dokumentus un vākt pierādījumus.</v>
+      </c>
+    </row>
+    <row r="5387">
+      <c r="A5387" t="str">
+        <v>Record audit findings with criteria, condition, cause, effect and recommendations.</v>
+      </c>
+      <c r="B5387" t="str">
+        <v>تسجيل ملاحظات التدقيق مع المعايير والحالة والسبب والأثر والتوصيات.</v>
+      </c>
+      <c r="C5387" t="str">
+        <v>Reģistrēt audita konstatējumus ar kritērijiem, stāvokli, cēloni, sekām un ieteikumiem.</v>
+      </c>
+    </row>
+    <row r="5388">
+      <c r="A5388" t="str">
+        <v>Validate facts, agree on action plans and finalize management responses; capture the Minutes of Meeting.</v>
+      </c>
+      <c r="B5388" t="str">
+        <v>التحقق من الحقائق والاتفاق على خطط العمل ووضع اللمسات النهائية على ردود الإدارة؛ وتسجيل محضر الاجتماع.</v>
+      </c>
+      <c r="C5388" t="str">
+        <v>Pārbaudīt faktus, vienoties par rīcības plāniem un pabeigt vadības atbildes; reģistrēt sanāksmes protokolu.</v>
+      </c>
+    </row>
+    <row r="5389">
+      <c r="A5389" t="str">
+        <v>Generate the draft and final audit reports and capture auditee responses.</v>
+      </c>
+      <c r="B5389" t="str">
+        <v>إنشاء مسودة تقارير التدقيق والتقارير النهائية وتسجيل ردود الجهة الخاضعة للتدقيق.</v>
+      </c>
+      <c r="C5389" t="str">
+        <v>Izveidot audita ziņojumu melnrakstus un galīgos ziņojumus un fiksēt auditējamās puses atbildes.</v>
+      </c>
+    </row>
+    <row r="5390">
+      <c r="A5390" t="str">
+        <v>Discuss final observations and action plans; capture the Minutes of Meeting.</v>
+      </c>
+      <c r="B5390" t="str">
+        <v>مناقشة الملاحظات النهائية وخطط العمل؛ وتسجيل محضر الاجتماع.</v>
+      </c>
+      <c r="C5390" t="str">
+        <v>Apspriest galīgos novērojumus un rīcības plānus; reģistrēt sanāksmes protokolu.</v>
+      </c>
+    </row>
+    <row r="5391">
+      <c r="A5391" t="str">
+        <v>Track implementation of recommendations, due dates and remediation progress.</v>
+      </c>
+      <c r="B5391" t="str">
+        <v>تتبع تنفيذ التوصيات وتواريخ الاستحقاق وتقدم المعالجة.</v>
+      </c>
+      <c r="C5391" t="str">
+        <v>Sekot līdzi ieteikumu ieviešanai, termiņiem un novēršanas progresam.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5306"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5391"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Arabic and Latvian translations for findings communication UI
Localize the Phase 4 findings communication component (mode selector,
share actions, helper text) — 19 new phrases added to translations.xlsx
with Arabic and Latvian, locale files regenerated.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5391"/>
+  <dimension ref="A1:C5410"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -59700,9 +59700,218 @@
         <v>Sekot līdzi ieteikumu ieviešanai, termiņiem un novēršanas progresam.</v>
       </c>
     </row>
+    <row r="5392">
+      <c r="A5392" t="str">
+        <v>Add findings in Fieldwork to communicate them here.</v>
+      </c>
+      <c r="B5392" t="str">
+        <v>أضف الملاحظات في العمل الميداني لإبلاغها هنا.</v>
+      </c>
+      <c r="C5392" t="str">
+        <v>Pievienojiet konstatējumus lauka darbā, lai tos šeit paziņotu.</v>
+      </c>
+    </row>
+    <row r="5393">
+      <c r="A5393" t="str">
+        <v>Aggregated</v>
+      </c>
+      <c r="B5393" t="str">
+        <v>مجمّع</v>
+      </c>
+      <c r="C5393" t="str">
+        <v>Apkopots</v>
+      </c>
+    </row>
+    <row r="5394">
+      <c r="A5394" t="str">
+        <v>Communication Mode</v>
+      </c>
+      <c r="B5394" t="str">
+        <v>وضع الإبلاغ</v>
+      </c>
+      <c r="C5394" t="str">
+        <v>Saziņas režīms</v>
+      </c>
+    </row>
+    <row r="5395">
+      <c r="A5395" t="str">
+        <v>Communication mode updated</v>
+      </c>
+      <c r="B5395" t="str">
+        <v>تم تحديث وضع الإبلاغ</v>
+      </c>
+      <c r="C5395" t="str">
+        <v>Saziņas režīms atjaunināts</v>
+      </c>
+    </row>
+    <row r="5396">
+      <c r="A5396" t="str">
+        <v>Continuous</v>
+      </c>
+      <c r="B5396" t="str">
+        <v>مستمر</v>
+      </c>
+      <c r="C5396" t="str">
+        <v>Nepārtraukts</v>
+      </c>
+    </row>
+    <row r="5397">
+      <c r="A5397" t="str">
+        <v>Failed to load findings</v>
+      </c>
+      <c r="B5397" t="str">
+        <v>فشل تحميل الملاحظات</v>
+      </c>
+      <c r="C5397" t="str">
+        <v>Neizdevās ielādēt konstatējumus</v>
+      </c>
+    </row>
+    <row r="5398">
+      <c r="A5398" t="str">
+        <v>Failed to share finding</v>
+      </c>
+      <c r="B5398" t="str">
+        <v>فشل مشاركة الملاحظة</v>
+      </c>
+      <c r="C5398" t="str">
+        <v>Neizdevās kopīgot konstatējumu</v>
+      </c>
+    </row>
+    <row r="5399">
+      <c r="A5399" t="str">
+        <v>Failed to unshare finding</v>
+      </c>
+      <c r="B5399" t="str">
+        <v>فشل إلغاء مشاركة الملاحظة</v>
+      </c>
+      <c r="C5399" t="str">
+        <v>Neizdevās atcelt konstatējuma kopīgošanu</v>
+      </c>
+    </row>
+    <row r="5400">
+      <c r="A5400" t="str">
+        <v>Failed to update communication mode</v>
+      </c>
+      <c r="B5400" t="str">
+        <v>فشل تحديث وضع الإبلاغ</v>
+      </c>
+      <c r="C5400" t="str">
+        <v>Neizdevās atjaunināt saziņas režīmu</v>
+      </c>
+    </row>
+    <row r="5401">
+      <c r="A5401" t="str">
+        <v>Finding shared with auditee</v>
+      </c>
+      <c r="B5401" t="str">
+        <v>تمت مشاركة الملاحظة مع الجهة الخاضعة للتدقيق</v>
+      </c>
+      <c r="C5401" t="str">
+        <v>Konstatējums kopīgots ar auditējamo pusi</v>
+      </c>
+    </row>
+    <row r="5402">
+      <c r="A5402" t="str">
+        <v>Finding unshared</v>
+      </c>
+      <c r="B5402" t="str">
+        <v>تم إلغاء مشاركة الملاحظة</v>
+      </c>
+      <c r="C5402" t="str">
+        <v>Konstatējuma kopīgošana atcelta</v>
+      </c>
+    </row>
+    <row r="5403">
+      <c r="A5403" t="str">
+        <v>Findings are consolidated into the draft detailed report.</v>
+      </c>
+      <c r="B5403" t="str">
+        <v>يتم تجميع الملاحظات في مسودة التقرير التفصيلي.</v>
+      </c>
+      <c r="C5403" t="str">
+        <v>Konstatējumi tiek apkopoti detalizētā ziņojuma melnrakstā.</v>
+      </c>
+    </row>
+    <row r="5404">
+      <c r="A5404" t="str">
+        <v>Findings are shared with the auditee individually as they are identified.</v>
+      </c>
+      <c r="B5404" t="str">
+        <v>تتم مشاركة الملاحظات مع الجهة الخاضعة للتدقيق بشكل فردي عند تحديدها.</v>
+      </c>
+      <c r="C5404" t="str">
+        <v>Konstatējumi tiek individuāli kopīgoti ar auditējamo pusi, tiklīdz tie tiek identificēti.</v>
+      </c>
+    </row>
+    <row r="5405">
+      <c r="A5405" t="str">
+        <v>Findings Communication</v>
+      </c>
+      <c r="B5405" t="str">
+        <v>إبلاغ الملاحظات</v>
+      </c>
+      <c r="C5405" t="str">
+        <v>Konstatējumu paziņošana</v>
+      </c>
+    </row>
+    <row r="5406">
+      <c r="A5406" t="str">
+        <v>No findings recorded yet.</v>
+      </c>
+      <c r="B5406" t="str">
+        <v>لم يتم تسجيل أي ملاحظات بعد.</v>
+      </c>
+      <c r="C5406" t="str">
+        <v>Vēl nav reģistrēts neviens konstatējums.</v>
+      </c>
+    </row>
+    <row r="5407">
+      <c r="A5407" t="str">
+        <v>Open in Fieldwork</v>
+      </c>
+      <c r="B5407" t="str">
+        <v>فتح في العمل الميداني</v>
+      </c>
+      <c r="C5407" t="str">
+        <v>Atvērt lauka darbā</v>
+      </c>
+    </row>
+    <row r="5408">
+      <c r="A5408" t="str">
+        <v>Share with auditee</v>
+      </c>
+      <c r="B5408" t="str">
+        <v>مشاركة مع الجهة الخاضعة للتدقيق</v>
+      </c>
+      <c r="C5408" t="str">
+        <v>Kopīgot ar auditējamo pusi</v>
+      </c>
+    </row>
+    <row r="5409">
+      <c r="A5409" t="str">
+        <v>Shared</v>
+      </c>
+      <c r="B5409" t="str">
+        <v>تمت المشاركة</v>
+      </c>
+      <c r="C5409" t="str">
+        <v>Kopīgots</v>
+      </c>
+    </row>
+    <row r="5410">
+      <c r="A5410" t="str">
+        <v>Unshare</v>
+      </c>
+      <c r="B5410" t="str">
+        <v>إلغاء المشاركة</v>
+      </c>
+      <c r="C5410" t="str">
+        <v>Atcelt kopīgošanu</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5391"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5410"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Arabic and Latvian translations for audit program and recommendation doc
Localize the new download controls (audit program overview/download and
implementation recommendation document) — 5 new phrases added to
translations.xlsx with Arabic and Latvian, locale files regenerated.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5410"/>
+  <dimension ref="A1:C5415"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -59909,9 +59909,64 @@
         <v>Atcelt kopīgošanu</v>
       </c>
     </row>
+    <row r="5411">
+      <c r="A5411" t="str">
+        <v>Audit Program Overview</v>
+      </c>
+      <c r="B5411" t="str">
+        <v>نظرة عامة على برنامج التدقيق</v>
+      </c>
+      <c r="C5411" t="str">
+        <v>Audita programmas pārskats</v>
+      </c>
+    </row>
+    <row r="5412">
+      <c r="A5412" t="str">
+        <v>Download Audit Program</v>
+      </c>
+      <c r="B5412" t="str">
+        <v>تنزيل برنامج التدقيق</v>
+      </c>
+      <c r="C5412" t="str">
+        <v>Lejupielādēt audita programmu</v>
+      </c>
+    </row>
+    <row r="5413">
+      <c r="A5413" t="str">
+        <v>Implementation Recommendation Document</v>
+      </c>
+      <c r="B5413" t="str">
+        <v>وثيقة توصيات التنفيذ</v>
+      </c>
+      <c r="C5413" t="str">
+        <v>Ieviešanas ieteikumu dokuments</v>
+      </c>
+    </row>
+    <row r="5414">
+      <c r="A5414" t="str">
+        <v>procedure</v>
+      </c>
+      <c r="B5414" t="str">
+        <v>إجراء</v>
+      </c>
+      <c r="C5414" t="str">
+        <v>procedūra</v>
+      </c>
+    </row>
+    <row r="5415">
+      <c r="A5415" t="str">
+        <v>procedures</v>
+      </c>
+      <c r="B5415" t="str">
+        <v>إجراءات</v>
+      </c>
+      <c r="C5415" t="str">
+        <v>procedūras</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5410"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5415"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add risk priority auto-sort and strategic plan Pending Approval state
- Risk register now auto-sorts by residual risk (highest first) instead of
  creation date
- Strategic plan approval is now a Draft -> Pending Approval -> Approved
  workflow: new submit/withdraw endpoint and a status-driven approval UI
  (submit for approval, then signed-copy upload to approve, or withdraw)
- Add Arabic and Latvian translations for the new submission strings
- Update docs/INTERNAL_AUDIT_MODULE.md (gaps closed) and add a CLAUDE.md
  rule to keep that doc updated whenever Internal Audit changes

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5415"/>
+  <dimension ref="A1:C5422"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -59964,9 +59964,86 @@
         <v>procedūras</v>
       </c>
     </row>
+    <row r="5416">
+      <c r="A5416" t="str">
+        <v>Failed to submit strategic plan</v>
+      </c>
+      <c r="B5416" t="str">
+        <v>فشل إرسال الخطة الاستراتيجية</v>
+      </c>
+      <c r="C5416" t="str">
+        <v>Neizdevās iesniegt stratēģisko plānu</v>
+      </c>
+    </row>
+    <row r="5417">
+      <c r="A5417" t="str">
+        <v>Failed to withdraw submission</v>
+      </c>
+      <c r="B5417" t="str">
+        <v>فشل سحب الطلب</v>
+      </c>
+      <c r="C5417" t="str">
+        <v>Neizdevās atsaukt iesniegumu</v>
+      </c>
+    </row>
+    <row r="5418">
+      <c r="A5418" t="str">
+        <v>Strategic plan submitted for approval</v>
+      </c>
+      <c r="B5418" t="str">
+        <v>تم إرسال الخطة الاستراتيجية للموافقة</v>
+      </c>
+      <c r="C5418" t="str">
+        <v>Stratēģiskais plāns iesniegts apstiprināšanai</v>
+      </c>
+    </row>
+    <row r="5419">
+      <c r="A5419" t="str">
+        <v>Submission withdrawn</v>
+      </c>
+      <c r="B5419" t="str">
+        <v>تم سحب الطلب</v>
+      </c>
+      <c r="C5419" t="str">
+        <v>Iesniegums atsaukts</v>
+      </c>
+    </row>
+    <row r="5420">
+      <c r="A5420" t="str">
+        <v>Submit this strategic plan for approval by the approving authority.</v>
+      </c>
+      <c r="B5420" t="str">
+        <v>إرسال هذه الخطة الاستراتيجية للموافقة من قبل الجهة المعتمِدة.</v>
+      </c>
+      <c r="C5420" t="str">
+        <v>Iesniegt šo stratēģisko plānu apstiprināšanai apstiprinātājinstitūcijā.</v>
+      </c>
+    </row>
+    <row r="5421">
+      <c r="A5421" t="str">
+        <v>This strategic plan is awaiting approval.</v>
+      </c>
+      <c r="B5421" t="str">
+        <v>هذه الخطة الاستراتيجية في انتظار الموافقة.</v>
+      </c>
+      <c r="C5421" t="str">
+        <v>Šis stratēģiskais plāns gaida apstiprinājumu.</v>
+      </c>
+    </row>
+    <row r="5422">
+      <c r="A5422" t="str">
+        <v>Withdraw to Draft</v>
+      </c>
+      <c r="B5422" t="str">
+        <v>إعادة إلى المسودة</v>
+      </c>
+      <c r="C5422" t="str">
+        <v>Atsaukt uz melnrakstu</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5415"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5422"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Show Risk Heat Map only after risk assessment is completed
In the Internal Audit Risk Register per-risk View modal, the Risk Heat Map
now renders only when the risk's assessmentStatus is "Assessed". For an
unassessed risk it shows a placeholder card prompting the user to complete
the assessment first. The assessed heat map is unchanged and still plots the
inherent point.

- Gate the heat map block on viewingRisk.assessmentStatus === "Assessed"
- Add placeholder: "Complete the risk assessment to view the heat map."
- Add assessmentStatus to the InternalAuditRiskDetail interface (already
  returned by the risks/[id] API via include)
- Add i18n phrases "Risk Heat Map" and the placeholder (init-translations.ts
  + translations.xlsx), regenerate locales

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5374"/>
+  <dimension ref="A1:C5376"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -59513,9 +59513,31 @@
         <v>Pievienojiet vairāk personu, kas saņems šo paziņojumu (CC).</v>
       </c>
     </row>
+    <row r="5375">
+      <c r="A5375" t="str">
+        <v>Risk Heat Map</v>
+      </c>
+      <c r="B5375" t="str">
+        <v>خريطة حرارة المخاطر</v>
+      </c>
+      <c r="C5375" t="str">
+        <v>Risku siltuma karte</v>
+      </c>
+    </row>
+    <row r="5376">
+      <c r="A5376" t="str">
+        <v>Complete the risk assessment to view the heat map.</v>
+      </c>
+      <c r="B5376" t="str">
+        <v>أكمل تقييم المخاطر لعرض خريطة الحرارة.</v>
+      </c>
+      <c r="C5376" t="str">
+        <v>Pabeidziet riska novērtējumu, lai skatītu siltuma karti.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5374"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5376"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add "Finish & Generate Report" action to engagement closing meeting
On the Closing Meeting (final workflow step), replace the generic step
buttons with a single "Finish & Generate Report" action that appears only
once every previous step is completed. Clicking it marks the engagement
Completed, generates the audit report, and opens it in the Report section.

- engagement/[id]: gate a single Finish button on all-prior-steps-complete;
  on click PATCH status=Completed + mark all stages complete, then POST
  report generate (treats an existing report as success) and navigate to
  the report
- show a hint until prerequisites are met; show "View Report" when the
  audit is already Completed
- i18n phrases added (en/ar/lv); sync teammate finding/recipient phrases
  into the xlsx and regenerate locales

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/i18n/translations.xlsx
+++ b/i18n/translations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5411"/>
+  <dimension ref="A1:C5423"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -59920,9 +59920,141 @@
         <v>Konstatējumi, kas izriet no neatbilstības tiesību aktiem, noteikumiem un likumiem.</v>
       </c>
     </row>
+    <row r="5412">
+      <c r="A5412" t="str">
+        <v>Finish &amp; Generate Report</v>
+      </c>
+      <c r="B5412" t="str">
+        <v>إنهاء وإنشاء التقرير</v>
+      </c>
+      <c r="C5412" t="str">
+        <v>Pabeigt un ģenerēt ziņojumu</v>
+      </c>
+    </row>
+    <row r="5413">
+      <c r="A5413" t="str">
+        <v>Complete all previous steps to finish the audit and generate the report.</v>
+      </c>
+      <c r="B5413" t="str">
+        <v>أكمل جميع الخطوات السابقة لإنهاء التدقيق وإنشاء التقرير.</v>
+      </c>
+      <c r="C5413" t="str">
+        <v>Pabeidziet visus iepriekšējos soļus, lai pabeigtu auditu un ģenerētu ziņojumu.</v>
+      </c>
+    </row>
+    <row r="5414">
+      <c r="A5414" t="str">
+        <v>Audit completed and report generated</v>
+      </c>
+      <c r="B5414" t="str">
+        <v>تم إكمال التدقيق وإنشاء التقرير</v>
+      </c>
+      <c r="C5414" t="str">
+        <v>Audits pabeigts un ziņojums ģenerēts</v>
+      </c>
+    </row>
+    <row r="5415">
+      <c r="A5415" t="str">
+        <v>Failed to finish audit and generate report</v>
+      </c>
+      <c r="B5415" t="str">
+        <v>فشل إنهاء التدقيق وإنشاء التقرير</v>
+      </c>
+      <c r="C5415" t="str">
+        <v>Neizdevās pabeigt auditu un ģenerēt ziņojumu</v>
+      </c>
+    </row>
+    <row r="5416">
+      <c r="A5416" t="str">
+        <v>View Report</v>
+      </c>
+      <c r="B5416" t="str">
+        <v>عرض التقرير</v>
+      </c>
+      <c r="C5416" t="str">
+        <v>Skatīt ziņojumu</v>
+      </c>
+    </row>
+    <row r="5417">
+      <c r="A5417" t="str">
+        <v>Add Findings</v>
+      </c>
+      <c r="B5417" t="str">
+        <v>إضافة ملاحظات</v>
+      </c>
+      <c r="C5417" t="str">
+        <v>Pievienot konstatējumus</v>
+      </c>
+    </row>
+    <row r="5418">
+      <c r="A5418" t="str">
+        <v>Save Findings</v>
+      </c>
+      <c r="B5418" t="str">
+        <v>حفظ الملاحظات</v>
+      </c>
+      <c r="C5418" t="str">
+        <v>Saglabāt konstatējumus</v>
+      </c>
+    </row>
+    <row r="5419">
+      <c r="A5419" t="str">
+        <v>Use Add Row to record multiple findings, then Save Findings.</v>
+      </c>
+      <c r="B5419" t="str">
+        <v>استخدم "إضافة صف" لتسجيل عدة ملاحظات، ثم احفظ الملاحظات.</v>
+      </c>
+      <c r="C5419" t="str">
+        <v>Izmantojiet "Pievienot rindu", lai reģistrētu vairākus konstatējumus, pēc tam saglabājiet.</v>
+      </c>
+    </row>
+    <row r="5420">
+      <c r="A5420" t="str">
+        <v>Recipients</v>
+      </c>
+      <c r="B5420" t="str">
+        <v>المستلمون</v>
+      </c>
+      <c r="C5420" t="str">
+        <v>Saņēmēji</v>
+      </c>
+    </row>
+    <row r="5421">
+      <c r="A5421" t="str">
+        <v>Select recipient</v>
+      </c>
+      <c r="B5421" t="str">
+        <v>اختر مستلمًا</v>
+      </c>
+      <c r="C5421" t="str">
+        <v>Atlasiet saņēmēju</v>
+      </c>
+    </row>
+    <row r="5422">
+      <c r="A5422" t="str">
+        <v>Select one or more recipients; their email is added automatically.</v>
+      </c>
+      <c r="B5422" t="str">
+        <v>اختر مستلمًا واحدًا أو أكثر؛ تتم إضافة بريدهم الإلكتروني تلقائيًا.</v>
+      </c>
+      <c r="C5422" t="str">
+        <v>Atlasiet vienu vai vairākus saņēmējus; viņu e-pasts tiek pievienots automātiski.</v>
+      </c>
+    </row>
+    <row r="5423">
+      <c r="A5423" t="str">
+        <v>All users already added</v>
+      </c>
+      <c r="B5423" t="str">
+        <v>تمت إضافة جميع المستخدمين بالفعل</v>
+      </c>
+      <c r="C5423" t="str">
+        <v>Visi lietotāji jau pievienoti</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5411"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5423"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>